<commit_message>
hnaya zadt ela if and condition
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2D74241-DC23-44F6-8B5D-061B700B1D3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D794754C-129F-4AFB-AD6A-570610D33694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
     <sheet name="trading_raw_data2" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="37">
   <si>
     <t>TradeID</t>
   </si>
@@ -145,6 +145,9 @@
   </si>
   <si>
     <t>excptation value</t>
+  </si>
+  <si>
+    <t>Risk Status</t>
   </si>
 </sst>
 </file>
@@ -721,7 +724,10 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
     </dxf>
@@ -739,12 +745,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E6EB144A-984A-4FCF-892A-EB44514BDE51}" name="Table1" displayName="Table1" ref="A1:I101" totalsRowShown="0">
-  <autoFilter ref="A1:I101" xr:uid="{E6EB144A-984A-4FCF-892A-EB44514BDE51}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I101">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E6EB144A-984A-4FCF-892A-EB44514BDE51}" name="Table1" displayName="Table1" ref="A1:J101" totalsRowShown="0">
+  <autoFilter ref="A1:J101" xr:uid="{E6EB144A-984A-4FCF-892A-EB44514BDE51}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J101">
     <sortCondition ref="C2:C101"/>
   </sortState>
-  <tableColumns count="9">
+  <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{897A45A9-8A0C-47F0-BAC4-2FB84871975D}" name="TradeID"/>
     <tableColumn id="2" xr3:uid="{2DC41DFE-2253-40BF-A088-0B1563C0DC81}" name="AccountID"/>
     <tableColumn id="3" xr3:uid="{A49B41A0-B5A8-4D84-9946-EDB3CB5DDF8D}" name="Pair"/>
@@ -752,8 +758,11 @@
     <tableColumn id="5" xr3:uid="{539426CC-F875-4D64-977A-05C6F1BCDBCD}" name="Direction"/>
     <tableColumn id="6" xr3:uid="{BFF7C4D2-29D9-4645-98DB-6FBF609AB80F}" name="Profit"/>
     <tableColumn id="7" xr3:uid="{CD8DBAA1-576E-4991-87E5-049F5C232A1F}" name="R"/>
+    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="0">
+      <calculatedColumnFormula>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</calculatedColumnFormula>
+    </tableColumn>
     <tableColumn id="8" xr3:uid="{CC96218F-2F0A-46BB-98E4-8AE8218DB3D7}" name="Result"/>
-    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="0"/>
+    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1076,17 +1085,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{906658B5-1F80-4C49-9035-7A91F11B2092}">
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:J101"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.33203125" customWidth="1"/>
     <col min="2" max="2" width="11.44140625" customWidth="1"/>
     <col min="4" max="4" width="9.33203125" customWidth="1"/>
     <col min="5" max="5" width="10.5546875" customWidth="1"/>
-    <col min="9" max="9" width="19.5546875" customWidth="1"/>
+    <col min="8" max="8" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1109,13 +1119,16 @@
         <v>6</v>
       </c>
       <c r="H1" t="s">
+        <v>36</v>
+      </c>
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>6</v>
       </c>
@@ -1137,14 +1150,18 @@
       <c r="G2">
         <v>3</v>
       </c>
-      <c r="H2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I2" s="1">
+      <c r="H2" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" s="1">
         <v>46164</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>80</v>
       </c>
@@ -1166,14 +1183,18 @@
       <c r="G3">
         <v>3</v>
       </c>
-      <c r="H3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I3" s="1">
+      <c r="H3" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J3" s="1">
         <v>46171</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>16</v>
       </c>
@@ -1195,14 +1216,18 @@
       <c r="G4">
         <v>2</v>
       </c>
-      <c r="H4" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" s="1">
+      <c r="H4" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J4" s="1">
         <v>46168</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>78</v>
       </c>
@@ -1224,14 +1249,18 @@
       <c r="G5">
         <v>2</v>
       </c>
-      <c r="H5" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5" s="1">
+      <c r="H5" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I5" t="s">
+        <v>12</v>
+      </c>
+      <c r="J5" s="1">
         <v>46182</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>35</v>
       </c>
@@ -1253,14 +1282,18 @@
       <c r="G6">
         <v>1.5</v>
       </c>
-      <c r="H6" t="s">
-        <v>12</v>
-      </c>
-      <c r="I6" s="1">
+      <c r="H6" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J6" s="1">
         <v>46041</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>45</v>
       </c>
@@ -1282,14 +1315,18 @@
       <c r="G7">
         <v>1.5</v>
       </c>
-      <c r="H7" t="s">
-        <v>12</v>
-      </c>
-      <c r="I7" s="1">
+      <c r="H7" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I7" t="s">
+        <v>12</v>
+      </c>
+      <c r="J7" s="1">
         <v>46055</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>43</v>
       </c>
@@ -1311,14 +1348,18 @@
       <c r="G8">
         <v>2</v>
       </c>
-      <c r="H8" t="s">
-        <v>12</v>
-      </c>
-      <c r="I8" s="1">
+      <c r="H8" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I8" t="s">
+        <v>12</v>
+      </c>
+      <c r="J8" s="1">
         <v>46091</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>77</v>
       </c>
@@ -1340,14 +1381,18 @@
       <c r="G9">
         <v>2</v>
       </c>
-      <c r="H9" t="s">
-        <v>12</v>
-      </c>
-      <c r="I9" s="1">
+      <c r="H9" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I9" t="s">
+        <v>12</v>
+      </c>
+      <c r="J9" s="1">
         <v>46198</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>99</v>
       </c>
@@ -1369,14 +1414,18 @@
       <c r="G10">
         <v>2.5</v>
       </c>
-      <c r="H10" t="s">
-        <v>12</v>
-      </c>
-      <c r="I10" s="1">
+      <c r="H10" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I10" t="s">
+        <v>12</v>
+      </c>
+      <c r="J10" s="1">
         <v>46101</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>97</v>
       </c>
@@ -1398,14 +1447,18 @@
       <c r="G11">
         <v>1</v>
       </c>
-      <c r="H11" t="s">
-        <v>12</v>
-      </c>
-      <c r="I11" s="1">
+      <c r="H11" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I11" t="s">
+        <v>12</v>
+      </c>
+      <c r="J11" s="1">
         <v>46172</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>93</v>
       </c>
@@ -1427,14 +1480,18 @@
       <c r="G12">
         <v>1.5</v>
       </c>
-      <c r="H12" t="s">
-        <v>12</v>
-      </c>
-      <c r="I12" s="1">
+      <c r="H12" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I12" t="s">
+        <v>12</v>
+      </c>
+      <c r="J12" s="1">
         <v>46053</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>1</v>
       </c>
@@ -1456,14 +1513,18 @@
       <c r="G13">
         <v>1</v>
       </c>
-      <c r="H13" t="s">
-        <v>12</v>
-      </c>
-      <c r="I13" s="1">
+      <c r="H13" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I13" t="s">
+        <v>12</v>
+      </c>
+      <c r="J13" s="1">
         <v>46190</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>38</v>
       </c>
@@ -1485,14 +1546,18 @@
       <c r="G14">
         <v>-0.5</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H14" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I14" t="s">
         <v>17</v>
       </c>
-      <c r="I14" s="1">
+      <c r="J14" s="1">
         <v>46107</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>30</v>
       </c>
@@ -1514,14 +1579,18 @@
       <c r="G15">
         <v>-0.5</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H15" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I15" t="s">
         <v>17</v>
       </c>
-      <c r="I15" s="1">
+      <c r="J15" s="1">
         <v>46167</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>46</v>
       </c>
@@ -1543,14 +1612,18 @@
       <c r="G16">
         <v>-0.5</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H16" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I16" t="s">
         <v>17</v>
       </c>
-      <c r="I16" s="1">
+      <c r="J16" s="1">
         <v>46059</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>47</v>
       </c>
@@ -1572,14 +1645,18 @@
       <c r="G17">
         <v>-0.5</v>
       </c>
-      <c r="H17" t="s">
+      <c r="H17" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I17" t="s">
         <v>17</v>
       </c>
-      <c r="I17" s="1">
+      <c r="J17" s="1">
         <v>46197</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>52</v>
       </c>
@@ -1601,14 +1678,18 @@
       <c r="G18">
         <v>-1</v>
       </c>
-      <c r="H18" t="s">
+      <c r="H18" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I18" t="s">
         <v>17</v>
       </c>
-      <c r="I18" s="1">
+      <c r="J18" s="1">
         <v>46034</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>8</v>
       </c>
@@ -1630,14 +1711,18 @@
       <c r="G19">
         <v>-1</v>
       </c>
-      <c r="H19" t="s">
+      <c r="H19" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I19" t="s">
         <v>17</v>
       </c>
-      <c r="I19" s="1">
+      <c r="J19" s="1">
         <v>46086</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>70</v>
       </c>
@@ -1659,14 +1744,18 @@
       <c r="G20">
         <v>-1</v>
       </c>
-      <c r="H20" t="s">
+      <c r="H20" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I20" t="s">
         <v>17</v>
       </c>
-      <c r="I20" s="1">
+      <c r="J20" s="1">
         <v>46149</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>86</v>
       </c>
@@ -1688,14 +1777,18 @@
       <c r="G21">
         <v>-1</v>
       </c>
-      <c r="H21" t="s">
+      <c r="H21" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I21" t="s">
         <v>17</v>
       </c>
-      <c r="I21" s="1">
+      <c r="J21" s="1">
         <v>46169</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>61</v>
       </c>
@@ -1717,14 +1810,18 @@
       <c r="G22">
         <v>-0.5</v>
       </c>
-      <c r="H22" t="s">
+      <c r="H22" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I22" t="s">
         <v>17</v>
       </c>
-      <c r="I22" s="1">
+      <c r="J22" s="1">
         <v>46033</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>34</v>
       </c>
@@ -1746,14 +1843,18 @@
       <c r="G23">
         <v>-1.5</v>
       </c>
-      <c r="H23" t="s">
+      <c r="H23" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I23" t="s">
         <v>17</v>
       </c>
-      <c r="I23" s="1">
+      <c r="J23" s="1">
         <v>46107</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>13</v>
       </c>
@@ -1775,14 +1876,18 @@
       <c r="G24">
         <v>3</v>
       </c>
-      <c r="H24" t="s">
-        <v>12</v>
-      </c>
-      <c r="I24" s="1">
+      <c r="H24" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I24" t="s">
+        <v>12</v>
+      </c>
+      <c r="J24" s="1">
         <v>46094</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>98</v>
       </c>
@@ -1804,14 +1909,18 @@
       <c r="G25">
         <v>3</v>
       </c>
-      <c r="H25" t="s">
-        <v>12</v>
-      </c>
-      <c r="I25" s="1">
+      <c r="H25" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I25" t="s">
+        <v>12</v>
+      </c>
+      <c r="J25" s="1">
         <v>46088</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>68</v>
       </c>
@@ -1833,14 +1942,18 @@
       <c r="G26">
         <v>2.5</v>
       </c>
-      <c r="H26" t="s">
-        <v>12</v>
-      </c>
-      <c r="I26" s="1">
+      <c r="H26" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I26" t="s">
+        <v>12</v>
+      </c>
+      <c r="J26" s="1">
         <v>46207</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>85</v>
       </c>
@@ -1862,14 +1975,18 @@
       <c r="G27">
         <v>3</v>
       </c>
-      <c r="H27" t="s">
-        <v>12</v>
-      </c>
-      <c r="I27" s="1">
+      <c r="H27" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I27" t="s">
+        <v>12</v>
+      </c>
+      <c r="J27" s="1">
         <v>46151</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>15</v>
       </c>
@@ -1891,14 +2008,18 @@
       <c r="G28">
         <v>2.5</v>
       </c>
-      <c r="H28" t="s">
-        <v>12</v>
-      </c>
-      <c r="I28" s="1">
+      <c r="H28" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I28" t="s">
+        <v>12</v>
+      </c>
+      <c r="J28" s="1">
         <v>46187</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>37</v>
       </c>
@@ -1920,14 +2041,18 @@
       <c r="G29">
         <v>2</v>
       </c>
-      <c r="H29" t="s">
-        <v>12</v>
-      </c>
-      <c r="I29" s="1">
+      <c r="H29" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I29" t="s">
+        <v>12</v>
+      </c>
+      <c r="J29" s="1">
         <v>46093</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>71</v>
       </c>
@@ -1949,14 +2074,18 @@
       <c r="G30">
         <v>2</v>
       </c>
-      <c r="H30" t="s">
-        <v>12</v>
-      </c>
-      <c r="I30" s="1">
+      <c r="H30" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I30" t="s">
+        <v>12</v>
+      </c>
+      <c r="J30" s="1">
         <v>46151</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>88</v>
       </c>
@@ -1978,14 +2107,18 @@
       <c r="G31">
         <v>2</v>
       </c>
-      <c r="H31" t="s">
-        <v>12</v>
-      </c>
-      <c r="I31" s="1">
+      <c r="H31" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I31" t="s">
+        <v>12</v>
+      </c>
+      <c r="J31" s="1">
         <v>46204</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>76</v>
       </c>
@@ -2007,14 +2140,18 @@
       <c r="G32">
         <v>1.5</v>
       </c>
-      <c r="H32" t="s">
-        <v>12</v>
-      </c>
-      <c r="I32" s="1">
+      <c r="H32" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I32" t="s">
+        <v>12</v>
+      </c>
+      <c r="J32" s="1">
         <v>46034</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>92</v>
       </c>
@@ -2036,14 +2173,18 @@
       <c r="G33">
         <v>1.5</v>
       </c>
-      <c r="H33" t="s">
-        <v>12</v>
-      </c>
-      <c r="I33" s="1">
+      <c r="H33" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I33" t="s">
+        <v>12</v>
+      </c>
+      <c r="J33" s="1">
         <v>46030</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>10</v>
       </c>
@@ -2065,14 +2206,18 @@
       <c r="G34">
         <v>3</v>
       </c>
-      <c r="H34" t="s">
-        <v>12</v>
-      </c>
-      <c r="I34" s="1">
+      <c r="H34" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I34" t="s">
+        <v>12</v>
+      </c>
+      <c r="J34" s="1">
         <v>46182</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>23</v>
       </c>
@@ -2094,14 +2239,18 @@
       <c r="G35">
         <v>3</v>
       </c>
-      <c r="H35" t="s">
-        <v>12</v>
-      </c>
-      <c r="I35" s="1">
+      <c r="H35" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I35" t="s">
+        <v>12</v>
+      </c>
+      <c r="J35" s="1">
         <v>46057</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>54</v>
       </c>
@@ -2123,14 +2272,18 @@
       <c r="G36">
         <v>3</v>
       </c>
-      <c r="H36" t="s">
-        <v>12</v>
-      </c>
-      <c r="I36" s="1">
+      <c r="H36" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I36" t="s">
+        <v>12</v>
+      </c>
+      <c r="J36" s="1">
         <v>46125</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>12</v>
       </c>
@@ -2152,14 +2305,18 @@
       <c r="G37">
         <v>2.5</v>
       </c>
-      <c r="H37" t="s">
-        <v>12</v>
-      </c>
-      <c r="I37" s="1">
+      <c r="H37" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I37" t="s">
+        <v>12</v>
+      </c>
+      <c r="J37" s="1">
         <v>46043</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>63</v>
       </c>
@@ -2181,14 +2338,18 @@
       <c r="G38">
         <v>1</v>
       </c>
-      <c r="H38" t="s">
-        <v>12</v>
-      </c>
-      <c r="I38" s="1">
+      <c r="H38" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I38" t="s">
+        <v>12</v>
+      </c>
+      <c r="J38" s="1">
         <v>46135</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>95</v>
       </c>
@@ -2210,14 +2371,18 @@
       <c r="G39">
         <v>2.5</v>
       </c>
-      <c r="H39" t="s">
-        <v>12</v>
-      </c>
-      <c r="I39" s="1">
+      <c r="H39" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I39" t="s">
+        <v>12</v>
+      </c>
+      <c r="J39" s="1">
         <v>46065</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>84</v>
       </c>
@@ -2239,14 +2404,18 @@
       <c r="G40">
         <v>2</v>
       </c>
-      <c r="H40" t="s">
-        <v>12</v>
-      </c>
-      <c r="I40" s="1">
+      <c r="H40" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I40" t="s">
+        <v>12</v>
+      </c>
+      <c r="J40" s="1">
         <v>46142</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>33</v>
       </c>
@@ -2268,14 +2437,18 @@
       <c r="G41">
         <v>3</v>
       </c>
-      <c r="H41" t="s">
-        <v>12</v>
-      </c>
-      <c r="I41" s="1">
+      <c r="H41" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I41" t="s">
+        <v>12</v>
+      </c>
+      <c r="J41" s="1">
         <v>46066</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>100</v>
       </c>
@@ -2297,14 +2470,18 @@
       <c r="G42">
         <v>1.5</v>
       </c>
-      <c r="H42" t="s">
-        <v>12</v>
-      </c>
-      <c r="I42" s="1">
+      <c r="H42" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I42" t="s">
+        <v>12</v>
+      </c>
+      <c r="J42" s="1">
         <v>46202</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>3</v>
       </c>
@@ -2326,14 +2503,18 @@
       <c r="G43">
         <v>1</v>
       </c>
-      <c r="H43" t="s">
-        <v>12</v>
-      </c>
-      <c r="I43" s="1">
+      <c r="H43" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I43" t="s">
+        <v>12</v>
+      </c>
+      <c r="J43" s="1">
         <v>46170</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>7</v>
       </c>
@@ -2355,14 +2536,18 @@
       <c r="G44">
         <v>2</v>
       </c>
-      <c r="H44" t="s">
-        <v>12</v>
-      </c>
-      <c r="I44" s="1">
+      <c r="H44" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I44" t="s">
+        <v>12</v>
+      </c>
+      <c r="J44" s="1">
         <v>46174</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>20</v>
       </c>
@@ -2384,14 +2569,18 @@
       <c r="G45">
         <v>1</v>
       </c>
-      <c r="H45" t="s">
-        <v>12</v>
-      </c>
-      <c r="I45" s="1">
+      <c r="H45" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I45" t="s">
+        <v>12</v>
+      </c>
+      <c r="J45" s="1">
         <v>46041</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>62</v>
       </c>
@@ -2413,14 +2602,18 @@
       <c r="G46">
         <v>1</v>
       </c>
-      <c r="H46" t="s">
-        <v>12</v>
-      </c>
-      <c r="I46" s="1">
+      <c r="H46" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I46" t="s">
+        <v>12</v>
+      </c>
+      <c r="J46" s="1">
         <v>46133</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>24</v>
       </c>
@@ -2442,14 +2635,18 @@
       <c r="G47">
         <v>-0.5</v>
       </c>
-      <c r="H47" t="s">
+      <c r="H47" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I47" t="s">
         <v>17</v>
       </c>
-      <c r="I47" s="1">
+      <c r="J47" s="1">
         <v>46177</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>14</v>
       </c>
@@ -2471,14 +2668,18 @@
       <c r="G48">
         <v>-0.5</v>
       </c>
-      <c r="H48" t="s">
+      <c r="H48" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I48" t="s">
         <v>17</v>
       </c>
-      <c r="I48" s="1">
+      <c r="J48" s="1">
         <v>46119</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>49</v>
       </c>
@@ -2500,14 +2701,18 @@
       <c r="G49">
         <v>-0.5</v>
       </c>
-      <c r="H49" t="s">
+      <c r="H49" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I49" t="s">
         <v>17</v>
       </c>
-      <c r="I49" s="1">
+      <c r="J49" s="1">
         <v>46095</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>79</v>
       </c>
@@ -2529,14 +2734,18 @@
       <c r="G50">
         <v>-1</v>
       </c>
-      <c r="H50" t="s">
+      <c r="H50" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I50" t="s">
         <v>17</v>
       </c>
-      <c r="I50" s="1">
+      <c r="J50" s="1">
         <v>46128</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>40</v>
       </c>
@@ -2558,14 +2767,18 @@
       <c r="G51">
         <v>-1.5</v>
       </c>
-      <c r="H51" t="s">
+      <c r="H51" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I51" t="s">
         <v>17</v>
       </c>
-      <c r="I51" s="1">
+      <c r="J51" s="1">
         <v>46099</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>39</v>
       </c>
@@ -2587,14 +2800,18 @@
       <c r="G52">
         <v>-0.5</v>
       </c>
-      <c r="H52" t="s">
+      <c r="H52" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I52" t="s">
         <v>17</v>
       </c>
-      <c r="I52" s="1">
+      <c r="J52" s="1">
         <v>46164</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>29</v>
       </c>
@@ -2616,14 +2833,18 @@
       <c r="G53">
         <v>-0.5</v>
       </c>
-      <c r="H53" t="s">
+      <c r="H53" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I53" t="s">
         <v>17</v>
       </c>
-      <c r="I53" s="1">
+      <c r="J53" s="1">
         <v>46135</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>69</v>
       </c>
@@ -2645,14 +2866,18 @@
       <c r="G54">
         <v>-0.5</v>
       </c>
-      <c r="H54" t="s">
+      <c r="H54" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I54" t="s">
         <v>17</v>
       </c>
-      <c r="I54" s="1">
+      <c r="J54" s="1">
         <v>46042</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>22</v>
       </c>
@@ -2674,14 +2899,18 @@
       <c r="G55">
         <v>-1</v>
       </c>
-      <c r="H55" t="s">
+      <c r="H55" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I55" t="s">
         <v>17</v>
       </c>
-      <c r="I55" s="1">
+      <c r="J55" s="1">
         <v>46165</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>36</v>
       </c>
@@ -2703,14 +2932,18 @@
       <c r="G56">
         <v>-1.5</v>
       </c>
-      <c r="H56" t="s">
+      <c r="H56" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I56" t="s">
         <v>17</v>
       </c>
-      <c r="I56" s="1">
+      <c r="J56" s="1">
         <v>46057</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>32</v>
       </c>
@@ -2732,14 +2965,18 @@
       <c r="G57">
         <v>3</v>
       </c>
-      <c r="H57" t="s">
-        <v>12</v>
-      </c>
-      <c r="I57" s="1">
+      <c r="H57" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I57" t="s">
+        <v>12</v>
+      </c>
+      <c r="J57" s="1">
         <v>46027</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>73</v>
       </c>
@@ -2761,14 +2998,18 @@
       <c r="G58">
         <v>2.5</v>
       </c>
-      <c r="H58" t="s">
-        <v>12</v>
-      </c>
-      <c r="I58" s="1">
+      <c r="H58" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I58" t="s">
+        <v>12</v>
+      </c>
+      <c r="J58" s="1">
         <v>46191</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>74</v>
       </c>
@@ -2790,14 +3031,18 @@
       <c r="G59">
         <v>2.5</v>
       </c>
-      <c r="H59" t="s">
-        <v>12</v>
-      </c>
-      <c r="I59" s="1">
+      <c r="H59" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I59" t="s">
+        <v>12</v>
+      </c>
+      <c r="J59" s="1">
         <v>46081</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>87</v>
       </c>
@@ -2819,14 +3064,18 @@
       <c r="G60">
         <v>1.5</v>
       </c>
-      <c r="H60" t="s">
-        <v>12</v>
-      </c>
-      <c r="I60" s="1">
+      <c r="H60" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I60" t="s">
+        <v>12</v>
+      </c>
+      <c r="J60" s="1">
         <v>46203</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>65</v>
       </c>
@@ -2848,14 +3097,18 @@
       <c r="G61">
         <v>1.5</v>
       </c>
-      <c r="H61" t="s">
-        <v>12</v>
-      </c>
-      <c r="I61" s="1">
+      <c r="H61" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I61" t="s">
+        <v>12</v>
+      </c>
+      <c r="J61" s="1">
         <v>46167</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>26</v>
       </c>
@@ -2877,14 +3130,18 @@
       <c r="G62">
         <v>1</v>
       </c>
-      <c r="H62" t="s">
-        <v>12</v>
-      </c>
-      <c r="I62" s="1">
+      <c r="H62" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I62" t="s">
+        <v>12</v>
+      </c>
+      <c r="J62" s="1">
         <v>46173</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>55</v>
       </c>
@@ -2906,14 +3163,18 @@
       <c r="G63">
         <v>1</v>
       </c>
-      <c r="H63" t="s">
-        <v>12</v>
-      </c>
-      <c r="I63" s="1">
+      <c r="H63" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I63" t="s">
+        <v>12</v>
+      </c>
+      <c r="J63" s="1">
         <v>46120</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>59</v>
       </c>
@@ -2935,14 +3196,18 @@
       <c r="G64">
         <v>1</v>
       </c>
-      <c r="H64" t="s">
-        <v>12</v>
-      </c>
-      <c r="I64" s="1">
+      <c r="H64" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I64" t="s">
+        <v>12</v>
+      </c>
+      <c r="J64" s="1">
         <v>46140</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>66</v>
       </c>
@@ -2964,14 +3229,18 @@
       <c r="G65">
         <v>2</v>
       </c>
-      <c r="H65" t="s">
-        <v>12</v>
-      </c>
-      <c r="I65" s="1">
+      <c r="H65" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I65" t="s">
+        <v>12</v>
+      </c>
+      <c r="J65" s="1">
         <v>46160</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>2</v>
       </c>
@@ -2993,14 +3262,18 @@
       <c r="G66">
         <v>3</v>
       </c>
-      <c r="H66" t="s">
-        <v>12</v>
-      </c>
-      <c r="I66" s="1">
+      <c r="H66" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I66" t="s">
+        <v>12</v>
+      </c>
+      <c r="J66" s="1">
         <v>46178</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>94</v>
       </c>
@@ -3022,14 +3295,18 @@
       <c r="G67">
         <v>3</v>
       </c>
-      <c r="H67" t="s">
-        <v>12</v>
-      </c>
-      <c r="I67" s="1">
+      <c r="H67" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I67" t="s">
+        <v>12</v>
+      </c>
+      <c r="J67" s="1">
         <v>46091</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>57</v>
       </c>
@@ -3051,14 +3328,18 @@
       <c r="G68">
         <v>2.5</v>
       </c>
-      <c r="H68" t="s">
-        <v>12</v>
-      </c>
-      <c r="I68" s="1">
+      <c r="H68" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I68" t="s">
+        <v>12</v>
+      </c>
+      <c r="J68" s="1">
         <v>46076</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>4</v>
       </c>
@@ -3080,14 +3361,18 @@
       <c r="G69">
         <v>2</v>
       </c>
-      <c r="H69" t="s">
-        <v>12</v>
-      </c>
-      <c r="I69" s="1">
+      <c r="H69" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I69" t="s">
+        <v>12</v>
+      </c>
+      <c r="J69" s="1">
         <v>46205</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>27</v>
       </c>
@@ -3109,14 +3394,18 @@
       <c r="G70">
         <v>1</v>
       </c>
-      <c r="H70" t="s">
-        <v>12</v>
-      </c>
-      <c r="I70" s="1">
+      <c r="H70" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I70" t="s">
+        <v>12</v>
+      </c>
+      <c r="J70" s="1">
         <v>46117</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>72</v>
       </c>
@@ -3138,14 +3427,18 @@
       <c r="G71">
         <v>1</v>
       </c>
-      <c r="H71" t="s">
-        <v>12</v>
-      </c>
-      <c r="I71" s="1">
+      <c r="H71" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I71" t="s">
+        <v>12</v>
+      </c>
+      <c r="J71" s="1">
         <v>46069</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>75</v>
       </c>
@@ -3167,14 +3460,18 @@
       <c r="G72">
         <v>1</v>
       </c>
-      <c r="H72" t="s">
-        <v>12</v>
-      </c>
-      <c r="I72" s="1">
+      <c r="H72" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I72" t="s">
+        <v>12</v>
+      </c>
+      <c r="J72" s="1">
         <v>46047</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>17</v>
       </c>
@@ -3196,14 +3493,18 @@
       <c r="G73">
         <v>-1.5</v>
       </c>
-      <c r="H73" t="s">
+      <c r="H73" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I73" t="s">
         <v>17</v>
       </c>
-      <c r="I73" s="1">
+      <c r="J73" s="1">
         <v>46067</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>53</v>
       </c>
@@ -3225,14 +3526,18 @@
       <c r="G74">
         <v>-1.5</v>
       </c>
-      <c r="H74" t="s">
+      <c r="H74" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I74" t="s">
         <v>17</v>
       </c>
-      <c r="I74" s="1">
+      <c r="J74" s="1">
         <v>46054</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>21</v>
       </c>
@@ -3254,14 +3559,18 @@
       <c r="G75">
         <v>-1</v>
       </c>
-      <c r="H75" t="s">
+      <c r="H75" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I75" t="s">
         <v>17</v>
       </c>
-      <c r="I75" s="1">
+      <c r="J75" s="1">
         <v>46059</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>48</v>
       </c>
@@ -3283,14 +3592,18 @@
       <c r="G76">
         <v>-1</v>
       </c>
-      <c r="H76" t="s">
+      <c r="H76" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I76" t="s">
         <v>17</v>
       </c>
-      <c r="I76" s="1">
+      <c r="J76" s="1">
         <v>46072</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>83</v>
       </c>
@@ -3312,14 +3625,18 @@
       <c r="G77">
         <v>-0.5</v>
       </c>
-      <c r="H77" t="s">
+      <c r="H77" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I77" t="s">
         <v>17</v>
       </c>
-      <c r="I77" s="1">
+      <c r="J77" s="1">
         <v>46146</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>5</v>
       </c>
@@ -3341,14 +3658,18 @@
       <c r="G78">
         <v>-0.5</v>
       </c>
-      <c r="H78" t="s">
+      <c r="H78" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I78" t="s">
         <v>17</v>
       </c>
-      <c r="I78" s="1">
+      <c r="J78" s="1">
         <v>46050</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>31</v>
       </c>
@@ -3370,14 +3691,18 @@
       <c r="G79">
         <v>-0.5</v>
       </c>
-      <c r="H79" t="s">
+      <c r="H79" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I79" t="s">
         <v>17</v>
       </c>
-      <c r="I79" s="1">
+      <c r="J79" s="1">
         <v>46131</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>96</v>
       </c>
@@ -3399,14 +3724,18 @@
       <c r="G80">
         <v>-1</v>
       </c>
-      <c r="H80" t="s">
+      <c r="H80" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I80" t="s">
         <v>17</v>
       </c>
-      <c r="I80" s="1">
+      <c r="J80" s="1">
         <v>46160</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>64</v>
       </c>
@@ -3428,14 +3757,18 @@
       <c r="G81">
         <v>-1.5</v>
       </c>
-      <c r="H81" t="s">
+      <c r="H81" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I81" t="s">
         <v>17</v>
       </c>
-      <c r="I81" s="1">
+      <c r="J81" s="1">
         <v>46061</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>81</v>
       </c>
@@ -3457,14 +3790,18 @@
       <c r="G82">
         <v>-1.5</v>
       </c>
-      <c r="H82" t="s">
+      <c r="H82" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I82" t="s">
         <v>17</v>
       </c>
-      <c r="I82" s="1">
+      <c r="J82" s="1">
         <v>46030</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>82</v>
       </c>
@@ -3486,14 +3823,18 @@
       <c r="G83">
         <v>-1.5</v>
       </c>
-      <c r="H83" t="s">
+      <c r="H83" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I83" t="s">
         <v>17</v>
       </c>
-      <c r="I83" s="1">
+      <c r="J83" s="1">
         <v>46066</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>90</v>
       </c>
@@ -3515,14 +3856,18 @@
       <c r="G84">
         <v>2.5</v>
       </c>
-      <c r="H84" t="s">
-        <v>12</v>
-      </c>
-      <c r="I84" s="1">
+      <c r="H84" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I84" t="s">
+        <v>12</v>
+      </c>
+      <c r="J84" s="1">
         <v>46076</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>50</v>
       </c>
@@ -3544,14 +3889,18 @@
       <c r="G85">
         <v>1.5</v>
       </c>
-      <c r="H85" t="s">
-        <v>12</v>
-      </c>
-      <c r="I85" s="1">
+      <c r="H85" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I85" t="s">
+        <v>12</v>
+      </c>
+      <c r="J85" s="1">
         <v>46144</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>91</v>
       </c>
@@ -3573,14 +3922,18 @@
       <c r="G86">
         <v>1.5</v>
       </c>
-      <c r="H86" t="s">
-        <v>12</v>
-      </c>
-      <c r="I86" s="1">
+      <c r="H86" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I86" t="s">
+        <v>12</v>
+      </c>
+      <c r="J86" s="1">
         <v>46177</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>28</v>
       </c>
@@ -3602,14 +3955,18 @@
       <c r="G87">
         <v>2.5</v>
       </c>
-      <c r="H87" t="s">
-        <v>12</v>
-      </c>
-      <c r="I87" s="1">
+      <c r="H87" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I87" t="s">
+        <v>12</v>
+      </c>
+      <c r="J87" s="1">
         <v>46130</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>67</v>
       </c>
@@ -3631,14 +3988,18 @@
       <c r="G88">
         <v>2.5</v>
       </c>
-      <c r="H88" t="s">
-        <v>12</v>
-      </c>
-      <c r="I88" s="1">
+      <c r="H88" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I88" t="s">
+        <v>12</v>
+      </c>
+      <c r="J88" s="1">
         <v>46096</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>60</v>
       </c>
@@ -3660,14 +4021,18 @@
       <c r="G89">
         <v>1.5</v>
       </c>
-      <c r="H89" t="s">
-        <v>12</v>
-      </c>
-      <c r="I89" s="1">
+      <c r="H89" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I89" t="s">
+        <v>12</v>
+      </c>
+      <c r="J89" s="1">
         <v>46158</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>41</v>
       </c>
@@ -3689,14 +4054,18 @@
       <c r="G90">
         <v>1</v>
       </c>
-      <c r="H90" t="s">
-        <v>12</v>
-      </c>
-      <c r="I90" s="1">
+      <c r="H90" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I90" t="s">
+        <v>12</v>
+      </c>
+      <c r="J90" s="1">
         <v>46197</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>89</v>
       </c>
@@ -3718,14 +4087,18 @@
       <c r="G91">
         <v>1.5</v>
       </c>
-      <c r="H91" t="s">
-        <v>12</v>
-      </c>
-      <c r="I91" s="1">
+      <c r="H91" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="I91" t="s">
+        <v>12</v>
+      </c>
+      <c r="J91" s="1">
         <v>46167</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>25</v>
       </c>
@@ -3747,14 +4120,18 @@
       <c r="G92">
         <v>-0.5</v>
       </c>
-      <c r="H92" t="s">
+      <c r="H92" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I92" t="s">
         <v>17</v>
       </c>
-      <c r="I92" s="1">
+      <c r="J92" s="1">
         <v>46035</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>9</v>
       </c>
@@ -3776,14 +4153,18 @@
       <c r="G93">
         <v>-1.5</v>
       </c>
-      <c r="H93" t="s">
+      <c r="H93" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I93" t="s">
         <v>17</v>
       </c>
-      <c r="I93" s="1">
+      <c r="J93" s="1">
         <v>46121</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>18</v>
       </c>
@@ -3805,14 +4186,18 @@
       <c r="G94">
         <v>-1.5</v>
       </c>
-      <c r="H94" t="s">
+      <c r="H94" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I94" t="s">
         <v>17</v>
       </c>
-      <c r="I94" s="1">
+      <c r="J94" s="1">
         <v>46187</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>44</v>
       </c>
@@ -3834,14 +4219,18 @@
       <c r="G95">
         <v>-1.5</v>
       </c>
-      <c r="H95" t="s">
+      <c r="H95" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I95" t="s">
         <v>17</v>
       </c>
-      <c r="I95" s="1">
+      <c r="J95" s="1">
         <v>46190</v>
       </c>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>19</v>
       </c>
@@ -3863,14 +4252,18 @@
       <c r="G96">
         <v>-1</v>
       </c>
-      <c r="H96" t="s">
+      <c r="H96" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I96" t="s">
         <v>17</v>
       </c>
-      <c r="I96" s="1">
+      <c r="J96" s="1">
         <v>46180</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>56</v>
       </c>
@@ -3892,14 +4285,18 @@
       <c r="G97">
         <v>-1.5</v>
       </c>
-      <c r="H97" t="s">
+      <c r="H97" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I97" t="s">
         <v>17</v>
       </c>
-      <c r="I97" s="1">
+      <c r="J97" s="1">
         <v>46156</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>11</v>
       </c>
@@ -3921,14 +4318,18 @@
       <c r="G98">
         <v>-1</v>
       </c>
-      <c r="H98" t="s">
+      <c r="H98" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I98" t="s">
         <v>17</v>
       </c>
-      <c r="I98" s="1">
+      <c r="J98" s="1">
         <v>46202</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>51</v>
       </c>
@@ -3950,14 +4351,18 @@
       <c r="G99">
         <v>-1</v>
       </c>
-      <c r="H99" t="s">
+      <c r="H99" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I99" t="s">
         <v>17</v>
       </c>
-      <c r="I99" s="1">
+      <c r="J99" s="1">
         <v>46111</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>42</v>
       </c>
@@ -3979,14 +4384,18 @@
       <c r="G100">
         <v>-1</v>
       </c>
-      <c r="H100" t="s">
+      <c r="H100" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I100" t="s">
         <v>17</v>
       </c>
-      <c r="I100" s="1">
+      <c r="J100" s="1">
         <v>46096</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>58</v>
       </c>
@@ -4008,10 +4417,14 @@
       <c r="G101">
         <v>-1</v>
       </c>
-      <c r="H101" t="s">
+      <c r="H101" t="str">
+        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
+      </c>
+      <c r="I101" t="s">
         <v>17</v>
       </c>
-      <c r="I101" s="1">
+      <c r="J101" s="1">
         <v>46104</v>
       </c>
     </row>

</xml_diff>

<commit_message>
hnaya zadt function dyal OR F if function
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D794754C-129F-4AFB-AD6A-570610D33694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{105E9416-9D0D-4910-B55A-F12230914383}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -759,7 +759,7 @@
     <tableColumn id="6" xr3:uid="{BFF7C4D2-29D9-4645-98DB-6FBF609AB80F}" name="Profit"/>
     <tableColumn id="7" xr3:uid="{CD8DBAA1-576E-4991-87E5-049F5C232A1F}" name="R"/>
     <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="0">
-      <calculatedColumnFormula>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{CC96218F-2F0A-46BB-98E4-8AE8218DB3D7}" name="Result"/>
     <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="1"/>
@@ -1151,7 +1151,7 @@
         <v>3</v>
       </c>
       <c r="H2" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I2" t="s">
@@ -1184,7 +1184,7 @@
         <v>3</v>
       </c>
       <c r="H3" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I3" t="s">
@@ -1217,7 +1217,7 @@
         <v>2</v>
       </c>
       <c r="H4" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I4" t="s">
@@ -1250,7 +1250,7 @@
         <v>2</v>
       </c>
       <c r="H5" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I5" t="s">
@@ -1283,8 +1283,8 @@
         <v>1.5</v>
       </c>
       <c r="H6" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I6" t="s">
         <v>12</v>
@@ -1316,8 +1316,8 @@
         <v>1.5</v>
       </c>
       <c r="H7" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I7" t="s">
         <v>12</v>
@@ -1349,7 +1349,7 @@
         <v>2</v>
       </c>
       <c r="H8" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I8" t="s">
@@ -1382,7 +1382,7 @@
         <v>2</v>
       </c>
       <c r="H9" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I9" t="s">
@@ -1415,7 +1415,7 @@
         <v>2.5</v>
       </c>
       <c r="H10" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I10" t="s">
@@ -1448,8 +1448,8 @@
         <v>1</v>
       </c>
       <c r="H11" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I11" t="s">
         <v>12</v>
@@ -1481,8 +1481,8 @@
         <v>1.5</v>
       </c>
       <c r="H12" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I12" t="s">
         <v>12</v>
@@ -1514,8 +1514,8 @@
         <v>1</v>
       </c>
       <c r="H13" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I13" t="s">
         <v>12</v>
@@ -1547,7 +1547,7 @@
         <v>-0.5</v>
       </c>
       <c r="H14" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I14" t="s">
@@ -1580,7 +1580,7 @@
         <v>-0.5</v>
       </c>
       <c r="H15" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I15" t="s">
@@ -1613,7 +1613,7 @@
         <v>-0.5</v>
       </c>
       <c r="H16" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I16" t="s">
@@ -1646,7 +1646,7 @@
         <v>-0.5</v>
       </c>
       <c r="H17" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I17" t="s">
@@ -1679,7 +1679,7 @@
         <v>-1</v>
       </c>
       <c r="H18" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I18" t="s">
@@ -1712,7 +1712,7 @@
         <v>-1</v>
       </c>
       <c r="H19" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I19" t="s">
@@ -1745,7 +1745,7 @@
         <v>-1</v>
       </c>
       <c r="H20" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I20" t="s">
@@ -1778,7 +1778,7 @@
         <v>-1</v>
       </c>
       <c r="H21" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I21" t="s">
@@ -1811,7 +1811,7 @@
         <v>-0.5</v>
       </c>
       <c r="H22" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I22" t="s">
@@ -1844,7 +1844,7 @@
         <v>-1.5</v>
       </c>
       <c r="H23" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I23" t="s">
@@ -1877,7 +1877,7 @@
         <v>3</v>
       </c>
       <c r="H24" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I24" t="s">
@@ -1910,7 +1910,7 @@
         <v>3</v>
       </c>
       <c r="H25" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I25" t="s">
@@ -1943,7 +1943,7 @@
         <v>2.5</v>
       </c>
       <c r="H26" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I26" t="s">
@@ -1976,7 +1976,7 @@
         <v>3</v>
       </c>
       <c r="H27" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I27" t="s">
@@ -2009,7 +2009,7 @@
         <v>2.5</v>
       </c>
       <c r="H28" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I28" t="s">
@@ -2042,7 +2042,7 @@
         <v>2</v>
       </c>
       <c r="H29" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I29" t="s">
@@ -2075,7 +2075,7 @@
         <v>2</v>
       </c>
       <c r="H30" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I30" t="s">
@@ -2108,7 +2108,7 @@
         <v>2</v>
       </c>
       <c r="H31" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I31" t="s">
@@ -2141,8 +2141,8 @@
         <v>1.5</v>
       </c>
       <c r="H32" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I32" t="s">
         <v>12</v>
@@ -2174,8 +2174,8 @@
         <v>1.5</v>
       </c>
       <c r="H33" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I33" t="s">
         <v>12</v>
@@ -2207,7 +2207,7 @@
         <v>3</v>
       </c>
       <c r="H34" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I34" t="s">
@@ -2240,7 +2240,7 @@
         <v>3</v>
       </c>
       <c r="H35" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I35" t="s">
@@ -2273,7 +2273,7 @@
         <v>3</v>
       </c>
       <c r="H36" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I36" t="s">
@@ -2306,7 +2306,7 @@
         <v>2.5</v>
       </c>
       <c r="H37" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I37" t="s">
@@ -2339,8 +2339,8 @@
         <v>1</v>
       </c>
       <c r="H38" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I38" t="s">
         <v>12</v>
@@ -2372,7 +2372,7 @@
         <v>2.5</v>
       </c>
       <c r="H39" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I39" t="s">
@@ -2405,7 +2405,7 @@
         <v>2</v>
       </c>
       <c r="H40" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I40" t="s">
@@ -2438,7 +2438,7 @@
         <v>3</v>
       </c>
       <c r="H41" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I41" t="s">
@@ -2471,8 +2471,8 @@
         <v>1.5</v>
       </c>
       <c r="H42" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I42" t="s">
         <v>12</v>
@@ -2504,8 +2504,8 @@
         <v>1</v>
       </c>
       <c r="H43" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I43" t="s">
         <v>12</v>
@@ -2537,7 +2537,7 @@
         <v>2</v>
       </c>
       <c r="H44" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I44" t="s">
@@ -2570,8 +2570,8 @@
         <v>1</v>
       </c>
       <c r="H45" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I45" t="s">
         <v>12</v>
@@ -2603,8 +2603,8 @@
         <v>1</v>
       </c>
       <c r="H46" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I46" t="s">
         <v>12</v>
@@ -2636,7 +2636,7 @@
         <v>-0.5</v>
       </c>
       <c r="H47" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I47" t="s">
@@ -2669,7 +2669,7 @@
         <v>-0.5</v>
       </c>
       <c r="H48" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I48" t="s">
@@ -2702,7 +2702,7 @@
         <v>-0.5</v>
       </c>
       <c r="H49" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I49" t="s">
@@ -2735,7 +2735,7 @@
         <v>-1</v>
       </c>
       <c r="H50" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I50" t="s">
@@ -2768,7 +2768,7 @@
         <v>-1.5</v>
       </c>
       <c r="H51" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I51" t="s">
@@ -2801,7 +2801,7 @@
         <v>-0.5</v>
       </c>
       <c r="H52" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I52" t="s">
@@ -2834,7 +2834,7 @@
         <v>-0.5</v>
       </c>
       <c r="H53" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I53" t="s">
@@ -2867,7 +2867,7 @@
         <v>-0.5</v>
       </c>
       <c r="H54" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I54" t="s">
@@ -2900,7 +2900,7 @@
         <v>-1</v>
       </c>
       <c r="H55" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I55" t="s">
@@ -2933,7 +2933,7 @@
         <v>-1.5</v>
       </c>
       <c r="H56" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I56" t="s">
@@ -2966,7 +2966,7 @@
         <v>3</v>
       </c>
       <c r="H57" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I57" t="s">
@@ -2999,7 +2999,7 @@
         <v>2.5</v>
       </c>
       <c r="H58" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I58" t="s">
@@ -3032,7 +3032,7 @@
         <v>2.5</v>
       </c>
       <c r="H59" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I59" t="s">
@@ -3065,8 +3065,8 @@
         <v>1.5</v>
       </c>
       <c r="H60" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I60" t="s">
         <v>12</v>
@@ -3098,8 +3098,8 @@
         <v>1.5</v>
       </c>
       <c r="H61" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I61" t="s">
         <v>12</v>
@@ -3131,8 +3131,8 @@
         <v>1</v>
       </c>
       <c r="H62" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I62" t="s">
         <v>12</v>
@@ -3164,8 +3164,8 @@
         <v>1</v>
       </c>
       <c r="H63" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I63" t="s">
         <v>12</v>
@@ -3197,8 +3197,8 @@
         <v>1</v>
       </c>
       <c r="H64" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I64" t="s">
         <v>12</v>
@@ -3230,7 +3230,7 @@
         <v>2</v>
       </c>
       <c r="H65" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I65" t="s">
@@ -3263,7 +3263,7 @@
         <v>3</v>
       </c>
       <c r="H66" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I66" t="s">
@@ -3296,7 +3296,7 @@
         <v>3</v>
       </c>
       <c r="H67" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I67" t="s">
@@ -3329,7 +3329,7 @@
         <v>2.5</v>
       </c>
       <c r="H68" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I68" t="s">
@@ -3362,7 +3362,7 @@
         <v>2</v>
       </c>
       <c r="H69" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I69" t="s">
@@ -3395,8 +3395,8 @@
         <v>1</v>
       </c>
       <c r="H70" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I70" t="s">
         <v>12</v>
@@ -3428,8 +3428,8 @@
         <v>1</v>
       </c>
       <c r="H71" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I71" t="s">
         <v>12</v>
@@ -3461,8 +3461,8 @@
         <v>1</v>
       </c>
       <c r="H72" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I72" t="s">
         <v>12</v>
@@ -3494,7 +3494,7 @@
         <v>-1.5</v>
       </c>
       <c r="H73" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I73" t="s">
@@ -3527,7 +3527,7 @@
         <v>-1.5</v>
       </c>
       <c r="H74" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I74" t="s">
@@ -3560,7 +3560,7 @@
         <v>-1</v>
       </c>
       <c r="H75" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I75" t="s">
@@ -3593,7 +3593,7 @@
         <v>-1</v>
       </c>
       <c r="H76" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I76" t="s">
@@ -3626,7 +3626,7 @@
         <v>-0.5</v>
       </c>
       <c r="H77" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I77" t="s">
@@ -3659,7 +3659,7 @@
         <v>-0.5</v>
       </c>
       <c r="H78" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I78" t="s">
@@ -3692,7 +3692,7 @@
         <v>-0.5</v>
       </c>
       <c r="H79" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I79" t="s">
@@ -3725,7 +3725,7 @@
         <v>-1</v>
       </c>
       <c r="H80" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I80" t="s">
@@ -3758,7 +3758,7 @@
         <v>-1.5</v>
       </c>
       <c r="H81" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I81" t="s">
@@ -3791,7 +3791,7 @@
         <v>-1.5</v>
       </c>
       <c r="H82" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I82" t="s">
@@ -3824,7 +3824,7 @@
         <v>-1.5</v>
       </c>
       <c r="H83" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I83" t="s">
@@ -3857,7 +3857,7 @@
         <v>2.5</v>
       </c>
       <c r="H84" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I84" t="s">
@@ -3890,8 +3890,8 @@
         <v>1.5</v>
       </c>
       <c r="H85" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I85" t="s">
         <v>12</v>
@@ -3923,8 +3923,8 @@
         <v>1.5</v>
       </c>
       <c r="H86" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I86" t="s">
         <v>12</v>
@@ -3956,7 +3956,7 @@
         <v>2.5</v>
       </c>
       <c r="H87" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I87" t="s">
@@ -3989,7 +3989,7 @@
         <v>2.5</v>
       </c>
       <c r="H88" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>GOOD</v>
       </c>
       <c r="I88" t="s">
@@ -4022,8 +4022,8 @@
         <v>1.5</v>
       </c>
       <c r="H89" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I89" t="s">
         <v>12</v>
@@ -4055,8 +4055,8 @@
         <v>1</v>
       </c>
       <c r="H90" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I90" t="s">
         <v>12</v>
@@ -4088,8 +4088,8 @@
         <v>1.5</v>
       </c>
       <c r="H91" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
-        <v>GOOD</v>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
+        <v>REVIEW</v>
       </c>
       <c r="I91" t="s">
         <v>12</v>
@@ -4121,7 +4121,7 @@
         <v>-0.5</v>
       </c>
       <c r="H92" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I92" t="s">
@@ -4154,7 +4154,7 @@
         <v>-1.5</v>
       </c>
       <c r="H93" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I93" t="s">
@@ -4187,7 +4187,7 @@
         <v>-1.5</v>
       </c>
       <c r="H94" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I94" t="s">
@@ -4220,7 +4220,7 @@
         <v>-1.5</v>
       </c>
       <c r="H95" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I95" t="s">
@@ -4253,7 +4253,7 @@
         <v>-1</v>
       </c>
       <c r="H96" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I96" t="s">
@@ -4286,7 +4286,7 @@
         <v>-1.5</v>
       </c>
       <c r="H97" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I97" t="s">
@@ -4319,7 +4319,7 @@
         <v>-1</v>
       </c>
       <c r="H98" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I98" t="s">
@@ -4352,7 +4352,7 @@
         <v>-1</v>
       </c>
       <c r="H99" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I99" t="s">
@@ -4385,7 +4385,7 @@
         <v>-1</v>
       </c>
       <c r="H100" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I100" t="s">
@@ -4418,7 +4418,7 @@
         <v>-1</v>
       </c>
       <c r="H101" t="str">
-        <f>IF(AND(Table1[[#This Row],[R]]&gt;=1,Table1[[#This Row],[Profit]]),"GOOD","REVIEW")</f>
+        <f>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</f>
         <v>REVIEW</v>
       </c>
       <c r="I101" t="s">

</xml_diff>

<commit_message>
hnaya zadt sheet akhra kan9ra fiha kifch nsla7 data li machi clean
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2BA9421-A467-439E-946D-DB3F52964D9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACCAE8A5-324B-4A5F-A234-44EA56BD4249}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
     <sheet name="trading_raw_data2" sheetId="1" r:id="rId1"/>
     <sheet name="data analysis" sheetId="2" r:id="rId2"/>
+    <sheet name="data cleaning " sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="47">
   <si>
     <t>TradeID</t>
   </si>
@@ -151,6 +152,33 @@
   </si>
   <si>
     <t>Profit per R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">missing value </t>
+  </si>
+  <si>
+    <t>columns</t>
+  </si>
+  <si>
+    <t>count R NUMBER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   eurusd</t>
+  </si>
+  <si>
+    <t>eurusd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    eurusd</t>
+  </si>
+  <si>
+    <t>gold</t>
+  </si>
+  <si>
+    <t>us30</t>
+  </si>
+  <si>
+    <t>Clean Space</t>
   </si>
 </sst>
 </file>
@@ -670,7 +698,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -683,6 +711,7 @@
     <xf numFmtId="0" fontId="0" fillId="33" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -729,15 +758,48 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="7">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -766,16 +828,30 @@
     <tableColumn id="5" xr3:uid="{539426CC-F875-4D64-977A-05C6F1BCDBCD}" name="Direction"/>
     <tableColumn id="6" xr3:uid="{BFF7C4D2-29D9-4645-98DB-6FBF609AB80F}" name="Profit"/>
     <tableColumn id="7" xr3:uid="{CD8DBAA1-576E-4991-87E5-049F5C232A1F}" name="R"/>
-    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="1">
+    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="6">
       <calculatedColumnFormula>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="0">
+    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="5">
       <calculatedColumnFormula>IFERROR(Table1[[#This Row],[Profit]]/Table1[[#This Row],[R]],"0")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{CC96218F-2F0A-46BB-98E4-8AE8218DB3D7}" name="Result"/>
-    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5280782B-FEC2-415C-8A49-51730C483074}" name="Table2" displayName="Table2" ref="F8:H13" totalsRowShown="0">
+  <autoFilter ref="F8:H13" xr:uid="{5280782B-FEC2-415C-8A49-51730C483074}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{DAF88BD0-F115-4C64-AE11-7DD8AB7505A7}" name="Pair"/>
+    <tableColumn id="2" xr3:uid="{89E35073-D474-496E-86E0-7646DF314B64}" name="Profit"/>
+    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="0">
+      <calculatedColumnFormula>TRIM(Table2[[#This Row],[Pair]])</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1101,7 +1177,7 @@
   <cols>
     <col min="1" max="1" width="9.33203125" customWidth="1"/>
     <col min="2" max="2" width="11.44140625" customWidth="1"/>
-    <col min="4" max="4" width="9.33203125" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="10.5546875" customWidth="1"/>
     <col min="8" max="8" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.44140625" customWidth="1"/>
@@ -4844,6 +4920,12 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A1">
+    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
@@ -4854,9 +4936,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC7DF93-3E77-4DA9-9925-C234221B379B}">
-  <dimension ref="C5:N19"/>
+  <dimension ref="B5:N30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="2" max="2" width="28.88671875" customWidth="1"/>
     <col min="3" max="3" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="16.109375" customWidth="1"/>
     <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
@@ -5078,7 +5161,7 @@
         <v>311.81818181818176</v>
       </c>
     </row>
-    <row r="17" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:14" x14ac:dyDescent="0.3">
       <c r="C17" s="3" t="s">
         <v>13</v>
       </c>
@@ -5127,7 +5210,7 @@
         <v>355.38720538720537</v>
       </c>
     </row>
-    <row r="18" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:14" x14ac:dyDescent="0.3">
       <c r="C18" s="3" t="s">
         <v>18</v>
       </c>
@@ -5176,8 +5259,104 @@
         <v>274.4444444444444</v>
       </c>
     </row>
-    <row r="19" spans="3:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:14" x14ac:dyDescent="0.3">
       <c r="I19" s="7"/>
+    </row>
+    <row r="21" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D21" t="s">
+        <v>40</v>
+      </c>
+      <c r="E21">
+        <f>COUNT(Table1[R])</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C22">
+        <f>COUNTBLANK(Table1[Profit])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B23" t="s">
+        <v>0</v>
+      </c>
+      <c r="C23">
+        <f>COUNTBLANK(Table1[TradeID])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C24">
+        <f>COUNTBLANK(Table1[AccountID])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B25" t="s">
+        <v>2</v>
+      </c>
+      <c r="C25">
+        <f>COUNTBLANK(Table1[Pair])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B26" t="s">
+        <v>3</v>
+      </c>
+      <c r="C26">
+        <f>COUNTBLANK(Table1[Session])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B27" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27">
+        <f>COUNTBLANK(Table1[Direction])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B28" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28">
+        <f>COUNTBLANK(Table1[R])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B29" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29">
+        <f>COUNTBLANK(Table1[Result])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B30" t="s">
+        <v>8</v>
+      </c>
+      <c r="C30">
+        <f>COUNTBLANK(Table1[TradeDate])</f>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C15:J18">
@@ -5186,4 +5365,93 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDB00B21-86E3-4E60-9B16-646B4376A26A}">
+  <dimension ref="F8:H13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="6" max="6" width="13.33203125" customWidth="1"/>
+    <col min="7" max="7" width="17.77734375" customWidth="1"/>
+    <col min="8" max="8" width="18.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="8" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="F8" t="s">
+        <v>2</v>
+      </c>
+      <c r="G8" t="s">
+        <v>5</v>
+      </c>
+      <c r="H8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="F9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9">
+        <v>749</v>
+      </c>
+      <c r="H9" t="str">
+        <f>TRIM(Table2[[#This Row],[Pair]])</f>
+        <v>eurusd</v>
+      </c>
+    </row>
+    <row r="10" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="F10" t="s">
+        <v>42</v>
+      </c>
+      <c r="G10">
+        <v>3773</v>
+      </c>
+      <c r="H10" t="str">
+        <f>TRIM(Table2[[#This Row],[Pair]])</f>
+        <v>eurusd</v>
+      </c>
+    </row>
+    <row r="11" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="F11" t="s">
+        <v>43</v>
+      </c>
+      <c r="G11">
+        <v>8383</v>
+      </c>
+      <c r="H11" t="str">
+        <f>TRIM(Table2[[#This Row],[Pair]])</f>
+        <v>eurusd</v>
+      </c>
+    </row>
+    <row r="12" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="F12" t="s">
+        <v>44</v>
+      </c>
+      <c r="G12">
+        <v>774</v>
+      </c>
+      <c r="H12" t="str">
+        <f>TRIM(Table2[[#This Row],[Pair]])</f>
+        <v>gold</v>
+      </c>
+    </row>
+    <row r="13" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="F13" t="s">
+        <v>45</v>
+      </c>
+      <c r="G13">
+        <v>88</v>
+      </c>
+      <c r="H13" t="str">
+        <f>TRIM(Table2[[#This Row],[Pair]])</f>
+        <v>us30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
hanaya akn3lam trim data w upper w lower w proper
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACCAE8A5-324B-4A5F-A234-44EA56BD4249}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CACBBB4-450B-4FF3-AF1D-82EC4D263598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="455" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="55">
   <si>
     <t>TradeID</t>
   </si>
@@ -179,6 +179,30 @@
   </si>
   <si>
     <t>Clean Space</t>
+  </si>
+  <si>
+    <t>trim</t>
+  </si>
+  <si>
+    <t>check trim</t>
+  </si>
+  <si>
+    <t>raw text</t>
+  </si>
+  <si>
+    <t>text</t>
+  </si>
+  <si>
+    <t>eur</t>
+  </si>
+  <si>
+    <t>GOLD</t>
+  </si>
+  <si>
+    <t>ud30</t>
+  </si>
+  <si>
+    <t>oil</t>
   </si>
 </sst>
 </file>
@@ -698,7 +722,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -712,6 +736,9 @@
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -758,7 +785,13 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="9">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -828,27 +861,43 @@
     <tableColumn id="5" xr3:uid="{539426CC-F875-4D64-977A-05C6F1BCDBCD}" name="Direction"/>
     <tableColumn id="6" xr3:uid="{BFF7C4D2-29D9-4645-98DB-6FBF609AB80F}" name="Profit"/>
     <tableColumn id="7" xr3:uid="{CD8DBAA1-576E-4991-87E5-049F5C232A1F}" name="R"/>
-    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="6">
+    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="8">
       <calculatedColumnFormula>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="5">
+    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="7">
       <calculatedColumnFormula>IFERROR(Table1[[#This Row],[Profit]]/Table1[[#This Row],[R]],"0")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{CC96218F-2F0A-46BB-98E4-8AE8218DB3D7}" name="Result"/>
-    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5280782B-FEC2-415C-8A49-51730C483074}" name="Table2" displayName="Table2" ref="F8:H13" totalsRowShown="0">
-  <autoFilter ref="F8:H13" xr:uid="{5280782B-FEC2-415C-8A49-51730C483074}"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5280782B-FEC2-415C-8A49-51730C483074}" name="Table2" displayName="Table2" ref="F8:I13" totalsRowShown="0">
+  <autoFilter ref="F8:I13" xr:uid="{5280782B-FEC2-415C-8A49-51730C483074}"/>
+  <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{DAF88BD0-F115-4C64-AE11-7DD8AB7505A7}" name="Pair"/>
     <tableColumn id="2" xr3:uid="{89E35073-D474-496E-86E0-7646DF314B64}" name="Profit"/>
-    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="0">
+    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="2">
       <calculatedColumnFormula>TRIM(Table2[[#This Row],[Pair]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="1">
+      <calculatedColumnFormula>IF(Table2[[#This Row],[Pair]]=Table2[[#This Row],[Clean Space]],"GOOD","NADFO")</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A99A2C5F-61E0-444B-907C-487860A13E40}" name="Table4" displayName="Table4" ref="K8:L12" totalsRowShown="0">
+  <autoFilter ref="K8:L12" xr:uid="{A99A2C5F-61E0-444B-907C-487860A13E40}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{0A321640-D79C-4135-83F6-E38913427047}" name="raw text"/>
+    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="0">
+      <calculatedColumnFormula>PROPER(Table4[[#This Row],[raw text]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -4921,10 +4970,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5369,15 +5418,23 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDB00B21-86E3-4E60-9B16-646B4376A26A}">
-  <dimension ref="F8:H13"/>
+  <dimension ref="F7:L13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="6" width="13.33203125" customWidth="1"/>
     <col min="7" max="7" width="17.77734375" customWidth="1"/>
     <col min="8" max="8" width="18.21875" customWidth="1"/>
+    <col min="9" max="9" width="15.44140625" customWidth="1"/>
+    <col min="11" max="11" width="13.88671875" customWidth="1"/>
+    <col min="12" max="12" width="14.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="8" spans="6:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="H7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F8" t="s">
         <v>2</v>
       </c>
@@ -5387,8 +5444,17 @@
       <c r="H8" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="9" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="I8" t="s">
+        <v>48</v>
+      </c>
+      <c r="K8" t="s">
+        <v>49</v>
+      </c>
+      <c r="L8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F9" t="s">
         <v>41</v>
       </c>
@@ -5399,8 +5465,19 @@
         <f>TRIM(Table2[[#This Row],[Pair]])</f>
         <v>eurusd</v>
       </c>
-    </row>
-    <row r="10" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="I9" t="str">
+        <f>IF(Table2[[#This Row],[Pair]]=Table2[[#This Row],[Clean Space]],"GOOD","NADFO")</f>
+        <v>NADFO</v>
+      </c>
+      <c r="K9" t="s">
+        <v>51</v>
+      </c>
+      <c r="L9" t="str">
+        <f>PROPER(Table4[[#This Row],[raw text]])</f>
+        <v>Eur</v>
+      </c>
+    </row>
+    <row r="10" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F10" t="s">
         <v>42</v>
       </c>
@@ -5411,8 +5488,19 @@
         <f>TRIM(Table2[[#This Row],[Pair]])</f>
         <v>eurusd</v>
       </c>
-    </row>
-    <row r="11" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="I10" t="str">
+        <f>IF(Table2[[#This Row],[Pair]]=Table2[[#This Row],[Clean Space]],"GOOD","NADFO")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="K10" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="L10" t="str">
+        <f>PROPER(Table4[[#This Row],[raw text]])</f>
+        <v>Gold</v>
+      </c>
+    </row>
+    <row r="11" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F11" t="s">
         <v>43</v>
       </c>
@@ -5423,8 +5511,19 @@
         <f>TRIM(Table2[[#This Row],[Pair]])</f>
         <v>eurusd</v>
       </c>
-    </row>
-    <row r="12" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="I11" t="str">
+        <f>IF(Table2[[#This Row],[Pair]]=Table2[[#This Row],[Clean Space]],"GOOD","NADFO")</f>
+        <v>NADFO</v>
+      </c>
+      <c r="K11" t="s">
+        <v>53</v>
+      </c>
+      <c r="L11" t="str">
+        <f>PROPER(Table4[[#This Row],[raw text]])</f>
+        <v>Ud30</v>
+      </c>
+    </row>
+    <row r="12" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F12" t="s">
         <v>44</v>
       </c>
@@ -5435,8 +5534,19 @@
         <f>TRIM(Table2[[#This Row],[Pair]])</f>
         <v>gold</v>
       </c>
-    </row>
-    <row r="13" spans="6:8" x14ac:dyDescent="0.3">
+      <c r="I12" t="str">
+        <f>IF(Table2[[#This Row],[Pair]]=Table2[[#This Row],[Clean Space]],"GOOD","NADFO")</f>
+        <v>GOOD</v>
+      </c>
+      <c r="K12" t="s">
+        <v>54</v>
+      </c>
+      <c r="L12" t="str">
+        <f>PROPER(Table4[[#This Row],[raw text]])</f>
+        <v>Oil</v>
+      </c>
+    </row>
+    <row r="13" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F13" t="s">
         <v>45</v>
       </c>
@@ -5447,11 +5557,16 @@
         <f>TRIM(Table2[[#This Row],[Pair]])</f>
         <v>us30</v>
       </c>
+      <c r="I13" t="str">
+        <f>IF(Table2[[#This Row],[Pair]]=Table2[[#This Row],[Clean Space]],"GOOD","NADFO")</f>
+        <v>GOOD</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
+  <tableParts count="2">
     <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
hnata zadt function dyal value li kat7awal text l number w check ila bghit n3taf wash kayn text blast number b function isnumber()
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CACBBB4-450B-4FF3-AF1D-82EC4D263598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F74CA4E3-168B-45FB-893B-668D13504D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="2" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
     <sheet name="trading_raw_data2" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="60">
   <si>
     <t>TradeID</t>
   </si>
@@ -203,6 +203,21 @@
   </si>
   <si>
     <t>oil</t>
+  </si>
+  <si>
+    <t>convert</t>
+  </si>
+  <si>
+    <t>text num</t>
+  </si>
+  <si>
+    <t>673</t>
+  </si>
+  <si>
+    <t>634</t>
+  </si>
+  <si>
+    <t>check</t>
   </si>
 </sst>
 </file>
@@ -722,7 +737,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -739,6 +754,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -785,10 +803,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="9">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
+  <dxfs count="10">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -816,14 +831,13 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
@@ -861,14 +875,14 @@
     <tableColumn id="5" xr3:uid="{539426CC-F875-4D64-977A-05C6F1BCDBCD}" name="Direction"/>
     <tableColumn id="6" xr3:uid="{BFF7C4D2-29D9-4645-98DB-6FBF609AB80F}" name="Profit"/>
     <tableColumn id="7" xr3:uid="{CD8DBAA1-576E-4991-87E5-049F5C232A1F}" name="R"/>
-    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="8">
+    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="9">
       <calculatedColumnFormula>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="7">
+    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="8">
       <calculatedColumnFormula>IFERROR(Table1[[#This Row],[Profit]]/Table1[[#This Row],[R]],"0")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{CC96218F-2F0A-46BB-98E4-8AE8218DB3D7}" name="Result"/>
-    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -880,10 +894,10 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{DAF88BD0-F115-4C64-AE11-7DD8AB7505A7}" name="Pair"/>
     <tableColumn id="2" xr3:uid="{89E35073-D474-496E-86E0-7646DF314B64}" name="Profit"/>
-    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="2">
+    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="6">
       <calculatedColumnFormula>TRIM(Table2[[#This Row],[Pair]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="1">
+    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="5">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Pair]]=Table2[[#This Row],[Clean Space]],"GOOD","NADFO")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -896,8 +910,24 @@
   <autoFilter ref="K8:L12" xr:uid="{A99A2C5F-61E0-444B-907C-487860A13E40}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{0A321640-D79C-4135-83F6-E38913427047}" name="raw text"/>
-    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="0">
+    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="4">
       <calculatedColumnFormula>PROPER(Table4[[#This Row],[raw text]])</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{4576F3CB-3E9B-40EE-B5BA-0228DC3EBD7C}" name="Table3" displayName="Table3" ref="K16:M19" totalsRowShown="0">
+  <autoFilter ref="K16:M19" xr:uid="{4576F3CB-3E9B-40EE-B5BA-0228DC3EBD7C}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{3D4EC290-099D-468C-B78D-8A8F427D8214}" name="text num"/>
+    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="1">
+      <calculatedColumnFormula>VALUE(Table3[[#This Row],[text num]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="0">
+      <calculatedColumnFormula>ISNUMBER(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -4970,10 +5000,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5418,7 +5448,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDB00B21-86E3-4E60-9B16-646B4376A26A}">
-  <dimension ref="F7:L13"/>
+  <dimension ref="F7:M19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="6" width="13.33203125" customWidth="1"/>
@@ -5427,14 +5457,15 @@
     <col min="9" max="9" width="15.44140625" customWidth="1"/>
     <col min="11" max="11" width="13.88671875" customWidth="1"/>
     <col min="12" max="12" width="14.77734375" customWidth="1"/>
+    <col min="13" max="13" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="7" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="6:13" x14ac:dyDescent="0.3">
       <c r="H7" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="6:13" x14ac:dyDescent="0.3">
       <c r="F8" t="s">
         <v>2</v>
       </c>
@@ -5454,7 +5485,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="6:13" x14ac:dyDescent="0.3">
       <c r="F9" t="s">
         <v>41</v>
       </c>
@@ -5477,7 +5508,7 @@
         <v>Eur</v>
       </c>
     </row>
-    <row r="10" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="6:13" x14ac:dyDescent="0.3">
       <c r="F10" t="s">
         <v>42</v>
       </c>
@@ -5500,7 +5531,7 @@
         <v>Gold</v>
       </c>
     </row>
-    <row r="11" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="6:13" x14ac:dyDescent="0.3">
       <c r="F11" t="s">
         <v>43</v>
       </c>
@@ -5523,7 +5554,7 @@
         <v>Ud30</v>
       </c>
     </row>
-    <row r="12" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="6:13" x14ac:dyDescent="0.3">
       <c r="F12" t="s">
         <v>44</v>
       </c>
@@ -5546,7 +5577,7 @@
         <v>Oil</v>
       </c>
     </row>
-    <row r="13" spans="6:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="6:13" x14ac:dyDescent="0.3">
       <c r="F13" t="s">
         <v>45</v>
       </c>
@@ -5562,11 +5593,62 @@
         <v>GOOD</v>
       </c>
     </row>
+    <row r="16" spans="6:13" x14ac:dyDescent="0.3">
+      <c r="K16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L16" t="s">
+        <v>55</v>
+      </c>
+      <c r="M16" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="11:13" x14ac:dyDescent="0.3">
+      <c r="K17" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="L17">
+        <f>VALUE(Table3[[#This Row],[text num]])</f>
+        <v>673</v>
+      </c>
+      <c r="M17" t="b">
+        <f>ISNUMBER(Table3[[#This Row],[text num]])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="11:13" x14ac:dyDescent="0.3">
+      <c r="K18" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L18">
+        <f>VALUE(Table3[[#This Row],[text num]])</f>
+        <v>634</v>
+      </c>
+      <c r="M18" t="b">
+        <f>ISNUMBER(Table3[[#This Row],[text num]])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="11:13" x14ac:dyDescent="0.3">
+      <c r="K19" s="15">
+        <v>7883</v>
+      </c>
+      <c r="L19">
+        <f>VALUE(Table3[[#This Row],[text num]])</f>
+        <v>7883</v>
+      </c>
+      <c r="M19" t="b">
+        <f>ISNUMBER(Table3[[#This Row],[text num]])</f>
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="2">
+  <tableParts count="3">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
hanay zadt wahd tool dmitha duplicated value bach im7i lia chi value ila kant matkarara
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F74CA4E3-168B-45FB-893B-668D13504D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D41E543-17D6-4DCE-9B50-B37100C2594B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="2" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="60">
   <si>
     <t>TradeID</t>
   </si>
@@ -737,7 +737,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -757,6 +757,9 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -803,7 +806,16 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="13">
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -875,14 +887,14 @@
     <tableColumn id="5" xr3:uid="{539426CC-F875-4D64-977A-05C6F1BCDBCD}" name="Direction"/>
     <tableColumn id="6" xr3:uid="{BFF7C4D2-29D9-4645-98DB-6FBF609AB80F}" name="Profit"/>
     <tableColumn id="7" xr3:uid="{CD8DBAA1-576E-4991-87E5-049F5C232A1F}" name="R"/>
-    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="9">
+    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="12">
       <calculatedColumnFormula>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="8">
+    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="11">
       <calculatedColumnFormula>IFERROR(Table1[[#This Row],[Profit]]/Table1[[#This Row],[R]],"0")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{CC96218F-2F0A-46BB-98E4-8AE8218DB3D7}" name="Result"/>
-    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="7"/>
+    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -894,10 +906,10 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{DAF88BD0-F115-4C64-AE11-7DD8AB7505A7}" name="Pair"/>
     <tableColumn id="2" xr3:uid="{89E35073-D474-496E-86E0-7646DF314B64}" name="Profit"/>
-    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="6">
+    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="9">
       <calculatedColumnFormula>TRIM(Table2[[#This Row],[Pair]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="5">
+    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="8">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Pair]]=Table2[[#This Row],[Clean Space]],"GOOD","NADFO")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -910,7 +922,7 @@
   <autoFilter ref="K8:L12" xr:uid="{A99A2C5F-61E0-444B-907C-487860A13E40}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{0A321640-D79C-4135-83F6-E38913427047}" name="raw text"/>
-    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="4">
+    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="7">
       <calculatedColumnFormula>PROPER(Table4[[#This Row],[raw text]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -923,12 +935,22 @@
   <autoFilter ref="K16:M19" xr:uid="{4576F3CB-3E9B-40EE-B5BA-0228DC3EBD7C}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{3D4EC290-099D-468C-B78D-8A8F427D8214}" name="text num"/>
-    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="1">
+    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="4">
       <calculatedColumnFormula>VALUE(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="0">
+    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="3">
       <calculatedColumnFormula>ISNUMBER(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}" name="Table5" displayName="Table5" ref="Q17:Q21" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+  <autoFilter ref="Q17:Q21" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}"/>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{B868BDD4-CA52-440D-A1EA-1585934AF042}" name="TradeID" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5000,10 +5022,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5448,7 +5470,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDB00B21-86E3-4E60-9B16-646B4376A26A}">
-  <dimension ref="F7:M19"/>
+  <dimension ref="F7:Q22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="6" width="13.33203125" customWidth="1"/>
@@ -5458,6 +5480,8 @@
     <col min="11" max="11" width="13.88671875" customWidth="1"/>
     <col min="12" max="12" width="14.77734375" customWidth="1"/>
     <col min="13" max="13" width="13.6640625" customWidth="1"/>
+    <col min="17" max="17" width="13" style="17" customWidth="1"/>
+    <col min="18" max="18" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="7" spans="6:13" x14ac:dyDescent="0.3">
@@ -5604,7 +5628,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="11:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="11:17" x14ac:dyDescent="0.3">
       <c r="K17" s="14" t="s">
         <v>57</v>
       </c>
@@ -5616,8 +5640,11 @@
         <f>ISNUMBER(Table3[[#This Row],[text num]])</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="11:13" x14ac:dyDescent="0.3">
+      <c r="Q17" s="17" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="11:17" x14ac:dyDescent="0.3">
       <c r="K18" s="16" t="s">
         <v>58</v>
       </c>
@@ -5629,8 +5656,11 @@
         <f>ISNUMBER(Table3[[#This Row],[text num]])</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="11:13" x14ac:dyDescent="0.3">
+      <c r="Q18" s="17">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="19" spans="11:17" x14ac:dyDescent="0.3">
       <c r="K19" s="15">
         <v>7883</v>
       </c>
@@ -5642,13 +5672,30 @@
         <f>ISNUMBER(Table3[[#This Row],[text num]])</f>
         <v>1</v>
       </c>
+      <c r="Q19" s="17">
+        <v>1002</v>
+      </c>
+    </row>
+    <row r="20" spans="11:17" x14ac:dyDescent="0.3">
+      <c r="Q20" s="17">
+        <v>1003</v>
+      </c>
+    </row>
+    <row r="21" spans="11:17" x14ac:dyDescent="0.3">
+      <c r="Q21" s="17">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="22" spans="11:17" x14ac:dyDescent="0.3">
+      <c r="Q22"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="3">
+  <tableParts count="4">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
hanaya zadt function clookup
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C771B124-CF70-4638-8FE7-25712611EBAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D4CCC48-EB09-4885-A299-B613853228C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
     <sheet name="trading_raw_data2" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="64">
   <si>
     <t>TradeID</t>
   </si>
@@ -218,6 +218,18 @@
   </si>
   <si>
     <t>check</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>profit</t>
+  </si>
+  <si>
+    <t>r</t>
+  </si>
+  <si>
+    <t>XLOOKUP</t>
   </si>
 </sst>
 </file>
@@ -737,7 +749,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -757,6 +769,9 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1273,7 +1288,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{906658B5-1F80-4C49-9035-7A91F11B2092}">
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:P101"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.33203125" customWidth="1"/>
@@ -1283,9 +1298,12 @@
     <col min="8" max="8" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.44140625" customWidth="1"/>
     <col min="11" max="11" width="19.5546875" customWidth="1"/>
+    <col min="14" max="14" width="13.21875" customWidth="1"/>
+    <col min="15" max="15" width="15.21875" customWidth="1"/>
+    <col min="16" max="16" width="14.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1320,7 +1338,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>6</v>
       </c>
@@ -1357,7 +1375,7 @@
         <v>46164</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>80</v>
       </c>
@@ -1394,7 +1412,7 @@
         <v>46171</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>16</v>
       </c>
@@ -1431,7 +1449,7 @@
         <v>46168</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>78</v>
       </c>
@@ -1468,7 +1486,7 @@
         <v>46182</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>35</v>
       </c>
@@ -1504,8 +1522,13 @@
       <c r="K6" s="1">
         <v>46041</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="N6" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="O6" s="18"/>
+      <c r="P6" s="18"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>45</v>
       </c>
@@ -1542,7 +1565,7 @@
         <v>46055</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>43</v>
       </c>
@@ -1578,8 +1601,17 @@
       <c r="K8" s="1">
         <v>46091</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="N8" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="O8" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="P8" s="10" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>77</v>
       </c>
@@ -1615,8 +1647,19 @@
       <c r="K9" s="1">
         <v>46198</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="N9">
+        <v>13</v>
+      </c>
+      <c r="O9">
+        <f>_xlfn.XLOOKUP(N9,A:A,F:F)</f>
+        <v>750</v>
+      </c>
+      <c r="P9">
+        <f>_xlfn.XLOOKUP(N9,A:A,G:G)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>99</v>
       </c>
@@ -1653,7 +1696,7 @@
         <v>46101</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>97</v>
       </c>
@@ -1690,7 +1733,7 @@
         <v>46172</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>93</v>
       </c>
@@ -1727,7 +1770,7 @@
         <v>46053</v>
       </c>
     </row>
-    <row r="13" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10">
         <v>1</v>
       </c>
@@ -1764,7 +1807,7 @@
         <v>46190</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>38</v>
       </c>
@@ -1801,7 +1844,7 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>30</v>
       </c>
@@ -1838,7 +1881,7 @@
         <v>46167</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>46</v>
       </c>
@@ -5021,6 +5064,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="N6:P6"/>
+  </mergeCells>
   <conditionalFormatting sqref="A1">
     <cfRule type="duplicateValues" dxfId="6" priority="2"/>
   </conditionalFormatting>

</xml_diff>

<commit_message>
hnaya zadt xlookup function
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C37A3A6A-89DB-41CA-938C-50F8BD7E9783}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1C81FED-92A4-424D-B629-A78B9C2FE2E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="2" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="70">
   <si>
     <t>TradeID</t>
   </si>
@@ -230,6 +230,24 @@
   </si>
   <si>
     <t>XLOOKUP</t>
+  </si>
+  <si>
+    <t>Account Type</t>
+  </si>
+  <si>
+    <t>A001</t>
+  </si>
+  <si>
+    <t>A002</t>
+  </si>
+  <si>
+    <t>A003</t>
+  </si>
+  <si>
+    <t>Funded</t>
+  </si>
+  <si>
+    <t>Challenge</t>
   </si>
 </sst>
 </file>
@@ -5516,7 +5534,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDB00B21-86E3-4E60-9B16-646B4376A26A}">
-  <dimension ref="F7:Q25"/>
+  <dimension ref="F7:X25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="6" width="13.33203125" customWidth="1"/>
@@ -5528,14 +5546,17 @@
     <col min="13" max="13" width="13.6640625" customWidth="1"/>
     <col min="17" max="17" width="13" style="17" customWidth="1"/>
     <col min="18" max="18" width="15.6640625" customWidth="1"/>
+    <col min="19" max="19" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="7" spans="6:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="6:24" x14ac:dyDescent="0.3">
       <c r="H7" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="6:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="6:24" x14ac:dyDescent="0.3">
       <c r="F8" t="s">
         <v>2</v>
       </c>
@@ -5555,7 +5576,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="6:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="6:24" x14ac:dyDescent="0.3">
       <c r="F9" t="s">
         <v>41</v>
       </c>
@@ -5578,7 +5599,7 @@
         <v>Eur</v>
       </c>
     </row>
-    <row r="10" spans="6:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="6:24" x14ac:dyDescent="0.3">
       <c r="F10" t="s">
         <v>42</v>
       </c>
@@ -5601,7 +5622,7 @@
         <v>Gold</v>
       </c>
     </row>
-    <row r="11" spans="6:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="6:24" x14ac:dyDescent="0.3">
       <c r="F11" t="s">
         <v>43</v>
       </c>
@@ -5624,7 +5645,7 @@
         <v>Ud30</v>
       </c>
     </row>
-    <row r="12" spans="6:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="6:24" x14ac:dyDescent="0.3">
       <c r="F12" t="s">
         <v>44</v>
       </c>
@@ -5647,7 +5668,7 @@
         <v>Oil</v>
       </c>
     </row>
-    <row r="13" spans="6:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="6:24" x14ac:dyDescent="0.3">
       <c r="F13" t="s">
         <v>45</v>
       </c>
@@ -5663,7 +5684,42 @@
         <v>GOOD</v>
       </c>
     </row>
-    <row r="16" spans="6:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="6:24" x14ac:dyDescent="0.3">
+      <c r="S14" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="T14" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="V14" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="W14" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="X14" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="6:24" x14ac:dyDescent="0.3">
+      <c r="S15" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="T15" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V15" s="2">
+        <v>1001</v>
+      </c>
+      <c r="W15" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="X15" s="2" t="str">
+        <f>_xlfn.XLOOKUP(W15,S14:S17,T14:T17)</f>
+        <v>Challenge</v>
+      </c>
+    </row>
+    <row r="16" spans="6:24" x14ac:dyDescent="0.3">
       <c r="K16" t="s">
         <v>56</v>
       </c>
@@ -5673,8 +5729,24 @@
       <c r="M16" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="17" spans="11:17" x14ac:dyDescent="0.3">
+      <c r="S16" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="T16" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="V16" s="2">
+        <v>1002</v>
+      </c>
+      <c r="W16" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="X16" s="2" t="str">
+        <f t="shared" ref="X16:X17" si="0">_xlfn.XLOOKUP(W16,S15:S18,T15:T18)</f>
+        <v>Funded</v>
+      </c>
+    </row>
+    <row r="17" spans="11:24" x14ac:dyDescent="0.3">
       <c r="K17" s="14" t="s">
         <v>57</v>
       </c>
@@ -5689,8 +5761,24 @@
       <c r="Q17" s="17" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="11:17" x14ac:dyDescent="0.3">
+      <c r="S17" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="T17" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="V17" s="2">
+        <v>1003</v>
+      </c>
+      <c r="W17" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="X17" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>Funded</v>
+      </c>
+    </row>
+    <row r="18" spans="11:24" x14ac:dyDescent="0.3">
       <c r="K18" s="16" t="s">
         <v>58</v>
       </c>
@@ -5706,7 +5794,7 @@
         <v>1001</v>
       </c>
     </row>
-    <row r="19" spans="11:17" x14ac:dyDescent="0.3">
+    <row r="19" spans="11:24" x14ac:dyDescent="0.3">
       <c r="K19" s="15">
         <v>7883</v>
       </c>
@@ -5722,32 +5810,32 @@
         <v>1002</v>
       </c>
     </row>
-    <row r="20" spans="11:17" x14ac:dyDescent="0.3">
+    <row r="20" spans="11:24" x14ac:dyDescent="0.3">
       <c r="Q20" s="17">
         <v>1003</v>
       </c>
     </row>
-    <row r="21" spans="11:17" x14ac:dyDescent="0.3">
+    <row r="21" spans="11:24" x14ac:dyDescent="0.3">
       <c r="Q21" s="17">
         <v>1004</v>
       </c>
     </row>
-    <row r="22" spans="11:17" x14ac:dyDescent="0.3">
+    <row r="22" spans="11:24" x14ac:dyDescent="0.3">
       <c r="Q22" s="17">
         <v>1005</v>
       </c>
     </row>
-    <row r="23" spans="11:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="11:24" x14ac:dyDescent="0.3">
       <c r="Q23" s="17">
         <v>1006</v>
       </c>
     </row>
-    <row r="24" spans="11:17" x14ac:dyDescent="0.3">
+    <row r="24" spans="11:24" x14ac:dyDescent="0.3">
       <c r="Q24" s="17">
         <v>1007</v>
       </c>
     </row>
-    <row r="25" spans="11:17" x14ac:dyDescent="0.3">
+    <row r="25" spans="11:24" x14ac:dyDescent="0.3">
       <c r="Q25" s="17">
         <v>1008</v>
       </c>

</xml_diff>

<commit_message>
hnaya 3awadt xlookup b update akhor
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1C81FED-92A4-424D-B629-A78B9C2FE2E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DBEE66B-FFE9-43D0-B9A6-39835B957ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="2" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
+    <workbookView xWindow="11436" yWindow="0" windowWidth="11700" windowHeight="12336" firstSheet="1" activeTab="2" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
     <sheet name="trading_raw_data2" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="71">
   <si>
     <t>TradeID</t>
   </si>
@@ -248,6 +248,9 @@
   </si>
   <si>
     <t>Challenge</t>
+  </si>
+  <si>
+    <t>A004</t>
   </si>
 </sst>
 </file>
@@ -767,7 +770,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -793,6 +796,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -5709,13 +5713,13 @@
         <v>68</v>
       </c>
       <c r="V15" s="2">
-        <v>1001</v>
+        <v>2001</v>
       </c>
       <c r="W15" s="2" t="s">
         <v>66</v>
       </c>
       <c r="X15" s="2" t="str">
-        <f>_xlfn.XLOOKUP(W15,S14:S17,T14:T17)</f>
+        <f>_xlfn.XLOOKUP(W15,S14:S18,T14:T18)</f>
         <v>Challenge</v>
       </c>
     </row>
@@ -5736,13 +5740,13 @@
         <v>69</v>
       </c>
       <c r="V16" s="2">
-        <v>1002</v>
+        <v>2002</v>
       </c>
       <c r="W16" s="2" t="s">
         <v>65</v>
       </c>
       <c r="X16" s="2" t="str">
-        <f t="shared" ref="X16:X17" si="0">_xlfn.XLOOKUP(W16,S15:S18,T15:T18)</f>
+        <f t="shared" ref="X16:X18" si="0">_xlfn.XLOOKUP(W16,S15:S19,T15:T19)</f>
         <v>Funded</v>
       </c>
     </row>
@@ -5768,7 +5772,7 @@
         <v>68</v>
       </c>
       <c r="V17" s="2">
-        <v>1003</v>
+        <v>2003</v>
       </c>
       <c r="W17" s="2" t="s">
         <v>67</v>
@@ -5792,6 +5796,22 @@
       </c>
       <c r="Q18" s="17">
         <v>1001</v>
+      </c>
+      <c r="S18" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="T18" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="V18" s="19">
+        <v>2004</v>
+      </c>
+      <c r="W18" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="X18" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>Challenge</v>
       </c>
     </row>
     <row r="19" spans="11:24" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
xlookup dartha dyal two table bach njib wahed calue mn table l table
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DBEE66B-FFE9-43D0-B9A6-39835B957ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC910028-BA33-4C34-AE19-115EBD6EDF48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11436" yWindow="0" windowWidth="11700" windowHeight="12336" firstSheet="1" activeTab="2" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
+    <workbookView xWindow="11496" yWindow="0" windowWidth="11640" windowHeight="12336" firstSheet="1" activeTab="2" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
     <sheet name="trading_raw_data2" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
hanya zadt iferror l xlookup
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC910028-BA33-4C34-AE19-115EBD6EDF48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44D32093-DE84-4A4C-80BE-A8237440433A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11496" yWindow="0" windowWidth="11640" windowHeight="12336" firstSheet="1" activeTab="2" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="2" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
     <sheet name="trading_raw_data2" sheetId="1" r:id="rId1"/>
@@ -37,8 +37,45 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="2">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <futureMetadata name="XLRICHVALUE" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+  <valueMetadata count="1">
+    <bk>
+      <rc t="2" v="0"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="71">
   <si>
     <t>TradeID</t>
   </si>
@@ -793,10 +830,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -908,6 +945,68 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <rv s="0">
+    <v>0</v>
+    <v>8</v>
+    <v>3</v>
+    <v>1</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_error">
+    <k n="colOffset" t="i"/>
+    <k n="errorType" t="i"/>
+    <k n="rwOffset" t="i"/>
+    <k n="subType" t="i"/>
+  </s>
+</rvStructures>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1544,11 +1643,11 @@
       <c r="K6" s="1">
         <v>46041</v>
       </c>
-      <c r="N6" s="18" t="s">
+      <c r="N6" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="O6" s="18"/>
-      <c r="P6" s="18"/>
+      <c r="O6" s="19"/>
+      <c r="P6" s="19"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7">
@@ -5709,18 +5808,16 @@
       <c r="S15" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="T15" s="2" t="s">
-        <v>68</v>
-      </c>
+      <c r="T15" s="2"/>
       <c r="V15" s="2">
         <v>2001</v>
       </c>
       <c r="W15" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="X15" s="2" t="str">
-        <f>_xlfn.XLOOKUP(W15,S14:S18,T14:T18)</f>
-        <v>Challenge</v>
+      <c r="X15" s="2" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="X15" ca="1">IFERROR(_xlfn.XLOOKUP(W15:W18,S15:S18,T15:T18),"not found")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="16" spans="6:24" x14ac:dyDescent="0.3">
@@ -5745,9 +5842,9 @@
       <c r="W16" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="X16" s="2" t="str">
-        <f t="shared" ref="X16:X18" si="0">_xlfn.XLOOKUP(W16,S15:S19,T15:T19)</f>
-        <v>Funded</v>
+      <c r="X16" s="2" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="X16" ca="1">IFERROR(_xlfn.XLOOKUP(W16:W19,S16:S19,T16:T19),"not found")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="17" spans="11:24" x14ac:dyDescent="0.3">
@@ -5777,9 +5874,9 @@
       <c r="W17" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="X17" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Funded</v>
+      <c r="X17" s="2" t="e" cm="1" vm="1">
+        <f t="array" aca="1" ref="X17" ca="1">IFERROR(_xlfn.XLOOKUP(W17:W20,S17:S20,T17:T20),"not found")</f>
+        <v>#VALUE!</v>
       </c>
     </row>
     <row r="18" spans="11:24" x14ac:dyDescent="0.3">
@@ -5797,20 +5894,20 @@
       <c r="Q18" s="17">
         <v>1001</v>
       </c>
-      <c r="S18" s="19" t="s">
+      <c r="S18" s="18" t="s">
         <v>70</v>
       </c>
       <c r="T18" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="V18" s="19">
+      <c r="V18" s="18">
         <v>2004</v>
       </c>
       <c r="W18" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="X18" s="2" t="str">
-        <f t="shared" si="0"/>
+      <c r="X18" s="2" t="str" cm="1">
+        <f t="array" ref="X18:X21">IFERROR(_xlfn.XLOOKUP(W18:W21,S18:S21,T18:T21),"not found")</f>
         <v>Challenge</v>
       </c>
     </row>
@@ -5829,15 +5926,24 @@
       <c r="Q19" s="17">
         <v>1002</v>
       </c>
+      <c r="X19">
+        <v>0</v>
+      </c>
     </row>
     <row r="20" spans="11:24" x14ac:dyDescent="0.3">
       <c r="Q20" s="17">
         <v>1003</v>
       </c>
+      <c r="X20">
+        <v>0</v>
+      </c>
     </row>
     <row r="21" spans="11:24" x14ac:dyDescent="0.3">
       <c r="Q21" s="17">
         <v>1004</v>
+      </c>
+      <c r="X21">
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="11:24" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
hnaya bdit nafham bali pivot table balo bhal group by f sql w pandas
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BB503C0-4604-46A2-BE68-E7F7D093F595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{429EC6E7-AD57-4DAC-8EF6-BB051230C2C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="4" r:id="rId1"/>
+    <sheet name="pivot table" sheetId="4" r:id="rId1"/>
     <sheet name="trading_raw_data2" sheetId="1" r:id="rId2"/>
     <sheet name="data analysis" sheetId="2" r:id="rId3"/>
     <sheet name="data cleaning " sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="3" r:id="rId5"/>
+    <pivotCache cacheId="5" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="75">
   <si>
     <t>TradeID</t>
   </si>
@@ -301,6 +301,9 @@
   </si>
   <si>
     <t>Sum of Profit</t>
+  </si>
+  <si>
+    <t>Column Labels</t>
   </si>
 </sst>
 </file>
@@ -986,7 +989,10 @@
       </sharedItems>
     </cacheField>
     <cacheField name="Session" numFmtId="0">
-      <sharedItems/>
+      <sharedItems count="2">
+        <s v="New York"/>
+        <s v="London"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Direction" numFmtId="0">
       <sharedItems/>
@@ -1004,7 +1010,10 @@
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="50" maxValue="250"/>
     </cacheField>
     <cacheField name="Result" numFmtId="0">
-      <sharedItems/>
+      <sharedItems count="2">
+        <s v="Win"/>
+        <s v="Loss"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="TradeDate" numFmtId="14">
       <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2026-01-05T00:00:00" maxDate="2026-07-05T00:00:00"/>
@@ -1024,1312 +1033,1312 @@
     <n v="6"/>
     <n v="10005"/>
     <x v="0"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Buy"/>
     <n v="600"/>
     <n v="3"/>
     <s v="GOOD"/>
     <n v="200"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-05-22T00:00:00"/>
   </r>
   <r>
     <n v="80"/>
     <n v="10006"/>
     <x v="0"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="600"/>
     <n v="3"/>
     <s v="GOOD"/>
     <n v="200"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-05-29T00:00:00"/>
   </r>
   <r>
     <n v="16"/>
     <n v="10006"/>
     <x v="0"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="500"/>
     <n v="2"/>
     <s v="GOOD"/>
     <n v="250"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-05-26T00:00:00"/>
   </r>
   <r>
     <n v="78"/>
     <n v="10001"/>
     <x v="0"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="500"/>
     <n v="2"/>
     <s v="GOOD"/>
     <n v="250"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-06-09T00:00:00"/>
   </r>
   <r>
     <n v="35"/>
     <n v="10005"/>
     <x v="0"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="375"/>
     <n v="1.5"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-01-19T00:00:00"/>
   </r>
   <r>
     <n v="45"/>
     <n v="10003"/>
     <x v="0"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="375"/>
     <n v="1.5"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-02-02T00:00:00"/>
   </r>
   <r>
     <n v="43"/>
     <n v="10003"/>
     <x v="0"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="200"/>
     <n v="2"/>
     <s v="GOOD"/>
     <n v="100"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-03-10T00:00:00"/>
   </r>
   <r>
     <n v="77"/>
     <n v="10006"/>
     <x v="0"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="200"/>
     <n v="2"/>
     <s v="GOOD"/>
     <n v="100"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-06-25T00:00:00"/>
   </r>
   <r>
     <n v="99"/>
     <n v="10006"/>
     <x v="0"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="125"/>
     <n v="2.5"/>
     <s v="GOOD"/>
     <n v="50"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-03-20T00:00:00"/>
   </r>
   <r>
     <n v="97"/>
     <n v="10006"/>
     <x v="0"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="100"/>
     <n v="1"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-05-30T00:00:00"/>
   </r>
   <r>
     <n v="93"/>
     <n v="10004"/>
     <x v="0"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="75"/>
     <n v="1.5"/>
     <s v="REVIEW"/>
     <n v="50"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-01-31T00:00:00"/>
   </r>
   <r>
     <n v="1"/>
     <n v="10002"/>
     <x v="0"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="50"/>
     <n v="1"/>
     <s v="REVIEW"/>
     <n v="50"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-06-17T00:00:00"/>
   </r>
   <r>
     <n v="38"/>
     <n v="10005"/>
     <x v="0"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="-25"/>
     <n v="-0.5"/>
     <s v="REVIEW"/>
     <n v="50"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-03-26T00:00:00"/>
   </r>
   <r>
     <n v="30"/>
     <n v="10001"/>
     <x v="0"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="-50"/>
     <n v="-0.5"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-05-25T00:00:00"/>
   </r>
   <r>
     <n v="46"/>
     <n v="10001"/>
     <x v="0"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="-50"/>
     <n v="-0.5"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-02-06T00:00:00"/>
   </r>
   <r>
     <n v="47"/>
     <n v="10005"/>
     <x v="0"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="-50"/>
     <n v="-0.5"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-06-24T00:00:00"/>
   </r>
   <r>
     <n v="52"/>
     <n v="10005"/>
     <x v="0"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Buy"/>
     <n v="-50"/>
     <n v="-1"/>
     <s v="REVIEW"/>
     <n v="50"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-01-12T00:00:00"/>
   </r>
   <r>
     <n v="8"/>
     <n v="10004"/>
     <x v="0"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="-100"/>
     <n v="-1"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-03-05T00:00:00"/>
   </r>
   <r>
     <n v="70"/>
     <n v="10004"/>
     <x v="0"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="-100"/>
     <n v="-1"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-05-07T00:00:00"/>
   </r>
   <r>
     <n v="86"/>
     <n v="10002"/>
     <x v="0"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="-100"/>
     <n v="-1"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-05-27T00:00:00"/>
   </r>
   <r>
     <n v="61"/>
     <n v="10005"/>
     <x v="0"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="-125"/>
     <n v="-0.5"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-01-11T00:00:00"/>
   </r>
   <r>
     <n v="34"/>
     <n v="10005"/>
     <x v="0"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="-150"/>
     <n v="-1.5"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-03-26T00:00:00"/>
   </r>
   <r>
     <n v="13"/>
     <n v="10006"/>
     <x v="1"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="750"/>
     <n v="3"/>
     <s v="GOOD"/>
     <n v="250"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-03-13T00:00:00"/>
   </r>
   <r>
     <n v="98"/>
     <n v="10001"/>
     <x v="1"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="750"/>
     <n v="3"/>
     <s v="GOOD"/>
     <n v="250"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-03-07T00:00:00"/>
   </r>
   <r>
     <n v="68"/>
     <n v="10004"/>
     <x v="1"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="625"/>
     <n v="2.5"/>
     <s v="GOOD"/>
     <n v="250"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-07-04T00:00:00"/>
   </r>
   <r>
     <n v="85"/>
     <n v="10003"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="600"/>
     <n v="3"/>
     <s v="GOOD"/>
     <n v="200"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-05-09T00:00:00"/>
   </r>
   <r>
     <n v="15"/>
     <n v="10004"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Buy"/>
     <n v="500"/>
     <n v="2.5"/>
     <s v="GOOD"/>
     <n v="200"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-06-14T00:00:00"/>
   </r>
   <r>
     <n v="37"/>
     <n v="10003"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Buy"/>
     <n v="500"/>
     <n v="2"/>
     <s v="GOOD"/>
     <n v="250"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-03-12T00:00:00"/>
   </r>
   <r>
     <n v="71"/>
     <n v="10004"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="500"/>
     <n v="2"/>
     <s v="GOOD"/>
     <n v="250"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-05-09T00:00:00"/>
   </r>
   <r>
     <n v="88"/>
     <n v="10004"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="500"/>
     <n v="2"/>
     <s v="GOOD"/>
     <n v="250"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-07-01T00:00:00"/>
   </r>
   <r>
     <n v="76"/>
     <n v="10005"/>
     <x v="1"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="375"/>
     <n v="1.5"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-01-12T00:00:00"/>
   </r>
   <r>
     <n v="92"/>
     <n v="10001"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Buy"/>
     <n v="375"/>
     <n v="1.5"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-01-08T00:00:00"/>
   </r>
   <r>
     <n v="10"/>
     <n v="10004"/>
     <x v="1"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="300"/>
     <n v="3"/>
     <s v="GOOD"/>
     <n v="100"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-06-09T00:00:00"/>
   </r>
   <r>
     <n v="23"/>
     <n v="10003"/>
     <x v="1"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="300"/>
     <n v="3"/>
     <s v="GOOD"/>
     <n v="100"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-02-04T00:00:00"/>
   </r>
   <r>
     <n v="54"/>
     <n v="10006"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Buy"/>
     <n v="300"/>
     <n v="3"/>
     <s v="GOOD"/>
     <n v="100"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-04-13T00:00:00"/>
   </r>
   <r>
     <n v="12"/>
     <n v="10006"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Buy"/>
     <n v="250"/>
     <n v="2.5"/>
     <s v="GOOD"/>
     <n v="100"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-01-21T00:00:00"/>
   </r>
   <r>
     <n v="63"/>
     <n v="10001"/>
     <x v="1"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="250"/>
     <n v="1"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-04-23T00:00:00"/>
   </r>
   <r>
     <n v="95"/>
     <n v="10002"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Buy"/>
     <n v="250"/>
     <n v="2.5"/>
     <s v="GOOD"/>
     <n v="100"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-02-12T00:00:00"/>
   </r>
   <r>
     <n v="84"/>
     <n v="10003"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="200"/>
     <n v="2"/>
     <s v="GOOD"/>
     <n v="100"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-04-30T00:00:00"/>
   </r>
   <r>
     <n v="33"/>
     <n v="10001"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Buy"/>
     <n v="150"/>
     <n v="3"/>
     <s v="GOOD"/>
     <n v="50"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-02-13T00:00:00"/>
   </r>
   <r>
     <n v="100"/>
     <n v="10004"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Buy"/>
     <n v="150"/>
     <n v="1.5"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-06-29T00:00:00"/>
   </r>
   <r>
     <n v="3"/>
     <n v="10004"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Buy"/>
     <n v="100"/>
     <n v="1"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-05-28T00:00:00"/>
   </r>
   <r>
     <n v="7"/>
     <n v="10006"/>
     <x v="1"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="100"/>
     <n v="2"/>
     <s v="GOOD"/>
     <n v="50"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-06-01T00:00:00"/>
   </r>
   <r>
     <n v="20"/>
     <n v="10006"/>
     <x v="1"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="100"/>
     <n v="1"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-01-19T00:00:00"/>
   </r>
   <r>
     <n v="62"/>
     <n v="10004"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="50"/>
     <n v="1"/>
     <s v="REVIEW"/>
     <n v="50"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-04-21T00:00:00"/>
   </r>
   <r>
     <n v="24"/>
     <n v="10006"/>
     <x v="1"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="-25"/>
     <n v="-0.5"/>
     <s v="REVIEW"/>
     <n v="50"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-06-04T00:00:00"/>
   </r>
   <r>
     <n v="14"/>
     <n v="10001"/>
     <x v="1"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="-50"/>
     <n v="-0.5"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-04-07T00:00:00"/>
   </r>
   <r>
     <n v="49"/>
     <n v="10001"/>
     <x v="1"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="-50"/>
     <n v="-0.5"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-03-14T00:00:00"/>
   </r>
   <r>
     <n v="79"/>
     <n v="10001"/>
     <x v="1"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="-50"/>
     <n v="-1"/>
     <s v="REVIEW"/>
     <n v="50"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-04-16T00:00:00"/>
   </r>
   <r>
     <n v="40"/>
     <n v="10005"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="-75"/>
     <n v="-1.5"/>
     <s v="REVIEW"/>
     <n v="50"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-03-18T00:00:00"/>
   </r>
   <r>
     <n v="39"/>
     <n v="10003"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Buy"/>
     <n v="-100"/>
     <n v="-0.5"/>
     <s v="REVIEW"/>
     <n v="200"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-05-22T00:00:00"/>
   </r>
   <r>
     <n v="29"/>
     <n v="10002"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="-125"/>
     <n v="-0.5"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-04-23T00:00:00"/>
   </r>
   <r>
     <n v="69"/>
     <n v="10005"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="-125"/>
     <n v="-0.5"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-01-20T00:00:00"/>
   </r>
   <r>
     <n v="22"/>
     <n v="10006"/>
     <x v="1"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="-250"/>
     <n v="-1"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-05-23T00:00:00"/>
   </r>
   <r>
     <n v="36"/>
     <n v="10004"/>
     <x v="1"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="-300"/>
     <n v="-1.5"/>
     <s v="REVIEW"/>
     <n v="200"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-02-04T00:00:00"/>
   </r>
   <r>
     <n v="32"/>
     <n v="10003"/>
     <x v="2"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="750"/>
     <n v="3"/>
     <s v="GOOD"/>
     <n v="250"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-01-05T00:00:00"/>
   </r>
   <r>
     <n v="73"/>
     <n v="10002"/>
     <x v="2"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="500"/>
     <n v="2.5"/>
     <s v="GOOD"/>
     <n v="200"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-06-18T00:00:00"/>
   </r>
   <r>
     <n v="74"/>
     <n v="10004"/>
     <x v="2"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="500"/>
     <n v="2.5"/>
     <s v="GOOD"/>
     <n v="200"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-02-28T00:00:00"/>
   </r>
   <r>
     <n v="87"/>
     <n v="10001"/>
     <x v="2"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="375"/>
     <n v="1.5"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-06-30T00:00:00"/>
   </r>
   <r>
     <n v="65"/>
     <n v="10004"/>
     <x v="2"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="300"/>
     <n v="1.5"/>
     <s v="REVIEW"/>
     <n v="200"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-05-25T00:00:00"/>
   </r>
   <r>
     <n v="26"/>
     <n v="10004"/>
     <x v="2"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="250"/>
     <n v="1"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-05-31T00:00:00"/>
   </r>
   <r>
     <n v="55"/>
     <n v="10005"/>
     <x v="2"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="200"/>
     <n v="1"/>
     <s v="REVIEW"/>
     <n v="200"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-04-08T00:00:00"/>
   </r>
   <r>
     <n v="59"/>
     <n v="10006"/>
     <x v="2"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="200"/>
     <n v="1"/>
     <s v="REVIEW"/>
     <n v="200"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-04-28T00:00:00"/>
   </r>
   <r>
     <n v="66"/>
     <n v="10004"/>
     <x v="2"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="200"/>
     <n v="2"/>
     <s v="GOOD"/>
     <n v="100"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-05-18T00:00:00"/>
   </r>
   <r>
     <n v="2"/>
     <n v="10001"/>
     <x v="2"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="150"/>
     <n v="3"/>
     <s v="GOOD"/>
     <n v="50"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-06-05T00:00:00"/>
   </r>
   <r>
     <n v="94"/>
     <n v="10004"/>
     <x v="2"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="150"/>
     <n v="3"/>
     <s v="GOOD"/>
     <n v="50"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-03-10T00:00:00"/>
   </r>
   <r>
     <n v="57"/>
     <n v="10005"/>
     <x v="2"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Buy"/>
     <n v="125"/>
     <n v="2.5"/>
     <s v="GOOD"/>
     <n v="50"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-02-23T00:00:00"/>
   </r>
   <r>
     <n v="4"/>
     <n v="10002"/>
     <x v="2"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="100"/>
     <n v="2"/>
     <s v="GOOD"/>
     <n v="50"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-07-02T00:00:00"/>
   </r>
   <r>
     <n v="27"/>
     <n v="10006"/>
     <x v="2"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="50"/>
     <n v="1"/>
     <s v="REVIEW"/>
     <n v="50"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-04-05T00:00:00"/>
   </r>
   <r>
     <n v="72"/>
     <n v="10004"/>
     <x v="2"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="50"/>
     <n v="1"/>
     <s v="REVIEW"/>
     <n v="50"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-02-16T00:00:00"/>
   </r>
   <r>
     <n v="75"/>
     <n v="10003"/>
     <x v="2"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="50"/>
     <n v="1"/>
     <s v="REVIEW"/>
     <n v="50"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-01-25T00:00:00"/>
   </r>
   <r>
     <n v="17"/>
     <n v="10005"/>
     <x v="2"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="-75"/>
     <n v="-1.5"/>
     <s v="REVIEW"/>
     <n v="50"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-02-14T00:00:00"/>
   </r>
   <r>
     <n v="53"/>
     <n v="10004"/>
     <x v="2"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="-75"/>
     <n v="-1.5"/>
     <s v="REVIEW"/>
     <n v="50"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-02-01T00:00:00"/>
   </r>
   <r>
     <n v="21"/>
     <n v="10005"/>
     <x v="2"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="-100"/>
     <n v="-1"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-02-06T00:00:00"/>
   </r>
   <r>
     <n v="48"/>
     <n v="10006"/>
     <x v="2"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="-100"/>
     <n v="-1"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-02-19T00:00:00"/>
   </r>
   <r>
     <n v="83"/>
     <n v="10002"/>
     <x v="2"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="-100"/>
     <n v="-0.5"/>
     <s v="REVIEW"/>
     <n v="200"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-05-04T00:00:00"/>
   </r>
   <r>
     <n v="5"/>
     <n v="10003"/>
     <x v="2"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="-125"/>
     <n v="-0.5"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-01-28T00:00:00"/>
   </r>
   <r>
     <n v="31"/>
     <n v="10004"/>
     <x v="2"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Buy"/>
     <n v="-125"/>
     <n v="-0.5"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-04-19T00:00:00"/>
   </r>
   <r>
     <n v="96"/>
     <n v="10003"/>
     <x v="2"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="-200"/>
     <n v="-1"/>
     <s v="REVIEW"/>
     <n v="200"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-05-18T00:00:00"/>
   </r>
   <r>
     <n v="64"/>
     <n v="10005"/>
     <x v="2"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="-375"/>
     <n v="-1.5"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-02-08T00:00:00"/>
   </r>
   <r>
     <n v="81"/>
     <n v="10004"/>
     <x v="2"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Buy"/>
     <n v="-375"/>
     <n v="-1.5"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-01-08T00:00:00"/>
   </r>
   <r>
     <n v="82"/>
     <n v="10005"/>
     <x v="2"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="-375"/>
     <n v="-1.5"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-02-13T00:00:00"/>
   </r>
   <r>
     <n v="90"/>
     <n v="10002"/>
     <x v="3"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="500"/>
     <n v="2.5"/>
     <s v="GOOD"/>
     <n v="200"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-02-23T00:00:00"/>
   </r>
   <r>
     <n v="50"/>
     <n v="10002"/>
     <x v="3"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Buy"/>
     <n v="375"/>
     <n v="1.5"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-05-02T00:00:00"/>
   </r>
   <r>
     <n v="91"/>
     <n v="10003"/>
     <x v="3"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="300"/>
     <n v="1.5"/>
     <s v="REVIEW"/>
     <n v="200"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-06-04T00:00:00"/>
   </r>
   <r>
     <n v="28"/>
     <n v="10002"/>
     <x v="3"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="250"/>
     <n v="2.5"/>
     <s v="GOOD"/>
     <n v="100"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-04-18T00:00:00"/>
   </r>
   <r>
     <n v="67"/>
     <n v="10002"/>
     <x v="3"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Buy"/>
     <n v="250"/>
     <n v="2.5"/>
     <s v="GOOD"/>
     <n v="100"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-03-15T00:00:00"/>
   </r>
   <r>
     <n v="60"/>
     <n v="10006"/>
     <x v="3"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="150"/>
     <n v="1.5"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-05-16T00:00:00"/>
   </r>
   <r>
     <n v="41"/>
     <n v="10003"/>
     <x v="3"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="100"/>
     <n v="1"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-06-24T00:00:00"/>
   </r>
   <r>
     <n v="89"/>
     <n v="10003"/>
     <x v="3"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="75"/>
     <n v="1.5"/>
     <s v="REVIEW"/>
     <n v="50"/>
-    <s v="Win"/>
+    <x v="0"/>
     <d v="2026-05-25T00:00:00"/>
   </r>
   <r>
     <n v="25"/>
     <n v="10003"/>
     <x v="3"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="-50"/>
     <n v="-0.5"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-01-13T00:00:00"/>
   </r>
   <r>
     <n v="9"/>
     <n v="10006"/>
     <x v="3"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="-75"/>
     <n v="-1.5"/>
     <s v="REVIEW"/>
     <n v="50"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-04-09T00:00:00"/>
   </r>
   <r>
     <n v="18"/>
     <n v="10003"/>
     <x v="3"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="-75"/>
     <n v="-1.5"/>
     <s v="REVIEW"/>
     <n v="50"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-06-14T00:00:00"/>
   </r>
   <r>
     <n v="44"/>
     <n v="10005"/>
     <x v="3"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="-75"/>
     <n v="-1.5"/>
     <s v="REVIEW"/>
     <n v="50"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-06-17T00:00:00"/>
   </r>
   <r>
     <n v="19"/>
     <n v="10001"/>
     <x v="3"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Buy"/>
     <n v="-100"/>
     <n v="-1"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-06-07T00:00:00"/>
   </r>
   <r>
     <n v="56"/>
     <n v="10004"/>
     <x v="3"/>
-    <s v="New York"/>
+    <x v="0"/>
     <s v="Sell"/>
     <n v="-150"/>
     <n v="-1.5"/>
     <s v="REVIEW"/>
     <n v="100"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-05-14T00:00:00"/>
   </r>
   <r>
     <n v="11"/>
     <n v="10001"/>
     <x v="3"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Buy"/>
     <n v="-200"/>
     <n v="-1"/>
     <s v="REVIEW"/>
     <n v="200"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-06-29T00:00:00"/>
   </r>
   <r>
     <n v="51"/>
     <n v="10003"/>
     <x v="3"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="-200"/>
     <n v="-1"/>
     <s v="REVIEW"/>
     <n v="200"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-03-30T00:00:00"/>
   </r>
   <r>
     <n v="42"/>
     <n v="10002"/>
     <x v="3"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="-250"/>
     <n v="-1"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-03-15T00:00:00"/>
   </r>
   <r>
     <n v="58"/>
     <n v="10005"/>
     <x v="3"/>
-    <s v="London"/>
+    <x v="1"/>
     <s v="Sell"/>
     <n v="-250"/>
     <n v="-1"/>
     <s v="REVIEW"/>
     <n v="250"/>
-    <s v="Loss"/>
+    <x v="1"/>
     <d v="2026-03-23T00:00:00"/>
   </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2DA79A61-38FD-45EA-A18C-EAC9CD91845A}" name="PivotTable1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2DA79A61-38FD-45EA-A18C-EAC9CD91845A}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:D7" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
+    <pivotField showAll="0">
       <items count="5">
         <item x="0"/>
         <item x="1"/>
@@ -2338,37 +2347,54 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="3">
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField numFmtId="14" showAll="0"/>
   </pivotFields>
   <rowFields count="1">
-    <field x="2"/>
+    <field x="3"/>
   </rowFields>
-  <rowItems count="5">
+  <rowItems count="3">
     <i>
       <x/>
     </i>
     <i>
       <x v="1"/>
     </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="9"/>
+  </colFields>
+  <colItems count="3">
     <i>
-      <x v="2"/>
+      <x/>
     </i>
     <i>
-      <x v="3"/>
+      <x v="1"/>
     </i>
     <i t="grand">
       <x/>
     </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
   </colItems>
   <dataFields count="1">
     <dataField name="Sum of Profit" fld="5" baseField="0" baseItem="0"/>
@@ -2847,58 +2873,76 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A00360D7-0D73-4CE4-AFB9-0AF5F61FAEDB}">
-  <dimension ref="A3:B8"/>
+  <dimension ref="A3:D7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="B3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="21" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="22">
-        <v>2900</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="21" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B5" s="22">
-        <v>6825</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+        <v>-2875</v>
+      </c>
+      <c r="C5" s="22">
+        <v>9325</v>
+      </c>
+      <c r="D5" s="22">
+        <v>6450</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="21" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B6" s="22">
-        <v>1925</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+        <v>-2525</v>
+      </c>
+      <c r="C6" s="22">
+        <v>8300</v>
+      </c>
+      <c r="D6" s="22">
+        <v>5775</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="21" t="s">
-        <v>18</v>
+        <v>72</v>
       </c>
       <c r="B7" s="22">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="B8" s="22">
+        <v>-5400</v>
+      </c>
+      <c r="C7" s="22">
+        <v>17625</v>
+      </c>
+      <c r="D7" s="22">
         <v>12225</v>
       </c>
     </row>

</xml_diff>

<commit_message>
hanaya dart groyb by l pairs w hsabt total profit
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{429EC6E7-AD57-4DAC-8EF6-BB051230C2C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24229C6E-87CF-4A43-A2FB-AED24890553A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="5" r:id="rId5"/>
+    <pivotCache cacheId="4" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -847,14 +847,14 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2333,7 +2333,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2DA79A61-38FD-45EA-A18C-EAC9CD91845A}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2DA79A61-38FD-45EA-A18C-EAC9CD91845A}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:D7" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
@@ -2880,18 +2880,21 @@
     <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="19" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="19" t="s">
         <v>71</v>
       </c>
       <c r="B4" t="s">
@@ -2905,44 +2908,44 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="22">
+      <c r="B5" s="21">
         <v>-2875</v>
       </c>
-      <c r="C5" s="22">
+      <c r="C5" s="21">
         <v>9325</v>
       </c>
-      <c r="D5" s="22">
+      <c r="D5" s="21">
         <v>6450</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="22">
+      <c r="B6" s="21">
         <v>-2525</v>
       </c>
-      <c r="C6" s="22">
+      <c r="C6" s="21">
         <v>8300</v>
       </c>
-      <c r="D6" s="22">
+      <c r="D6" s="21">
         <v>5775</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="22">
+      <c r="B7" s="21">
         <v>-5400</v>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="21">
         <v>17625</v>
       </c>
-      <c r="D7" s="22">
+      <c r="D7" s="21">
         <v>12225</v>
       </c>
     </row>
@@ -3188,11 +3191,11 @@
       <c r="K6" s="1">
         <v>46041</v>
       </c>
-      <c r="N6" s="19" t="s">
+      <c r="N6" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="O6" s="19"/>
-      <c r="P6" s="19"/>
+      <c r="O6" s="22"/>
+      <c r="P6" s="22"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7">

</xml_diff>

<commit_message>
hnaya dart count l trade hasab group dyal kola pair
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24229C6E-87CF-4A43-A2FB-AED24890553A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF1402EA-519A-4C45-854E-5B08AAF2B112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="4" r:id="rId5"/>
+    <pivotCache cacheId="20" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="74">
   <si>
     <t>TradeID</t>
   </si>
@@ -300,10 +300,7 @@
     <t>Grand Total</t>
   </si>
   <si>
-    <t>Sum of Profit</t>
-  </si>
-  <si>
-    <t>Column Labels</t>
+    <t>Count of TradeID</t>
   </si>
 </sst>
 </file>
@@ -969,7 +966,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="THINKPAD" refreshedDate="46283.837479513888" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="100" xr:uid="{B5704D22-3EE7-4BB0-8E8C-6CA18976C1C7}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="THINKPAD" refreshedDate="46284.786864351852" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="100" xr:uid="{B5704D22-3EE7-4BB0-8E8C-6CA18976C1C7}">
   <cacheSource type="worksheet">
     <worksheetSource name="Table1"/>
   </cacheSource>
@@ -2333,12 +2330,12 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2DA79A61-38FD-45EA-A18C-EAC9CD91845A}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:D7" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2DA79A61-38FD-45EA-A18C-EAC9CD91845A}" name="PivotTable1" cacheId="20" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
+    <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
+    <pivotField axis="axisRow" showAll="0">
       <items count="5">
         <item x="0"/>
         <item x="1"/>
@@ -2347,7 +2344,7 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField axis="axisRow" showAll="0">
+    <pivotField showAll="0">
       <items count="3">
         <item x="1"/>
         <item x="0"/>
@@ -2355,11 +2352,11 @@
       </items>
     </pivotField>
     <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField axis="axisCol" showAll="0">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
       <items count="3">
         <item x="1"/>
         <item x="0"/>
@@ -2369,35 +2366,30 @@
     <pivotField numFmtId="14" showAll="0"/>
   </pivotFields>
   <rowFields count="1">
-    <field x="3"/>
+    <field x="2"/>
   </rowFields>
-  <rowItems count="3">
+  <rowItems count="5">
     <i>
       <x/>
     </i>
     <i>
       <x v="1"/>
     </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
     <i t="grand">
       <x/>
     </i>
   </rowItems>
-  <colFields count="1">
-    <field x="9"/>
-  </colFields>
-  <colItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
+  <colItems count="1">
+    <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Sum of Profit" fld="5" baseField="0" baseItem="0"/>
+    <dataField name="Count of TradeID" fld="0" subtotal="count" baseField="3" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -2873,80 +2865,64 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A00360D7-0D73-4CE4-AFB9-0AF5F61FAEDB}">
-  <dimension ref="A3:D7"/>
+  <dimension ref="A3:B8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.21875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="19" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="19" t="s">
-        <v>71</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="21">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="21">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="21">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="21">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="20" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="21">
-        <v>-2875</v>
-      </c>
-      <c r="C5" s="21">
-        <v>9325</v>
-      </c>
-      <c r="D5" s="21">
-        <v>6450</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="20" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" s="21">
-        <v>-2525</v>
-      </c>
-      <c r="C6" s="21">
-        <v>8300</v>
-      </c>
-      <c r="D6" s="21">
-        <v>5775</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="20" t="s">
-        <v>72</v>
-      </c>
-      <c r="B7" s="21">
-        <v>-5400</v>
-      </c>
-      <c r="C7" s="21">
-        <v>17625</v>
-      </c>
-      <c r="D7" s="21">
-        <v>12225</v>
+      <c r="B8" s="21">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
hanay zadt everage profit dyal kol pair
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF1402EA-519A-4C45-854E-5B08AAF2B112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01105BA2-9301-463A-8E3C-6936D0964982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="75">
   <si>
     <t>TradeID</t>
   </si>
@@ -301,6 +301,9 @@
   </si>
   <si>
     <t>Count of TradeID</t>
+  </si>
+  <si>
+    <t>Average of Profit</t>
   </si>
 </sst>
 </file>
@@ -898,7 +901,28 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="20">
+    <dxf>
+      <numFmt numFmtId="169" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.00000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.000000"/>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2331,7 +2355,7 @@
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2DA79A61-38FD-45EA-A18C-EAC9CD91845A}" name="PivotTable1" cacheId="20" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A3:C8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
@@ -2352,7 +2376,7 @@
       </items>
     </pivotField>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -2385,12 +2409,33 @@
       <x/>
     </i>
   </rowItems>
-  <colItems count="1">
-    <i/>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
   </colItems>
-  <dataFields count="1">
+  <dataFields count="2">
     <dataField name="Count of TradeID" fld="0" subtotal="count" baseField="3" baseItem="0"/>
+    <dataField name="Average of Profit" fld="5" subtotal="average" baseField="2" baseItem="2"/>
   </dataFields>
+  <formats count="1">
+    <format dxfId="1">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="2" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -2479,14 +2524,14 @@
     <tableColumn id="5" xr3:uid="{539426CC-F875-4D64-977A-05C6F1BCDBCD}" name="Direction"/>
     <tableColumn id="6" xr3:uid="{BFF7C4D2-29D9-4645-98DB-6FBF609AB80F}" name="Profit"/>
     <tableColumn id="7" xr3:uid="{CD8DBAA1-576E-4991-87E5-049F5C232A1F}" name="R"/>
-    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="12">
+    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="19">
       <calculatedColumnFormula>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="11">
+    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="18">
       <calculatedColumnFormula>IFERROR(Table1[[#This Row],[Profit]]/Table1[[#This Row],[R]],"0")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{CC96218F-2F0A-46BB-98E4-8AE8218DB3D7}" name="Result"/>
-    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2498,10 +2543,10 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{DAF88BD0-F115-4C64-AE11-7DD8AB7505A7}" name="Pair"/>
     <tableColumn id="2" xr3:uid="{89E35073-D474-496E-86E0-7646DF314B64}" name="Profit"/>
-    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="9">
+    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="16">
       <calculatedColumnFormula>TRIM(Table2[[#This Row],[Pair]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="8">
+    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="15">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Pair]]=Table2[[#This Row],[Clean Space]],"GOOD","NADFO")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2514,7 +2559,7 @@
   <autoFilter ref="K8:L12" xr:uid="{A99A2C5F-61E0-444B-907C-487860A13E40}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{0A321640-D79C-4135-83F6-E38913427047}" name="raw text"/>
-    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="7">
+    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="14">
       <calculatedColumnFormula>PROPER(Table4[[#This Row],[raw text]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2527,10 +2572,10 @@
   <autoFilter ref="K16:M19" xr:uid="{4576F3CB-3E9B-40EE-B5BA-0228DC3EBD7C}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{3D4EC290-099D-468C-B78D-8A8F427D8214}" name="text num"/>
-    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="6">
+    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="13">
       <calculatedColumnFormula>VALUE(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="5">
+    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="12">
       <calculatedColumnFormula>ISNUMBER(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2539,10 +2584,10 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}" name="Table5" displayName="Table5" ref="Q17:Q25" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}" name="Table5" displayName="Table5" ref="Q17:Q25" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
   <autoFilter ref="Q17:Q25" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{B868BDD4-CA52-440D-A1EA-1585934AF042}" name="TradeID" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{B868BDD4-CA52-440D-A1EA-1585934AF042}" name="TradeID" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2865,64 +2910,82 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A00360D7-0D73-4CE4-AFB9-0AF5F61FAEDB}">
-  <dimension ref="A3:B8"/>
+  <dimension ref="A3:C8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.21875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
         <v>71</v>
       </c>
       <c r="B3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="20" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="21">
         <v>22</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C4" s="15">
+        <v>131.81818181818181</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="20" t="s">
         <v>15</v>
       </c>
       <c r="B5" s="21">
         <v>33</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C5" s="15">
+        <v>206.81818181818181</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="20" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="21">
         <v>27</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C6" s="15">
+        <v>71.296296296296291</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="20" t="s">
         <v>18</v>
       </c>
       <c r="B7" s="21">
         <v>18</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C7" s="15">
+        <v>31.944444444444443</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="20" t="s">
         <v>72</v>
       </c>
       <c r="B8" s="21">
         <v>100</v>
+      </c>
+      <c r="C8" s="21">
+        <v>122.25</v>
       </c>
     </row>
   </sheetData>
@@ -6713,10 +6776,10 @@
     <mergeCell ref="N6:P6"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
hnaya zadt column dyal result bach na3raf chhal khsartw chhal rba7t fkol group dyal pair
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01105BA2-9301-463A-8E3C-6936D0964982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A129A4B7-84E7-42D3-9670-901CF0B82796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="75">
   <si>
     <t>TradeID</t>
   </si>
@@ -300,10 +300,10 @@
     <t>Grand Total</t>
   </si>
   <si>
-    <t>Count of TradeID</t>
+    <t>Column Labels</t>
   </si>
   <si>
-    <t>Average of Profit</t>
+    <t>Count of TradeID</t>
   </si>
 </sst>
 </file>
@@ -903,10 +903,10 @@
   </cellStyles>
   <dxfs count="20">
     <dxf>
-      <numFmt numFmtId="169" formatCode="0.0"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="169" formatCode="0.0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -2355,7 +2355,7 @@
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2DA79A61-38FD-45EA-A18C-EAC9CD91845A}" name="PivotTable1" cacheId="20" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:C8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <location ref="A3:D9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
@@ -2376,11 +2376,11 @@
       </items>
     </pivotField>
     <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
       <items count="3">
         <item x="1"/>
         <item x="0"/>
@@ -2410,32 +2410,22 @@
     </i>
   </rowItems>
   <colFields count="1">
-    <field x="-2"/>
+    <field x="9"/>
   </colFields>
-  <colItems count="2">
+  <colItems count="3">
     <i>
       <x/>
     </i>
-    <i i="1">
+    <i>
       <x v="1"/>
     </i>
+    <i t="grand">
+      <x/>
+    </i>
   </colItems>
-  <dataFields count="2">
+  <dataFields count="1">
     <dataField name="Count of TradeID" fld="0" subtotal="count" baseField="3" baseItem="0"/>
-    <dataField name="Average of Profit" fld="5" subtotal="average" baseField="2" baseItem="2"/>
   </dataFields>
-  <formats count="1">
-    <format dxfId="1">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="2" count="0"/>
-        </references>
-      </pivotArea>
-    </format>
-  </formats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -2910,82 +2900,108 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A00360D7-0D73-4CE4-AFB9-0AF5F61FAEDB}">
-  <dimension ref="A3:C8"/>
+  <dimension ref="A3:D9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.21875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="B3" t="s">
-        <v>73</v>
-      </c>
-      <c r="C3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="20" t="s">
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="21">
+      <c r="B5" s="21">
+        <v>10</v>
+      </c>
+      <c r="C5" s="21">
+        <v>12</v>
+      </c>
+      <c r="D5" s="21">
         <v>22</v>
       </c>
-      <c r="C4" s="15">
-        <v>131.81818181818181</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="20" t="s">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="21">
+      <c r="B6" s="21">
+        <v>10</v>
+      </c>
+      <c r="C6" s="21">
+        <v>23</v>
+      </c>
+      <c r="D6" s="21">
         <v>33</v>
       </c>
-      <c r="C5" s="15">
-        <v>206.81818181818181</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="20" t="s">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="21">
+      <c r="B7" s="21">
+        <v>11</v>
+      </c>
+      <c r="C7" s="21">
+        <v>16</v>
+      </c>
+      <c r="D7" s="21">
         <v>27</v>
       </c>
-      <c r="C6" s="15">
-        <v>71.296296296296291</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="20" t="s">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="21">
+      <c r="B8" s="21">
+        <v>10</v>
+      </c>
+      <c r="C8" s="21">
+        <v>8</v>
+      </c>
+      <c r="D8" s="21">
         <v>18</v>
       </c>
-      <c r="C7" s="15">
-        <v>31.944444444444443</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="20" t="s">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="B8" s="21">
+      <c r="B9" s="21">
+        <v>41</v>
+      </c>
+      <c r="C9" s="21">
+        <v>59</v>
+      </c>
+      <c r="D9" s="21">
         <v>100</v>
-      </c>
-      <c r="C8" s="21">
-        <v>122.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
hanya zadt row dyal session bach n7awal ndir group w n7sab majmo3 profit dyal kol session
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A129A4B7-84E7-42D3-9670-901CF0B82796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61553E5D-930C-433D-B433-1305BDFE9A8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="74">
   <si>
     <t>TradeID</t>
   </si>
@@ -300,10 +300,7 @@
     <t>Grand Total</t>
   </si>
   <si>
-    <t>Column Labels</t>
-  </si>
-  <si>
-    <t>Count of TradeID</t>
+    <t>Sum of Profit</t>
   </si>
 </sst>
 </file>
@@ -2355,11 +2352,11 @@
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2DA79A61-38FD-45EA-A18C-EAC9CD91845A}" name="PivotTable1" cacheId="20" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:D9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <location ref="A3:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
-    <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
       <items count="5">
         <item x="0"/>
         <item x="1"/>
@@ -2368,7 +2365,7 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField showAll="0">
+    <pivotField axis="axisRow" showAll="0">
       <items count="3">
         <item x="1"/>
         <item x="0"/>
@@ -2376,11 +2373,11 @@
       </items>
     </pivotField>
     <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisCol" showAll="0">
+    <pivotField showAll="0">
       <items count="3">
         <item x="1"/>
         <item x="0"/>
@@ -2390,29 +2387,9 @@
     <pivotField numFmtId="14" showAll="0"/>
   </pivotFields>
   <rowFields count="1">
-    <field x="2"/>
+    <field x="3"/>
   </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="9"/>
-  </colFields>
-  <colItems count="3">
+  <rowItems count="3">
     <i>
       <x/>
     </i>
@@ -2422,9 +2399,12 @@
     <i t="grand">
       <x/>
     </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Count of TradeID" fld="0" subtotal="count" baseField="3" baseItem="0"/>
+    <dataField name="Sum of Profit" fld="5" baseField="0" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -2900,11 +2880,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A00360D7-0D73-4CE4-AFB9-0AF5F61FAEDB}">
-  <dimension ref="A3:D9"/>
+  <dimension ref="A3:B6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
@@ -2912,96 +2892,36 @@
     <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="B3" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="19" t="s">
-        <v>71</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="21">
+        <v>6450</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="21">
+        <v>5775</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="20" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="21">
-        <v>10</v>
-      </c>
-      <c r="C5" s="21">
-        <v>12</v>
-      </c>
-      <c r="D5" s="21">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="20" t="s">
-        <v>15</v>
-      </c>
       <c r="B6" s="21">
-        <v>10</v>
-      </c>
-      <c r="C6" s="21">
-        <v>23</v>
-      </c>
-      <c r="D6" s="21">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="20" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="21">
-        <v>11</v>
-      </c>
-      <c r="C7" s="21">
-        <v>16</v>
-      </c>
-      <c r="D7" s="21">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="21">
-        <v>10</v>
-      </c>
-      <c r="C8" s="21">
-        <v>8</v>
-      </c>
-      <c r="D8" s="21">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="20" t="s">
-        <v>72</v>
-      </c>
-      <c r="B9" s="21">
-        <v>41</v>
-      </c>
-      <c r="C9" s="21">
-        <v>59</v>
-      </c>
-      <c r="D9" s="21">
-        <v>100</v>
+        <v>12225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
hnaya dart analysis dyal pair w session w9aranthom ela hsab profit bach na3raf ina session dyal kola pair kat3ti mz1
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02296191-3952-4689-8A0A-252B2B6FF5E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BB07F58-B1F6-4F17-AFAE-F16B6DEB57D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
     <sheet name="pivot table" sheetId="4" r:id="rId1"/>
@@ -20,7 +20,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="21" r:id="rId5"/>
+    <pivotCache cacheId="0" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="75">
   <si>
     <t>TradeID</t>
   </si>
@@ -297,13 +297,13 @@
     <t>Grand Total</t>
   </si>
   <si>
-    <t>Count of TradeID</t>
-  </si>
-  <si>
     <t>result column</t>
   </si>
   <si>
     <t>session rows</t>
+  </si>
+  <si>
+    <t>Sum of Profit</t>
   </si>
 </sst>
 </file>
@@ -2412,12 +2412,12 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2DA79A61-38FD-45EA-A18C-EAC9CD91845A}" name="PivotTable1" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="session rows" colHeaderCaption="result column">
-  <location ref="A3:D7" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2DA79A61-38FD-45EA-A18C-EAC9CD91845A}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="session rows" colHeaderCaption="result column">
+  <location ref="A3:D9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="11">
-    <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
       <items count="5">
         <item x="0"/>
         <item x="1"/>
@@ -2426,7 +2426,7 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField axis="axisRow" showAll="0">
+    <pivotField axis="axisCol" showAll="0">
       <items count="3">
         <item x="1"/>
         <item x="0"/>
@@ -2434,11 +2434,11 @@
       </items>
     </pivotField>
     <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisCol" showAll="0">
+    <pivotField showAll="0">
       <items count="3">
         <item x="1"/>
         <item x="0"/>
@@ -2530,21 +2530,27 @@
     </pivotField>
   </pivotFields>
   <rowFields count="1">
-    <field x="3"/>
+    <field x="2"/>
   </rowFields>
-  <rowItems count="3">
+  <rowItems count="5">
     <i>
       <x/>
     </i>
     <i>
       <x v="1"/>
     </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
     <i t="grand">
       <x/>
     </i>
   </rowItems>
   <colFields count="1">
-    <field x="9"/>
+    <field x="3"/>
   </colFields>
   <colItems count="3">
     <i>
@@ -2558,7 +2564,7 @@
     </i>
   </colItems>
   <dataFields count="1">
-    <dataField name="Count of TradeID" fld="0" subtotal="count" baseField="3" baseItem="0"/>
+    <dataField name="Sum of Profit" fld="5" baseField="0" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -3034,35 +3040,36 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A00360D7-0D73-4CE4-AFB9-0AF5F61FAEDB}">
-  <dimension ref="A3:D7"/>
+  <dimension ref="A3:D9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="B3" s="19" t="s">
         <v>72</v>
-      </c>
-      <c r="B3" s="19" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D4" t="s">
         <v>71</v>
@@ -3070,44 +3077,72 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="20" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B5" s="21">
-        <v>23</v>
+        <v>1975</v>
       </c>
       <c r="C5" s="21">
-        <v>33</v>
+        <v>925</v>
       </c>
       <c r="D5" s="21">
-        <v>56</v>
+        <v>2900</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B6" s="21">
-        <v>18</v>
+        <v>3075</v>
       </c>
       <c r="C6" s="21">
-        <v>26</v>
+        <v>3750</v>
       </c>
       <c r="D6" s="21">
-        <v>44</v>
+        <v>6825</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="21">
+        <v>1275</v>
+      </c>
+      <c r="C7" s="21">
+        <v>650</v>
+      </c>
+      <c r="D7" s="21">
+        <v>1925</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="21">
+        <v>125</v>
+      </c>
+      <c r="C8" s="21">
+        <v>450</v>
+      </c>
+      <c r="D8" s="21">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="B7" s="21">
-        <v>41</v>
-      </c>
-      <c r="C7" s="21">
-        <v>59</v>
-      </c>
-      <c r="D7" s="21">
-        <v>100</v>
+      <c r="B9" s="21">
+        <v>6450</v>
+      </c>
+      <c r="C9" s="21">
+        <v>5775</v>
+      </c>
+      <c r="D9" s="21">
+        <v>12225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
hnaya zadt average profit dyal kol pair ela hsab session
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BB07F58-B1F6-4F17-AFAE-F16B6DEB57D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14F8A184-D81A-4108-B159-15FA5AEDE627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
-    <sheet name="pivot table" sheetId="4" r:id="rId1"/>
-    <sheet name="trading_raw_data2" sheetId="1" r:id="rId2"/>
-    <sheet name="data analysis" sheetId="2" r:id="rId3"/>
-    <sheet name="data cleaning " sheetId="3" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="5" r:id="rId1"/>
+    <sheet name="pivot table" sheetId="4" r:id="rId2"/>
+    <sheet name="trading_raw_data2" sheetId="1" r:id="rId3"/>
+    <sheet name="data analysis" sheetId="2" r:id="rId4"/>
+    <sheet name="data cleaning " sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId5"/>
+    <pivotCache cacheId="0" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -79,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="77">
   <si>
     <t>TradeID</t>
   </si>
@@ -303,7 +304,13 @@
     <t>session rows</t>
   </si>
   <si>
-    <t>Sum of Profit</t>
+    <t>GOOD</t>
+  </si>
+  <si>
+    <t>REVIEW</t>
+  </si>
+  <si>
+    <t>Average of Profit</t>
   </si>
 </sst>
 </file>
@@ -901,7 +908,25 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="19">
+    <dxf>
+      <numFmt numFmtId="168" formatCode="0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="167" formatCode="0.0000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="166" formatCode="0.00000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.000000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2564,8 +2589,17 @@
     </i>
   </colItems>
   <dataFields count="1">
-    <dataField name="Sum of Profit" fld="5" baseField="0" baseItem="0"/>
+    <dataField name="Average of Profit" fld="5" subtotal="average" baseField="2" baseItem="1"/>
   </dataFields>
+  <formats count="1">
+    <format dxfId="1">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="1">
+          <reference field="2" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -2641,6 +2675,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{3E02DECA-88F9-4E49-B9E5-EC28AE4B45F9}" name="Table6" displayName="Table6" ref="A1:K57" totalsRowShown="0">
+  <autoFilter ref="A1:K57" xr:uid="{3E02DECA-88F9-4E49-B9E5-EC28AE4B45F9}"/>
+  <tableColumns count="11">
+    <tableColumn id="1" xr3:uid="{37C8F018-C5F6-4B41-B7EC-08016868A732}" name="TradeID"/>
+    <tableColumn id="2" xr3:uid="{76FD4B7D-B7A9-4301-9985-DA8BC98B8253}" name="AccountID"/>
+    <tableColumn id="3" xr3:uid="{9195B2E7-A1DC-4F68-BCFE-F436A5F42CF9}" name="Pair"/>
+    <tableColumn id="4" xr3:uid="{640A7DC7-1688-480E-89F1-0C1DF4CF8DDC}" name="Session"/>
+    <tableColumn id="5" xr3:uid="{003D0FE2-16A7-4C56-A80C-17A9CD790A0F}" name="Direction"/>
+    <tableColumn id="6" xr3:uid="{9196FB82-D35E-4156-BFCE-F69F992A7299}" name="Profit"/>
+    <tableColumn id="7" xr3:uid="{86776ACD-4D39-428F-A446-A0957F0111A8}" name="R"/>
+    <tableColumn id="8" xr3:uid="{011760A3-A9D1-4015-8D75-7EFE2A2FEB20}" name="Risk Status"/>
+    <tableColumn id="9" xr3:uid="{8E6DF200-182D-483A-8ED0-12101EFECD0F}" name="Profit per R"/>
+    <tableColumn id="10" xr3:uid="{BB6361CF-CAA7-4423-9C5D-82E0E0F6DBCD}" name="Result"/>
+    <tableColumn id="11" xr3:uid="{420DB1BF-4073-4932-87BC-11D2FECAB843}" name="TradeDate" dataDxfId="5"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E6EB144A-984A-4FCF-892A-EB44514BDE51}" name="Table1" displayName="Table1" ref="A1:K101" totalsRowShown="0">
   <autoFilter ref="A1:K101" xr:uid="{E6EB144A-984A-4FCF-892A-EB44514BDE51}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K101">
@@ -2654,29 +2708,29 @@
     <tableColumn id="5" xr3:uid="{539426CC-F875-4D64-977A-05C6F1BCDBCD}" name="Direction"/>
     <tableColumn id="6" xr3:uid="{BFF7C4D2-29D9-4645-98DB-6FBF609AB80F}" name="Profit"/>
     <tableColumn id="7" xr3:uid="{CD8DBAA1-576E-4991-87E5-049F5C232A1F}" name="R"/>
-    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="12">
+    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="18">
       <calculatedColumnFormula>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="11">
+    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="17">
       <calculatedColumnFormula>IFERROR(Table1[[#This Row],[Profit]]/Table1[[#This Row],[R]],"0")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{CC96218F-2F0A-46BB-98E4-8AE8218DB3D7}" name="Result"/>
-    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5280782B-FEC2-415C-8A49-51730C483074}" name="Table2" displayName="Table2" ref="F8:I13" totalsRowShown="0">
   <autoFilter ref="F8:I13" xr:uid="{5280782B-FEC2-415C-8A49-51730C483074}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{DAF88BD0-F115-4C64-AE11-7DD8AB7505A7}" name="Pair"/>
     <tableColumn id="2" xr3:uid="{89E35073-D474-496E-86E0-7646DF314B64}" name="Profit"/>
-    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="9">
+    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="15">
       <calculatedColumnFormula>TRIM(Table2[[#This Row],[Pair]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="8">
+    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="14">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Pair]]=Table2[[#This Row],[Clean Space]],"GOOD","NADFO")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2684,12 +2738,12 @@
 </table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{A99A2C5F-61E0-444B-907C-487860A13E40}" name="Table4" displayName="Table4" ref="K8:L12" totalsRowShown="0">
   <autoFilter ref="K8:L12" xr:uid="{A99A2C5F-61E0-444B-907C-487860A13E40}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{0A321640-D79C-4135-83F6-E38913427047}" name="raw text"/>
-    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="7">
+    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="13">
       <calculatedColumnFormula>PROPER(Table4[[#This Row],[raw text]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2697,15 +2751,15 @@
 </table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{4576F3CB-3E9B-40EE-B5BA-0228DC3EBD7C}" name="Table3" displayName="Table3" ref="K16:M19" totalsRowShown="0">
   <autoFilter ref="K16:M19" xr:uid="{4576F3CB-3E9B-40EE-B5BA-0228DC3EBD7C}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{3D4EC290-099D-468C-B78D-8A8F427D8214}" name="text num"/>
-    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="6">
+    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="12">
       <calculatedColumnFormula>VALUE(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="5">
+    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="11">
       <calculatedColumnFormula>ISNUMBER(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2713,11 +2767,11 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}" name="Table5" displayName="Table5" ref="Q17:Q25" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}" name="Table5" displayName="Table5" ref="Q17:Q25" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="Q17:Q25" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{B868BDD4-CA52-440D-A1EA-1585934AF042}" name="TradeID" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{B868BDD4-CA52-440D-A1EA-1585934AF042}" name="TradeID" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3039,14 +3093,2030 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F1F068E-53F4-486C-916C-A193B94A4681}">
+  <dimension ref="A1:K57"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.33203125" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" customWidth="1"/>
+    <col min="5" max="5" width="10.5546875" customWidth="1"/>
+    <col min="8" max="8" width="12.109375" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+    <col min="11" max="11" width="11.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>36</v>
+      </c>
+      <c r="I1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>16</v>
+      </c>
+      <c r="B2">
+        <v>10006</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2">
+        <v>500</v>
+      </c>
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2" t="s">
+        <v>74</v>
+      </c>
+      <c r="I2">
+        <v>250</v>
+      </c>
+      <c r="J2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K2" s="1">
+        <v>46168</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>78</v>
+      </c>
+      <c r="B3">
+        <v>10001</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3">
+        <v>500</v>
+      </c>
+      <c r="G3">
+        <v>2</v>
+      </c>
+      <c r="H3" t="s">
+        <v>74</v>
+      </c>
+      <c r="I3">
+        <v>250</v>
+      </c>
+      <c r="J3" t="s">
+        <v>12</v>
+      </c>
+      <c r="K3" s="1">
+        <v>46182</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>35</v>
+      </c>
+      <c r="B4">
+        <v>10005</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4">
+        <v>375</v>
+      </c>
+      <c r="G4">
+        <v>1.5</v>
+      </c>
+      <c r="H4" t="s">
+        <v>75</v>
+      </c>
+      <c r="I4">
+        <v>250</v>
+      </c>
+      <c r="J4" t="s">
+        <v>12</v>
+      </c>
+      <c r="K4" s="1">
+        <v>46041</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>45</v>
+      </c>
+      <c r="B5">
+        <v>10003</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5">
+        <v>375</v>
+      </c>
+      <c r="G5">
+        <v>1.5</v>
+      </c>
+      <c r="H5" t="s">
+        <v>75</v>
+      </c>
+      <c r="I5">
+        <v>250</v>
+      </c>
+      <c r="J5" t="s">
+        <v>12</v>
+      </c>
+      <c r="K5" s="1">
+        <v>46055</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>43</v>
+      </c>
+      <c r="B6">
+        <v>10003</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6">
+        <v>200</v>
+      </c>
+      <c r="G6">
+        <v>2</v>
+      </c>
+      <c r="H6" t="s">
+        <v>74</v>
+      </c>
+      <c r="I6">
+        <v>100</v>
+      </c>
+      <c r="J6" t="s">
+        <v>12</v>
+      </c>
+      <c r="K6" s="1">
+        <v>46091</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>77</v>
+      </c>
+      <c r="B7">
+        <v>10006</v>
+      </c>
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7">
+        <v>200</v>
+      </c>
+      <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7" t="s">
+        <v>74</v>
+      </c>
+      <c r="I7">
+        <v>100</v>
+      </c>
+      <c r="J7" t="s">
+        <v>12</v>
+      </c>
+      <c r="K7" s="1">
+        <v>46198</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>99</v>
+      </c>
+      <c r="B8">
+        <v>10006</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" t="s">
+        <v>10</v>
+      </c>
+      <c r="E8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8">
+        <v>125</v>
+      </c>
+      <c r="G8">
+        <v>2.5</v>
+      </c>
+      <c r="H8" t="s">
+        <v>74</v>
+      </c>
+      <c r="I8">
+        <v>50</v>
+      </c>
+      <c r="J8" t="s">
+        <v>12</v>
+      </c>
+      <c r="K8" s="1">
+        <v>46101</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>97</v>
+      </c>
+      <c r="B9">
+        <v>10006</v>
+      </c>
+      <c r="C9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9">
+        <v>100</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9" t="s">
+        <v>75</v>
+      </c>
+      <c r="I9">
+        <v>100</v>
+      </c>
+      <c r="J9" t="s">
+        <v>12</v>
+      </c>
+      <c r="K9" s="1">
+        <v>46172</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>1</v>
+      </c>
+      <c r="B10">
+        <v>10002</v>
+      </c>
+      <c r="C10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10">
+        <v>50</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10" t="s">
+        <v>75</v>
+      </c>
+      <c r="I10">
+        <v>50</v>
+      </c>
+      <c r="J10" t="s">
+        <v>12</v>
+      </c>
+      <c r="K10" s="1">
+        <v>46190</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>38</v>
+      </c>
+      <c r="B11">
+        <v>10005</v>
+      </c>
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11">
+        <v>-25</v>
+      </c>
+      <c r="G11">
+        <v>-0.5</v>
+      </c>
+      <c r="H11" t="s">
+        <v>75</v>
+      </c>
+      <c r="I11">
+        <v>50</v>
+      </c>
+      <c r="J11" t="s">
+        <v>17</v>
+      </c>
+      <c r="K11" s="1">
+        <v>46107</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>30</v>
+      </c>
+      <c r="B12">
+        <v>10001</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12">
+        <v>-50</v>
+      </c>
+      <c r="G12">
+        <v>-0.5</v>
+      </c>
+      <c r="H12" t="s">
+        <v>75</v>
+      </c>
+      <c r="I12">
+        <v>100</v>
+      </c>
+      <c r="J12" t="s">
+        <v>17</v>
+      </c>
+      <c r="K12" s="1">
+        <v>46167</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>86</v>
+      </c>
+      <c r="B13">
+        <v>10002</v>
+      </c>
+      <c r="C13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13">
+        <v>-100</v>
+      </c>
+      <c r="G13">
+        <v>-1</v>
+      </c>
+      <c r="H13" t="s">
+        <v>75</v>
+      </c>
+      <c r="I13">
+        <v>100</v>
+      </c>
+      <c r="J13" t="s">
+        <v>17</v>
+      </c>
+      <c r="K13" s="1">
+        <v>46169</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>61</v>
+      </c>
+      <c r="B14">
+        <v>10005</v>
+      </c>
+      <c r="C14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14">
+        <v>-125</v>
+      </c>
+      <c r="G14">
+        <v>-0.5</v>
+      </c>
+      <c r="H14" t="s">
+        <v>75</v>
+      </c>
+      <c r="I14">
+        <v>250</v>
+      </c>
+      <c r="J14" t="s">
+        <v>17</v>
+      </c>
+      <c r="K14" s="1">
+        <v>46033</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>34</v>
+      </c>
+      <c r="B15">
+        <v>10005</v>
+      </c>
+      <c r="C15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15">
+        <v>-150</v>
+      </c>
+      <c r="G15">
+        <v>-1.5</v>
+      </c>
+      <c r="H15" t="s">
+        <v>75</v>
+      </c>
+      <c r="I15">
+        <v>100</v>
+      </c>
+      <c r="J15" t="s">
+        <v>17</v>
+      </c>
+      <c r="K15" s="1">
+        <v>46107</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>13</v>
+      </c>
+      <c r="B16">
+        <v>10006</v>
+      </c>
+      <c r="C16" t="s">
+        <v>15</v>
+      </c>
+      <c r="D16" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16">
+        <v>750</v>
+      </c>
+      <c r="G16">
+        <v>3</v>
+      </c>
+      <c r="H16" t="s">
+        <v>74</v>
+      </c>
+      <c r="I16">
+        <v>250</v>
+      </c>
+      <c r="J16" t="s">
+        <v>12</v>
+      </c>
+      <c r="K16" s="1">
+        <v>46094</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>98</v>
+      </c>
+      <c r="B17">
+        <v>10001</v>
+      </c>
+      <c r="C17" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17">
+        <v>750</v>
+      </c>
+      <c r="G17">
+        <v>3</v>
+      </c>
+      <c r="H17" t="s">
+        <v>74</v>
+      </c>
+      <c r="I17">
+        <v>250</v>
+      </c>
+      <c r="J17" t="s">
+        <v>12</v>
+      </c>
+      <c r="K17" s="1">
+        <v>46088</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>68</v>
+      </c>
+      <c r="B18">
+        <v>10004</v>
+      </c>
+      <c r="C18" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18">
+        <v>625</v>
+      </c>
+      <c r="G18">
+        <v>2.5</v>
+      </c>
+      <c r="H18" t="s">
+        <v>74</v>
+      </c>
+      <c r="I18">
+        <v>250</v>
+      </c>
+      <c r="J18" t="s">
+        <v>12</v>
+      </c>
+      <c r="K18" s="1">
+        <v>46207</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>76</v>
+      </c>
+      <c r="B19">
+        <v>10005</v>
+      </c>
+      <c r="C19" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19">
+        <v>375</v>
+      </c>
+      <c r="G19">
+        <v>1.5</v>
+      </c>
+      <c r="H19" t="s">
+        <v>75</v>
+      </c>
+      <c r="I19">
+        <v>250</v>
+      </c>
+      <c r="J19" t="s">
+        <v>12</v>
+      </c>
+      <c r="K19" s="1">
+        <v>46034</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>10</v>
+      </c>
+      <c r="B20">
+        <v>10004</v>
+      </c>
+      <c r="C20" t="s">
+        <v>15</v>
+      </c>
+      <c r="D20" t="s">
+        <v>10</v>
+      </c>
+      <c r="E20" t="s">
+        <v>14</v>
+      </c>
+      <c r="F20">
+        <v>300</v>
+      </c>
+      <c r="G20">
+        <v>3</v>
+      </c>
+      <c r="H20" t="s">
+        <v>74</v>
+      </c>
+      <c r="I20">
+        <v>100</v>
+      </c>
+      <c r="J20" t="s">
+        <v>12</v>
+      </c>
+      <c r="K20" s="1">
+        <v>46182</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>23</v>
+      </c>
+      <c r="B21">
+        <v>10003</v>
+      </c>
+      <c r="C21" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" t="s">
+        <v>10</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21">
+        <v>300</v>
+      </c>
+      <c r="G21">
+        <v>3</v>
+      </c>
+      <c r="H21" t="s">
+        <v>74</v>
+      </c>
+      <c r="I21">
+        <v>100</v>
+      </c>
+      <c r="J21" t="s">
+        <v>12</v>
+      </c>
+      <c r="K21" s="1">
+        <v>46057</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>63</v>
+      </c>
+      <c r="B22">
+        <v>10001</v>
+      </c>
+      <c r="C22" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22" t="s">
+        <v>10</v>
+      </c>
+      <c r="E22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22">
+        <v>250</v>
+      </c>
+      <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22" t="s">
+        <v>75</v>
+      </c>
+      <c r="I22">
+        <v>250</v>
+      </c>
+      <c r="J22" t="s">
+        <v>12</v>
+      </c>
+      <c r="K22" s="1">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>7</v>
+      </c>
+      <c r="B23">
+        <v>10006</v>
+      </c>
+      <c r="C23" t="s">
+        <v>15</v>
+      </c>
+      <c r="D23" t="s">
+        <v>10</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23">
+        <v>100</v>
+      </c>
+      <c r="G23">
+        <v>2</v>
+      </c>
+      <c r="H23" t="s">
+        <v>74</v>
+      </c>
+      <c r="I23">
+        <v>50</v>
+      </c>
+      <c r="J23" t="s">
+        <v>12</v>
+      </c>
+      <c r="K23" s="1">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>20</v>
+      </c>
+      <c r="B24">
+        <v>10006</v>
+      </c>
+      <c r="C24" t="s">
+        <v>15</v>
+      </c>
+      <c r="D24" t="s">
+        <v>10</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24">
+        <v>100</v>
+      </c>
+      <c r="G24">
+        <v>1</v>
+      </c>
+      <c r="H24" t="s">
+        <v>75</v>
+      </c>
+      <c r="I24">
+        <v>100</v>
+      </c>
+      <c r="J24" t="s">
+        <v>12</v>
+      </c>
+      <c r="K24" s="1">
+        <v>46041</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>10006</v>
+      </c>
+      <c r="C25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D25" t="s">
+        <v>10</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25">
+        <v>-25</v>
+      </c>
+      <c r="G25">
+        <v>-0.5</v>
+      </c>
+      <c r="H25" t="s">
+        <v>75</v>
+      </c>
+      <c r="I25">
+        <v>50</v>
+      </c>
+      <c r="J25" t="s">
+        <v>17</v>
+      </c>
+      <c r="K25" s="1">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>14</v>
+      </c>
+      <c r="B26">
+        <v>10001</v>
+      </c>
+      <c r="C26" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" t="s">
+        <v>10</v>
+      </c>
+      <c r="E26" t="s">
+        <v>11</v>
+      </c>
+      <c r="F26">
+        <v>-50</v>
+      </c>
+      <c r="G26">
+        <v>-0.5</v>
+      </c>
+      <c r="H26" t="s">
+        <v>75</v>
+      </c>
+      <c r="I26">
+        <v>100</v>
+      </c>
+      <c r="J26" t="s">
+        <v>17</v>
+      </c>
+      <c r="K26" s="1">
+        <v>46119</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>49</v>
+      </c>
+      <c r="B27">
+        <v>10001</v>
+      </c>
+      <c r="C27" t="s">
+        <v>15</v>
+      </c>
+      <c r="D27" t="s">
+        <v>10</v>
+      </c>
+      <c r="E27" t="s">
+        <v>11</v>
+      </c>
+      <c r="F27">
+        <v>-50</v>
+      </c>
+      <c r="G27">
+        <v>-0.5</v>
+      </c>
+      <c r="H27" t="s">
+        <v>75</v>
+      </c>
+      <c r="I27">
+        <v>100</v>
+      </c>
+      <c r="J27" t="s">
+        <v>17</v>
+      </c>
+      <c r="K27" s="1">
+        <v>46095</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>79</v>
+      </c>
+      <c r="B28">
+        <v>10001</v>
+      </c>
+      <c r="C28" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" t="s">
+        <v>10</v>
+      </c>
+      <c r="E28" t="s">
+        <v>14</v>
+      </c>
+      <c r="F28">
+        <v>-50</v>
+      </c>
+      <c r="G28">
+        <v>-1</v>
+      </c>
+      <c r="H28" t="s">
+        <v>75</v>
+      </c>
+      <c r="I28">
+        <v>50</v>
+      </c>
+      <c r="J28" t="s">
+        <v>17</v>
+      </c>
+      <c r="K28" s="1">
+        <v>46128</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>36</v>
+      </c>
+      <c r="B29">
+        <v>10004</v>
+      </c>
+      <c r="C29" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" t="s">
+        <v>10</v>
+      </c>
+      <c r="E29" t="s">
+        <v>14</v>
+      </c>
+      <c r="F29">
+        <v>-300</v>
+      </c>
+      <c r="G29">
+        <v>-1.5</v>
+      </c>
+      <c r="H29" t="s">
+        <v>75</v>
+      </c>
+      <c r="I29">
+        <v>200</v>
+      </c>
+      <c r="J29" t="s">
+        <v>17</v>
+      </c>
+      <c r="K29" s="1">
+        <v>46057</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>82</v>
+      </c>
+      <c r="B30">
+        <v>10005</v>
+      </c>
+      <c r="C30" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30">
+        <v>-375</v>
+      </c>
+      <c r="G30">
+        <v>-1.5</v>
+      </c>
+      <c r="H30" t="s">
+        <v>75</v>
+      </c>
+      <c r="I30">
+        <v>250</v>
+      </c>
+      <c r="J30" t="s">
+        <v>17</v>
+      </c>
+      <c r="K30" s="1">
+        <v>46066</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>5</v>
+      </c>
+      <c r="B31">
+        <v>10003</v>
+      </c>
+      <c r="C31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" t="s">
+        <v>10</v>
+      </c>
+      <c r="E31" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31">
+        <v>-125</v>
+      </c>
+      <c r="G31">
+        <v>-0.5</v>
+      </c>
+      <c r="H31" t="s">
+        <v>75</v>
+      </c>
+      <c r="I31">
+        <v>250</v>
+      </c>
+      <c r="J31" t="s">
+        <v>17</v>
+      </c>
+      <c r="K31" s="1">
+        <v>46050</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>48</v>
+      </c>
+      <c r="B32">
+        <v>10006</v>
+      </c>
+      <c r="C32" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" t="s">
+        <v>10</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32">
+        <v>-100</v>
+      </c>
+      <c r="G32">
+        <v>-1</v>
+      </c>
+      <c r="H32" t="s">
+        <v>75</v>
+      </c>
+      <c r="I32">
+        <v>100</v>
+      </c>
+      <c r="J32" t="s">
+        <v>17</v>
+      </c>
+      <c r="K32" s="1">
+        <v>46072</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>21</v>
+      </c>
+      <c r="B33">
+        <v>10005</v>
+      </c>
+      <c r="C33" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" t="s">
+        <v>10</v>
+      </c>
+      <c r="E33" t="s">
+        <v>11</v>
+      </c>
+      <c r="F33">
+        <v>-100</v>
+      </c>
+      <c r="G33">
+        <v>-1</v>
+      </c>
+      <c r="H33" t="s">
+        <v>75</v>
+      </c>
+      <c r="I33">
+        <v>100</v>
+      </c>
+      <c r="J33" t="s">
+        <v>17</v>
+      </c>
+      <c r="K33" s="1">
+        <v>46059</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>17</v>
+      </c>
+      <c r="B34">
+        <v>10005</v>
+      </c>
+      <c r="C34" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" t="s">
+        <v>10</v>
+      </c>
+      <c r="E34" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34">
+        <v>-75</v>
+      </c>
+      <c r="G34">
+        <v>-1.5</v>
+      </c>
+      <c r="H34" t="s">
+        <v>75</v>
+      </c>
+      <c r="I34">
+        <v>50</v>
+      </c>
+      <c r="J34" t="s">
+        <v>17</v>
+      </c>
+      <c r="K34" s="1">
+        <v>46067</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>75</v>
+      </c>
+      <c r="B35">
+        <v>10003</v>
+      </c>
+      <c r="C35" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" t="s">
+        <v>10</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35">
+        <v>50</v>
+      </c>
+      <c r="G35">
+        <v>1</v>
+      </c>
+      <c r="H35" t="s">
+        <v>75</v>
+      </c>
+      <c r="I35">
+        <v>50</v>
+      </c>
+      <c r="J35" t="s">
+        <v>12</v>
+      </c>
+      <c r="K35" s="1">
+        <v>46047</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>72</v>
+      </c>
+      <c r="B36">
+        <v>10004</v>
+      </c>
+      <c r="C36" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" t="s">
+        <v>10</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36">
+        <v>50</v>
+      </c>
+      <c r="G36">
+        <v>1</v>
+      </c>
+      <c r="H36" t="s">
+        <v>75</v>
+      </c>
+      <c r="I36">
+        <v>50</v>
+      </c>
+      <c r="J36" t="s">
+        <v>12</v>
+      </c>
+      <c r="K36" s="1">
+        <v>46069</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>94</v>
+      </c>
+      <c r="B37">
+        <v>10004</v>
+      </c>
+      <c r="C37" t="s">
+        <v>13</v>
+      </c>
+      <c r="D37" t="s">
+        <v>10</v>
+      </c>
+      <c r="E37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F37">
+        <v>150</v>
+      </c>
+      <c r="G37">
+        <v>3</v>
+      </c>
+      <c r="H37" t="s">
+        <v>74</v>
+      </c>
+      <c r="I37">
+        <v>50</v>
+      </c>
+      <c r="J37" t="s">
+        <v>12</v>
+      </c>
+      <c r="K37" s="1">
+        <v>46091</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>2</v>
+      </c>
+      <c r="B38">
+        <v>10001</v>
+      </c>
+      <c r="C38" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" t="s">
+        <v>10</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38">
+        <v>150</v>
+      </c>
+      <c r="G38">
+        <v>3</v>
+      </c>
+      <c r="H38" t="s">
+        <v>74</v>
+      </c>
+      <c r="I38">
+        <v>50</v>
+      </c>
+      <c r="J38" t="s">
+        <v>12</v>
+      </c>
+      <c r="K38" s="1">
+        <v>46178</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>66</v>
+      </c>
+      <c r="B39">
+        <v>10004</v>
+      </c>
+      <c r="C39" t="s">
+        <v>13</v>
+      </c>
+      <c r="D39" t="s">
+        <v>10</v>
+      </c>
+      <c r="E39" t="s">
+        <v>11</v>
+      </c>
+      <c r="F39">
+        <v>200</v>
+      </c>
+      <c r="G39">
+        <v>2</v>
+      </c>
+      <c r="H39" t="s">
+        <v>74</v>
+      </c>
+      <c r="I39">
+        <v>100</v>
+      </c>
+      <c r="J39" t="s">
+        <v>12</v>
+      </c>
+      <c r="K39" s="1">
+        <v>46160</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>59</v>
+      </c>
+      <c r="B40">
+        <v>10006</v>
+      </c>
+      <c r="C40" t="s">
+        <v>13</v>
+      </c>
+      <c r="D40" t="s">
+        <v>10</v>
+      </c>
+      <c r="E40" t="s">
+        <v>11</v>
+      </c>
+      <c r="F40">
+        <v>200</v>
+      </c>
+      <c r="G40">
+        <v>1</v>
+      </c>
+      <c r="H40" t="s">
+        <v>75</v>
+      </c>
+      <c r="I40">
+        <v>200</v>
+      </c>
+      <c r="J40" t="s">
+        <v>12</v>
+      </c>
+      <c r="K40" s="1">
+        <v>46140</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>55</v>
+      </c>
+      <c r="B41">
+        <v>10005</v>
+      </c>
+      <c r="C41" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" t="s">
+        <v>10</v>
+      </c>
+      <c r="E41" t="s">
+        <v>11</v>
+      </c>
+      <c r="F41">
+        <v>200</v>
+      </c>
+      <c r="G41">
+        <v>1</v>
+      </c>
+      <c r="H41" t="s">
+        <v>75</v>
+      </c>
+      <c r="I41">
+        <v>200</v>
+      </c>
+      <c r="J41" t="s">
+        <v>12</v>
+      </c>
+      <c r="K41" s="1">
+        <v>46120</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>26</v>
+      </c>
+      <c r="B42">
+        <v>10004</v>
+      </c>
+      <c r="C42" t="s">
+        <v>13</v>
+      </c>
+      <c r="D42" t="s">
+        <v>10</v>
+      </c>
+      <c r="E42" t="s">
+        <v>11</v>
+      </c>
+      <c r="F42">
+        <v>250</v>
+      </c>
+      <c r="G42">
+        <v>1</v>
+      </c>
+      <c r="H42" t="s">
+        <v>75</v>
+      </c>
+      <c r="I42">
+        <v>250</v>
+      </c>
+      <c r="J42" t="s">
+        <v>12</v>
+      </c>
+      <c r="K42" s="1">
+        <v>46173</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>65</v>
+      </c>
+      <c r="B43">
+        <v>10004</v>
+      </c>
+      <c r="C43" t="s">
+        <v>13</v>
+      </c>
+      <c r="D43" t="s">
+        <v>10</v>
+      </c>
+      <c r="E43" t="s">
+        <v>11</v>
+      </c>
+      <c r="F43">
+        <v>300</v>
+      </c>
+      <c r="G43">
+        <v>1.5</v>
+      </c>
+      <c r="H43" t="s">
+        <v>75</v>
+      </c>
+      <c r="I43">
+        <v>200</v>
+      </c>
+      <c r="J43" t="s">
+        <v>12</v>
+      </c>
+      <c r="K43" s="1">
+        <v>46167</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>73</v>
+      </c>
+      <c r="B44">
+        <v>10002</v>
+      </c>
+      <c r="C44" t="s">
+        <v>13</v>
+      </c>
+      <c r="D44" t="s">
+        <v>10</v>
+      </c>
+      <c r="E44" t="s">
+        <v>11</v>
+      </c>
+      <c r="F44">
+        <v>500</v>
+      </c>
+      <c r="G44">
+        <v>2.5</v>
+      </c>
+      <c r="H44" t="s">
+        <v>74</v>
+      </c>
+      <c r="I44">
+        <v>200</v>
+      </c>
+      <c r="J44" t="s">
+        <v>12</v>
+      </c>
+      <c r="K44" s="1">
+        <v>46191</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <v>58</v>
+      </c>
+      <c r="B45">
+        <v>10005</v>
+      </c>
+      <c r="C45" t="s">
+        <v>18</v>
+      </c>
+      <c r="D45" t="s">
+        <v>10</v>
+      </c>
+      <c r="E45" t="s">
+        <v>11</v>
+      </c>
+      <c r="F45">
+        <v>-250</v>
+      </c>
+      <c r="G45">
+        <v>-1</v>
+      </c>
+      <c r="H45" t="s">
+        <v>75</v>
+      </c>
+      <c r="I45">
+        <v>250</v>
+      </c>
+      <c r="J45" t="s">
+        <v>17</v>
+      </c>
+      <c r="K45" s="1">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>42</v>
+      </c>
+      <c r="B46">
+        <v>10002</v>
+      </c>
+      <c r="C46" t="s">
+        <v>18</v>
+      </c>
+      <c r="D46" t="s">
+        <v>10</v>
+      </c>
+      <c r="E46" t="s">
+        <v>11</v>
+      </c>
+      <c r="F46">
+        <v>-250</v>
+      </c>
+      <c r="G46">
+        <v>-1</v>
+      </c>
+      <c r="H46" t="s">
+        <v>75</v>
+      </c>
+      <c r="I46">
+        <v>250</v>
+      </c>
+      <c r="J46" t="s">
+        <v>17</v>
+      </c>
+      <c r="K46" s="1">
+        <v>46096</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <v>51</v>
+      </c>
+      <c r="B47">
+        <v>10003</v>
+      </c>
+      <c r="C47" t="s">
+        <v>18</v>
+      </c>
+      <c r="D47" t="s">
+        <v>10</v>
+      </c>
+      <c r="E47" t="s">
+        <v>11</v>
+      </c>
+      <c r="F47">
+        <v>-200</v>
+      </c>
+      <c r="G47">
+        <v>-1</v>
+      </c>
+      <c r="H47" t="s">
+        <v>75</v>
+      </c>
+      <c r="I47">
+        <v>200</v>
+      </c>
+      <c r="J47" t="s">
+        <v>17</v>
+      </c>
+      <c r="K47" s="1">
+        <v>46111</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>11</v>
+      </c>
+      <c r="B48">
+        <v>10001</v>
+      </c>
+      <c r="C48" t="s">
+        <v>18</v>
+      </c>
+      <c r="D48" t="s">
+        <v>10</v>
+      </c>
+      <c r="E48" t="s">
+        <v>14</v>
+      </c>
+      <c r="F48">
+        <v>-200</v>
+      </c>
+      <c r="G48">
+        <v>-1</v>
+      </c>
+      <c r="H48" t="s">
+        <v>75</v>
+      </c>
+      <c r="I48">
+        <v>200</v>
+      </c>
+      <c r="J48" t="s">
+        <v>17</v>
+      </c>
+      <c r="K48" s="1">
+        <v>46202</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>44</v>
+      </c>
+      <c r="B49">
+        <v>10005</v>
+      </c>
+      <c r="C49" t="s">
+        <v>18</v>
+      </c>
+      <c r="D49" t="s">
+        <v>10</v>
+      </c>
+      <c r="E49" t="s">
+        <v>11</v>
+      </c>
+      <c r="F49">
+        <v>-75</v>
+      </c>
+      <c r="G49">
+        <v>-1.5</v>
+      </c>
+      <c r="H49" t="s">
+        <v>75</v>
+      </c>
+      <c r="I49">
+        <v>50</v>
+      </c>
+      <c r="J49" t="s">
+        <v>17</v>
+      </c>
+      <c r="K49" s="1">
+        <v>46190</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>18</v>
+      </c>
+      <c r="B50">
+        <v>10003</v>
+      </c>
+      <c r="C50" t="s">
+        <v>18</v>
+      </c>
+      <c r="D50" t="s">
+        <v>10</v>
+      </c>
+      <c r="E50" t="s">
+        <v>14</v>
+      </c>
+      <c r="F50">
+        <v>-75</v>
+      </c>
+      <c r="G50">
+        <v>-1.5</v>
+      </c>
+      <c r="H50" t="s">
+        <v>75</v>
+      </c>
+      <c r="I50">
+        <v>50</v>
+      </c>
+      <c r="J50" t="s">
+        <v>17</v>
+      </c>
+      <c r="K50" s="1">
+        <v>46187</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>9</v>
+      </c>
+      <c r="B51">
+        <v>10006</v>
+      </c>
+      <c r="C51" t="s">
+        <v>18</v>
+      </c>
+      <c r="D51" t="s">
+        <v>10</v>
+      </c>
+      <c r="E51" t="s">
+        <v>11</v>
+      </c>
+      <c r="F51">
+        <v>-75</v>
+      </c>
+      <c r="G51">
+        <v>-1.5</v>
+      </c>
+      <c r="H51" t="s">
+        <v>75</v>
+      </c>
+      <c r="I51">
+        <v>50</v>
+      </c>
+      <c r="J51" t="s">
+        <v>17</v>
+      </c>
+      <c r="K51" s="1">
+        <v>46121</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>25</v>
+      </c>
+      <c r="B52">
+        <v>10003</v>
+      </c>
+      <c r="C52" t="s">
+        <v>18</v>
+      </c>
+      <c r="D52" t="s">
+        <v>10</v>
+      </c>
+      <c r="E52" t="s">
+        <v>14</v>
+      </c>
+      <c r="F52">
+        <v>-50</v>
+      </c>
+      <c r="G52">
+        <v>-0.5</v>
+      </c>
+      <c r="H52" t="s">
+        <v>75</v>
+      </c>
+      <c r="I52">
+        <v>100</v>
+      </c>
+      <c r="J52" t="s">
+        <v>17</v>
+      </c>
+      <c r="K52" s="1">
+        <v>46035</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>41</v>
+      </c>
+      <c r="B53">
+        <v>10003</v>
+      </c>
+      <c r="C53" t="s">
+        <v>18</v>
+      </c>
+      <c r="D53" t="s">
+        <v>10</v>
+      </c>
+      <c r="E53" t="s">
+        <v>14</v>
+      </c>
+      <c r="F53">
+        <v>100</v>
+      </c>
+      <c r="G53">
+        <v>1</v>
+      </c>
+      <c r="H53" t="s">
+        <v>75</v>
+      </c>
+      <c r="I53">
+        <v>100</v>
+      </c>
+      <c r="J53" t="s">
+        <v>12</v>
+      </c>
+      <c r="K53" s="1">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A54">
+        <v>60</v>
+      </c>
+      <c r="B54">
+        <v>10006</v>
+      </c>
+      <c r="C54" t="s">
+        <v>18</v>
+      </c>
+      <c r="D54" t="s">
+        <v>10</v>
+      </c>
+      <c r="E54" t="s">
+        <v>14</v>
+      </c>
+      <c r="F54">
+        <v>150</v>
+      </c>
+      <c r="G54">
+        <v>1.5</v>
+      </c>
+      <c r="H54" t="s">
+        <v>75</v>
+      </c>
+      <c r="I54">
+        <v>100</v>
+      </c>
+      <c r="J54" t="s">
+        <v>12</v>
+      </c>
+      <c r="K54" s="1">
+        <v>46158</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A55">
+        <v>28</v>
+      </c>
+      <c r="B55">
+        <v>10002</v>
+      </c>
+      <c r="C55" t="s">
+        <v>18</v>
+      </c>
+      <c r="D55" t="s">
+        <v>10</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55">
+        <v>250</v>
+      </c>
+      <c r="G55">
+        <v>2.5</v>
+      </c>
+      <c r="H55" t="s">
+        <v>74</v>
+      </c>
+      <c r="I55">
+        <v>100</v>
+      </c>
+      <c r="J55" t="s">
+        <v>12</v>
+      </c>
+      <c r="K55" s="1">
+        <v>46130</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A56">
+        <v>91</v>
+      </c>
+      <c r="B56">
+        <v>10003</v>
+      </c>
+      <c r="C56" t="s">
+        <v>18</v>
+      </c>
+      <c r="D56" t="s">
+        <v>10</v>
+      </c>
+      <c r="E56" t="s">
+        <v>14</v>
+      </c>
+      <c r="F56">
+        <v>300</v>
+      </c>
+      <c r="G56">
+        <v>1.5</v>
+      </c>
+      <c r="H56" t="s">
+        <v>75</v>
+      </c>
+      <c r="I56">
+        <v>200</v>
+      </c>
+      <c r="J56" t="s">
+        <v>12</v>
+      </c>
+      <c r="K56" s="1">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A57">
+        <v>90</v>
+      </c>
+      <c r="B57">
+        <v>10002</v>
+      </c>
+      <c r="C57" t="s">
+        <v>18</v>
+      </c>
+      <c r="D57" t="s">
+        <v>10</v>
+      </c>
+      <c r="E57" t="s">
+        <v>14</v>
+      </c>
+      <c r="F57">
+        <v>500</v>
+      </c>
+      <c r="G57">
+        <v>2.5</v>
+      </c>
+      <c r="H57" t="s">
+        <v>74</v>
+      </c>
+      <c r="I57">
+        <v>200</v>
+      </c>
+      <c r="J57" t="s">
+        <v>12</v>
+      </c>
+      <c r="K57" s="1">
+        <v>46076</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A00360D7-0D73-4CE4-AFB9-0AF5F61FAEDB}">
   <dimension ref="A3:D9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7.21875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.6640625" bestFit="1" customWidth="1"/>
@@ -3055,7 +5125,7 @@
   <sheetData>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B3" s="19" t="s">
         <v>72</v>
@@ -3079,56 +5149,56 @@
       <c r="A5" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="21">
-        <v>1975</v>
-      </c>
-      <c r="C5" s="21">
-        <v>925</v>
-      </c>
-      <c r="D5" s="21">
-        <v>2900</v>
+      <c r="B5" s="15">
+        <v>141.07142857142858</v>
+      </c>
+      <c r="C5" s="15">
+        <v>115.625</v>
+      </c>
+      <c r="D5" s="15">
+        <v>131.81818181818181</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="21">
-        <v>3075</v>
-      </c>
-      <c r="C6" s="21">
-        <v>3750</v>
-      </c>
-      <c r="D6" s="21">
-        <v>6825</v>
+      <c r="B6" s="15">
+        <v>219.64285714285714</v>
+      </c>
+      <c r="C6" s="15">
+        <v>197.36842105263159</v>
+      </c>
+      <c r="D6" s="15">
+        <v>206.81818181818181</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="21">
-        <v>1275</v>
-      </c>
-      <c r="C7" s="21">
-        <v>650</v>
-      </c>
-      <c r="D7" s="21">
-        <v>1925</v>
+      <c r="B7" s="15">
+        <v>85</v>
+      </c>
+      <c r="C7" s="15">
+        <v>54.166666666666664</v>
+      </c>
+      <c r="D7" s="15">
+        <v>71.296296296296291</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="21">
-        <v>125</v>
-      </c>
-      <c r="C8" s="21">
-        <v>450</v>
-      </c>
-      <c r="D8" s="21">
-        <v>575</v>
+      <c r="B8" s="15">
+        <v>9.615384615384615</v>
+      </c>
+      <c r="C8" s="15">
+        <v>90</v>
+      </c>
+      <c r="D8" s="15">
+        <v>31.944444444444443</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -3136,13 +5206,13 @@
         <v>71</v>
       </c>
       <c r="B9" s="21">
-        <v>6450</v>
+        <v>115.17857142857143</v>
       </c>
       <c r="C9" s="21">
-        <v>5775</v>
+        <v>131.25</v>
       </c>
       <c r="D9" s="21">
-        <v>12225</v>
+        <v>122.25</v>
       </c>
     </row>
   </sheetData>
@@ -3151,7 +5221,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{906658B5-1F80-4C49-9035-7A91F11B2092}">
   <dimension ref="A1:P101"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -6933,10 +9003,10 @@
     <mergeCell ref="N6:P6"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6946,7 +9016,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC7DF93-3E77-4DA9-9925-C234221B379B}">
   <dimension ref="B5:N30"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -7379,7 +9449,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDB00B21-86E3-4E60-9B16-646B4376A26A}">
   <dimension ref="F7:X25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
hanya dart column dyal resut bach kola session ta3tini win w loss dyalha bch na7sab win rate
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14F8A184-D81A-4108-B159-15FA5AEDE627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F30ECB3-FD03-4F2B-A88B-75DEAD6729DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
+    <workbookView xWindow="9324" yWindow="0" windowWidth="13812" windowHeight="12336" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="5" r:id="rId1"/>
@@ -80,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="797" uniqueCount="79">
   <si>
     <t>TradeID</t>
   </si>
@@ -298,6 +298,9 @@
     <t>Grand Total</t>
   </si>
   <si>
+    <t>Count of TradeID</t>
+  </si>
+  <si>
     <t>result column</t>
   </si>
   <si>
@@ -310,7 +313,10 @@
     <t>REVIEW</t>
   </si>
   <si>
-    <t>Average of Profit</t>
+    <t>London Total</t>
+  </si>
+  <si>
+    <t>New York Total</t>
   </si>
 </sst>
 </file>
@@ -830,7 +836,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -862,6 +868,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -908,12 +915,30 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="25">
     <dxf>
-      <numFmt numFmtId="168" formatCode="0.000"/>
+      <numFmt numFmtId="169" formatCode="0.0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="168" formatCode="0.000"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="167" formatCode="0.0000"/>
@@ -2438,9 +2463,9 @@
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2DA79A61-38FD-45EA-A18C-EAC9CD91845A}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="session rows" colHeaderCaption="result column">
-  <location ref="A3:D9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <location ref="A3:H10" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="11">
-    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
       <items count="5">
@@ -2459,11 +2484,11 @@
       </items>
     </pivotField>
     <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
       <items count="3">
         <item x="1"/>
         <item x="0"/>
@@ -2574,14 +2599,29 @@
       <x/>
     </i>
   </rowItems>
-  <colFields count="1">
+  <colFields count="2">
     <field x="3"/>
+    <field x="9"/>
   </colFields>
-  <colItems count="3">
+  <colItems count="7">
     <i>
+      <x/>
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i t="default">
       <x/>
     </i>
     <i>
+      <x v="1"/>
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i t="default">
       <x v="1"/>
     </i>
     <i t="grand">
@@ -2589,7 +2629,7 @@
     </i>
   </colItems>
   <dataFields count="1">
-    <dataField name="Average of Profit" fld="5" subtotal="average" baseField="2" baseItem="1"/>
+    <dataField name="Count of TradeID" fld="0" subtotal="count" baseField="2" baseItem="1"/>
   </dataFields>
   <formats count="1">
     <format dxfId="1">
@@ -2688,7 +2728,7 @@
     <tableColumn id="8" xr3:uid="{011760A3-A9D1-4015-8D75-7EFE2A2FEB20}" name="Risk Status"/>
     <tableColumn id="9" xr3:uid="{8E6DF200-182D-483A-8ED0-12101EFECD0F}" name="Profit per R"/>
     <tableColumn id="10" xr3:uid="{BB6361CF-CAA7-4423-9C5D-82E0E0F6DBCD}" name="Result"/>
-    <tableColumn id="11" xr3:uid="{420DB1BF-4073-4932-87BC-11D2FECAB843}" name="TradeDate" dataDxfId="5"/>
+    <tableColumn id="11" xr3:uid="{420DB1BF-4073-4932-87BC-11D2FECAB843}" name="TradeDate" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2708,14 +2748,14 @@
     <tableColumn id="5" xr3:uid="{539426CC-F875-4D64-977A-05C6F1BCDBCD}" name="Direction"/>
     <tableColumn id="6" xr3:uid="{BFF7C4D2-29D9-4645-98DB-6FBF609AB80F}" name="Profit"/>
     <tableColumn id="7" xr3:uid="{CD8DBAA1-576E-4991-87E5-049F5C232A1F}" name="R"/>
-    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="18">
+    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="24">
       <calculatedColumnFormula>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="17">
+    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="23">
       <calculatedColumnFormula>IFERROR(Table1[[#This Row],[Profit]]/Table1[[#This Row],[R]],"0")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{CC96218F-2F0A-46BB-98E4-8AE8218DB3D7}" name="Result"/>
-    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="16"/>
+    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2727,10 +2767,10 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{DAF88BD0-F115-4C64-AE11-7DD8AB7505A7}" name="Pair"/>
     <tableColumn id="2" xr3:uid="{89E35073-D474-496E-86E0-7646DF314B64}" name="Profit"/>
-    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="15">
+    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="21">
       <calculatedColumnFormula>TRIM(Table2[[#This Row],[Pair]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="14">
+    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="20">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Pair]]=Table2[[#This Row],[Clean Space]],"GOOD","NADFO")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2743,7 +2783,7 @@
   <autoFilter ref="K8:L12" xr:uid="{A99A2C5F-61E0-444B-907C-487860A13E40}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{0A321640-D79C-4135-83F6-E38913427047}" name="raw text"/>
-    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="13">
+    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="19">
       <calculatedColumnFormula>PROPER(Table4[[#This Row],[raw text]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2756,10 +2796,10 @@
   <autoFilter ref="K16:M19" xr:uid="{4576F3CB-3E9B-40EE-B5BA-0228DC3EBD7C}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{3D4EC290-099D-468C-B78D-8A8F427D8214}" name="text num"/>
-    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="12">
+    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="18">
       <calculatedColumnFormula>VALUE(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="11">
+    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="17">
       <calculatedColumnFormula>ISNUMBER(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2768,10 +2808,10 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}" name="Table5" displayName="Table5" ref="Q17:Q25" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}" name="Table5" displayName="Table5" ref="Q17:Q25" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <autoFilter ref="Q17:Q25" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{B868BDD4-CA52-440D-A1EA-1585934AF042}" name="TradeID" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{B868BDD4-CA52-440D-A1EA-1585934AF042}" name="TradeID" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3164,7 +3204,7 @@
         <v>2</v>
       </c>
       <c r="H2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I2">
         <v>250</v>
@@ -3199,7 +3239,7 @@
         <v>2</v>
       </c>
       <c r="H3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I3">
         <v>250</v>
@@ -3234,7 +3274,7 @@
         <v>1.5</v>
       </c>
       <c r="H4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I4">
         <v>250</v>
@@ -3269,7 +3309,7 @@
         <v>1.5</v>
       </c>
       <c r="H5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I5">
         <v>250</v>
@@ -3304,7 +3344,7 @@
         <v>2</v>
       </c>
       <c r="H6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I6">
         <v>100</v>
@@ -3339,7 +3379,7 @@
         <v>2</v>
       </c>
       <c r="H7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I7">
         <v>100</v>
@@ -3374,7 +3414,7 @@
         <v>2.5</v>
       </c>
       <c r="H8" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I8">
         <v>50</v>
@@ -3409,7 +3449,7 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I9">
         <v>100</v>
@@ -3444,7 +3484,7 @@
         <v>1</v>
       </c>
       <c r="H10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I10">
         <v>50</v>
@@ -3479,7 +3519,7 @@
         <v>-0.5</v>
       </c>
       <c r="H11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I11">
         <v>50</v>
@@ -3514,7 +3554,7 @@
         <v>-0.5</v>
       </c>
       <c r="H12" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I12">
         <v>100</v>
@@ -3549,7 +3589,7 @@
         <v>-1</v>
       </c>
       <c r="H13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I13">
         <v>100</v>
@@ -3584,7 +3624,7 @@
         <v>-0.5</v>
       </c>
       <c r="H14" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I14">
         <v>250</v>
@@ -3619,7 +3659,7 @@
         <v>-1.5</v>
       </c>
       <c r="H15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I15">
         <v>100</v>
@@ -3654,7 +3694,7 @@
         <v>3</v>
       </c>
       <c r="H16" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I16">
         <v>250</v>
@@ -3689,7 +3729,7 @@
         <v>3</v>
       </c>
       <c r="H17" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I17">
         <v>250</v>
@@ -3724,7 +3764,7 @@
         <v>2.5</v>
       </c>
       <c r="H18" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I18">
         <v>250</v>
@@ -3759,7 +3799,7 @@
         <v>1.5</v>
       </c>
       <c r="H19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I19">
         <v>250</v>
@@ -3794,7 +3834,7 @@
         <v>3</v>
       </c>
       <c r="H20" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I20">
         <v>100</v>
@@ -3829,7 +3869,7 @@
         <v>3</v>
       </c>
       <c r="H21" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I21">
         <v>100</v>
@@ -3864,7 +3904,7 @@
         <v>1</v>
       </c>
       <c r="H22" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I22">
         <v>250</v>
@@ -3899,7 +3939,7 @@
         <v>2</v>
       </c>
       <c r="H23" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I23">
         <v>50</v>
@@ -3934,7 +3974,7 @@
         <v>1</v>
       </c>
       <c r="H24" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I24">
         <v>100</v>
@@ -3969,7 +4009,7 @@
         <v>-0.5</v>
       </c>
       <c r="H25" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I25">
         <v>50</v>
@@ -4004,7 +4044,7 @@
         <v>-0.5</v>
       </c>
       <c r="H26" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I26">
         <v>100</v>
@@ -4039,7 +4079,7 @@
         <v>-0.5</v>
       </c>
       <c r="H27" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I27">
         <v>100</v>
@@ -4074,7 +4114,7 @@
         <v>-1</v>
       </c>
       <c r="H28" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I28">
         <v>50</v>
@@ -4109,7 +4149,7 @@
         <v>-1.5</v>
       </c>
       <c r="H29" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I29">
         <v>200</v>
@@ -4144,7 +4184,7 @@
         <v>-1.5</v>
       </c>
       <c r="H30" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I30">
         <v>250</v>
@@ -4179,7 +4219,7 @@
         <v>-0.5</v>
       </c>
       <c r="H31" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I31">
         <v>250</v>
@@ -4214,7 +4254,7 @@
         <v>-1</v>
       </c>
       <c r="H32" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I32">
         <v>100</v>
@@ -4249,7 +4289,7 @@
         <v>-1</v>
       </c>
       <c r="H33" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I33">
         <v>100</v>
@@ -4284,7 +4324,7 @@
         <v>-1.5</v>
       </c>
       <c r="H34" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I34">
         <v>50</v>
@@ -4319,7 +4359,7 @@
         <v>1</v>
       </c>
       <c r="H35" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I35">
         <v>50</v>
@@ -4354,7 +4394,7 @@
         <v>1</v>
       </c>
       <c r="H36" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I36">
         <v>50</v>
@@ -4389,7 +4429,7 @@
         <v>3</v>
       </c>
       <c r="H37" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I37">
         <v>50</v>
@@ -4424,7 +4464,7 @@
         <v>3</v>
       </c>
       <c r="H38" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I38">
         <v>50</v>
@@ -4459,7 +4499,7 @@
         <v>2</v>
       </c>
       <c r="H39" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I39">
         <v>100</v>
@@ -4494,7 +4534,7 @@
         <v>1</v>
       </c>
       <c r="H40" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I40">
         <v>200</v>
@@ -4529,7 +4569,7 @@
         <v>1</v>
       </c>
       <c r="H41" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I41">
         <v>200</v>
@@ -4564,7 +4604,7 @@
         <v>1</v>
       </c>
       <c r="H42" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I42">
         <v>250</v>
@@ -4599,7 +4639,7 @@
         <v>1.5</v>
       </c>
       <c r="H43" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I43">
         <v>200</v>
@@ -4634,7 +4674,7 @@
         <v>2.5</v>
       </c>
       <c r="H44" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I44">
         <v>200</v>
@@ -4669,7 +4709,7 @@
         <v>-1</v>
       </c>
       <c r="H45" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I45">
         <v>250</v>
@@ -4704,7 +4744,7 @@
         <v>-1</v>
       </c>
       <c r="H46" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I46">
         <v>250</v>
@@ -4739,7 +4779,7 @@
         <v>-1</v>
       </c>
       <c r="H47" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I47">
         <v>200</v>
@@ -4774,7 +4814,7 @@
         <v>-1</v>
       </c>
       <c r="H48" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I48">
         <v>200</v>
@@ -4809,7 +4849,7 @@
         <v>-1.5</v>
       </c>
       <c r="H49" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I49">
         <v>50</v>
@@ -4844,7 +4884,7 @@
         <v>-1.5</v>
       </c>
       <c r="H50" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I50">
         <v>50</v>
@@ -4879,7 +4919,7 @@
         <v>-1.5</v>
       </c>
       <c r="H51" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I51">
         <v>50</v>
@@ -4914,7 +4954,7 @@
         <v>-0.5</v>
       </c>
       <c r="H52" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I52">
         <v>100</v>
@@ -4949,7 +4989,7 @@
         <v>1</v>
       </c>
       <c r="H53" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I53">
         <v>100</v>
@@ -4984,7 +5024,7 @@
         <v>1.5</v>
       </c>
       <c r="H54" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I54">
         <v>100</v>
@@ -5019,7 +5059,7 @@
         <v>2.5</v>
       </c>
       <c r="H55" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I55">
         <v>100</v>
@@ -5054,7 +5094,7 @@
         <v>1.5</v>
       </c>
       <c r="H56" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I56">
         <v>200</v>
@@ -5089,7 +5129,7 @@
         <v>2.5</v>
       </c>
       <c r="H57" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I57">
         <v>200</v>
@@ -5111,108 +5151,189 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A00360D7-0D73-4CE4-AFB9-0AF5F61FAEDB}">
-  <dimension ref="A3:D9"/>
+  <dimension ref="A3:H10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="19" t="s">
         <v>73</v>
       </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>10</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E4" t="s">
         <v>16</v>
       </c>
-      <c r="D4" t="s">
+      <c r="G4" t="s">
+        <v>78</v>
+      </c>
+      <c r="H4" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="20" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="15">
-        <v>141.07142857142858</v>
-      </c>
-      <c r="C5" s="15">
-        <v>115.625</v>
-      </c>
-      <c r="D5" s="15">
-        <v>131.81818181818181</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="20" t="s">
+      <c r="B6" s="23">
+        <v>5</v>
+      </c>
+      <c r="C6" s="23">
+        <v>9</v>
+      </c>
+      <c r="D6" s="23">
+        <v>14</v>
+      </c>
+      <c r="E6" s="23">
+        <v>5</v>
+      </c>
+      <c r="F6" s="23">
+        <v>3</v>
+      </c>
+      <c r="G6" s="23">
+        <v>8</v>
+      </c>
+      <c r="H6" s="23">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="15">
-        <v>219.64285714285714</v>
-      </c>
-      <c r="C6" s="15">
-        <v>197.36842105263159</v>
-      </c>
-      <c r="D6" s="15">
-        <v>206.81818181818181</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="20" t="s">
+      <c r="B7" s="23">
+        <v>5</v>
+      </c>
+      <c r="C7" s="23">
+        <v>9</v>
+      </c>
+      <c r="D7" s="23">
+        <v>14</v>
+      </c>
+      <c r="E7" s="23">
+        <v>5</v>
+      </c>
+      <c r="F7" s="23">
+        <v>14</v>
+      </c>
+      <c r="G7" s="23">
+        <v>19</v>
+      </c>
+      <c r="H7" s="23">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="15">
-        <v>85</v>
-      </c>
-      <c r="C7" s="15">
-        <v>54.166666666666664</v>
-      </c>
-      <c r="D7" s="15">
-        <v>71.296296296296291</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="20" t="s">
+      <c r="B8" s="23">
+        <v>5</v>
+      </c>
+      <c r="C8" s="23">
+        <v>10</v>
+      </c>
+      <c r="D8" s="23">
+        <v>15</v>
+      </c>
+      <c r="E8" s="23">
+        <v>6</v>
+      </c>
+      <c r="F8" s="23">
+        <v>6</v>
+      </c>
+      <c r="G8" s="23">
+        <v>12</v>
+      </c>
+      <c r="H8" s="23">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="15">
-        <v>9.615384615384615</v>
-      </c>
-      <c r="C8" s="15">
-        <v>90</v>
-      </c>
-      <c r="D8" s="15">
-        <v>31.944444444444443</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="20" t="s">
+      <c r="B9" s="23">
+        <v>8</v>
+      </c>
+      <c r="C9" s="23">
+        <v>5</v>
+      </c>
+      <c r="D9" s="23">
+        <v>13</v>
+      </c>
+      <c r="E9" s="23">
+        <v>2</v>
+      </c>
+      <c r="F9" s="23">
+        <v>3</v>
+      </c>
+      <c r="G9" s="23">
+        <v>5</v>
+      </c>
+      <c r="H9" s="23">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="B9" s="21">
-        <v>115.17857142857143</v>
-      </c>
-      <c r="C9" s="21">
-        <v>131.25</v>
-      </c>
-      <c r="D9" s="21">
-        <v>122.25</v>
+      <c r="B10" s="21">
+        <v>23</v>
+      </c>
+      <c r="C10" s="21">
+        <v>33</v>
+      </c>
+      <c r="D10" s="21">
+        <v>56</v>
+      </c>
+      <c r="E10" s="21">
+        <v>18</v>
+      </c>
+      <c r="F10" s="21">
+        <v>26</v>
+      </c>
+      <c r="G10" s="21">
+        <v>44</v>
+      </c>
+      <c r="H10" s="21">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -9003,10 +9124,10 @@
     <mergeCell ref="N6:P6"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="7" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="6" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
hnaya adt chart pivot
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F30ECB3-FD03-4F2B-A88B-75DEAD6729DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADD6BDFA-A858-4534-82D6-E5556A2C4FA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9324" yWindow="0" windowWidth="13812" windowHeight="12336" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="5" r:id="rId1"/>
@@ -915,7 +915,31 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="25">
+  <dxfs count="33">
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="169" formatCode="0.0"/>
     </dxf>
@@ -1016,6 +1040,1578 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="106"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="6"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:pivotSource>
+    <c:name>[trading_raw_data-main.xlsx]pivot table!PivotTable1</c:name>
+    <c:fmtId val="0"/>
+  </c:pivotSource>
+  <c:chart>
+    <c:autoTitleDeleted val="0"/>
+    <c:pivotFmts>
+      <c:pivotFmt>
+        <c:idx val="0"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="circle"/>
+          <c:size val="8"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent4">
+                <a:tint val="58000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:solidFill>
+                    <a:srgbClr val="00B0F0"/>
+                  </a:solidFill>
+                  <a:effectLst>
+                    <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="000000">
+                        <a:alpha val="43137"/>
+                      </a:srgbClr>
+                    </a:outerShdw>
+                  </a:effectLst>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="1"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent3">
+              <a:lumMod val="60000"/>
+              <a:lumOff val="40000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="circle"/>
+          <c:size val="8"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent4">
+                <a:tint val="86000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:solidFill>
+                    <a:srgbClr val="00B0F0"/>
+                  </a:solidFill>
+                  <a:effectLst>
+                    <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="000000">
+                        <a:alpha val="43137"/>
+                      </a:srgbClr>
+                    </a:outerShdw>
+                  </a:effectLst>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="2"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="circle"/>
+          <c:size val="8"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent4">
+                <a:shade val="86000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:solidFill>
+                    <a:srgbClr val="00B0F0"/>
+                  </a:solidFill>
+                  <a:effectLst>
+                    <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="000000">
+                        <a:alpha val="43137"/>
+                      </a:srgbClr>
+                    </a:outerShdw>
+                  </a:effectLst>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="3"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent3">
+              <a:lumMod val="60000"/>
+              <a:lumOff val="40000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:marker>
+          <c:symbol val="circle"/>
+          <c:size val="8"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent4">
+                <a:shade val="58000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                  <a:solidFill>
+                    <a:srgbClr val="00B0F0"/>
+                  </a:solidFill>
+                  <a:effectLst>
+                    <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
+                      <a:srgbClr val="000000">
+                        <a:alpha val="43137"/>
+                      </a:srgbClr>
+                    </a:outerShdw>
+                  </a:effectLst>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+    </c:pivotFmts>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'pivot table'!$B$3:$B$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>London - Loss</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:ln>
+                      <a:noFill/>
+                    </a:ln>
+                    <a:solidFill>
+                      <a:srgbClr val="00B0F0"/>
+                    </a:solidFill>
+                    <a:effectLst>
+                      <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
+                        <a:srgbClr val="000000">
+                          <a:alpha val="43137"/>
+                        </a:srgbClr>
+                      </a:outerShdw>
+                    </a:effectLst>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'pivot table'!$A$6:$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>EURUSD</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>GBPUSD</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>US30</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>XAUUSD</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'pivot table'!$B$6:$B$10</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-0375-4A3D-B9BB-59EE074CEEA9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'pivot table'!$C$3:$C$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>London - Win</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3">
+                <a:lumMod val="60000"/>
+                <a:lumOff val="40000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:ln>
+                      <a:noFill/>
+                    </a:ln>
+                    <a:solidFill>
+                      <a:srgbClr val="00B0F0"/>
+                    </a:solidFill>
+                    <a:effectLst>
+                      <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
+                        <a:srgbClr val="000000">
+                          <a:alpha val="43137"/>
+                        </a:srgbClr>
+                      </a:outerShdw>
+                    </a:effectLst>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'pivot table'!$A$6:$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>EURUSD</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>GBPUSD</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>US30</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>XAUUSD</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'pivot table'!$C$6:$C$10</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-0375-4A3D-B9BB-59EE074CEEA9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'pivot table'!$E$3:$E$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>New York - Loss</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="FF0000"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:delete val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'pivot table'!$A$6:$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>EURUSD</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>GBPUSD</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>US30</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>XAUUSD</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'pivot table'!$E$6:$E$10</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000007-0375-4A3D-B9BB-59EE074CEEA9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'pivot table'!$F$3:$F$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>New York - Win</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3">
+                <a:lumMod val="60000"/>
+                <a:lumOff val="40000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:delete val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'pivot table'!$A$6:$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>EURUSD</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>GBPUSD</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>US30</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>XAUUSD</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'pivot table'!$F$6:$F$10</c:f>
+              <c:numCache>
+                <c:formatCode>0</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000008-0375-4A3D-B9BB-59EE074CEEA9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="199"/>
+        <c:axId val="310799823"/>
+        <c:axId val="310801263"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="310799823"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0">
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="00B0F0"/>
+                </a:solidFill>
+                <a:effectLst>
+                  <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
+                    <a:srgbClr val="000000">
+                      <a:alpha val="43137"/>
+                    </a:srgbClr>
+                  </a:outerShdw>
+                </a:effectLst>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="310801263"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="310801263"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="0" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="00B0F0"/>
+                </a:solidFill>
+                <a:effectLst>
+                  <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
+                    <a:srgbClr val="000000">
+                      <a:alpha val="43137"/>
+                    </a:srgbClr>
+                  </a:outerShdw>
+                </a:effectLst>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="310799823"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="25400">
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:solidFill>
+                <a:srgbClr val="00B0F0"/>
+              </a:solidFill>
+              <a:effectLst>
+                <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
+                  <a:srgbClr val="000000">
+                    <a:alpha val="43137"/>
+                  </a:srgbClr>
+                </a:outerShdw>
+              </a:effectLst>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst>
+      <a:glow rad="381000">
+        <a:schemeClr val="accent1">
+          <a:alpha val="16000"/>
+        </a:schemeClr>
+      </a:glow>
+      <a:outerShdw blurRad="546100" dir="21540000" algn="t" rotWithShape="0">
+        <a:schemeClr val="accent6">
+          <a:lumMod val="75000"/>
+          <a:alpha val="40000"/>
+        </a:schemeClr>
+      </a:outerShdw>
+      <a:softEdge rad="0"/>
+    </a:effectLst>
+    <a:scene3d>
+      <a:camera prst="orthographicFront"/>
+      <a:lightRig rig="threePt" dir="t">
+        <a:rot lat="0" lon="0" rev="12000000"/>
+      </a:lightRig>
+    </a:scene3d>
+    <a:sp3d prstMaterial="dkEdge">
+      <a:bevelT w="165100" prst="coolSlant"/>
+    </a:sp3d>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:solidFill>
+            <a:srgbClr val="00B0F0"/>
+          </a:solidFill>
+          <a:effectLst>
+            <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="43137"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:defRPr>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:extLst>
+    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
+      <c14:pivotOptions>
+        <c14:dropZoneFilter val="1"/>
+        <c14:dropZoneCategories val="1"/>
+        <c14:dropZoneData val="1"/>
+        <c14:dropZoneSeries val="1"/>
+        <c14:dropZonesVisible val="1"/>
+      </c14:pivotOptions>
+    </c:ext>
+    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
+      <c16:pivotOptions16>
+        <c16:showExpandCollapseFieldButtons val="1"/>
+      </c16:pivotOptions16>
+    </c:ext>
+  </c:extLst>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinearReversed" id="24">
+  <a:schemeClr val="accent4"/>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="212">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200" cap="all"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" b="0" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="38100" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="8"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:prstDash val="dash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="major">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="2000" b="0" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>75508</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>41564</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>699654</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>55418</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{633DD137-88C9-F68F-6DBE-95146FAF6680}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2462,7 +4058,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2DA79A61-38FD-45EA-A18C-EAC9CD91845A}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="session rows" colHeaderCaption="result column">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2DA79A61-38FD-45EA-A18C-EAC9CD91845A}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7" rowHeaderCaption="session rows" colHeaderCaption="result column">
   <location ref="A3:H10" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField dataField="1" showAll="0"/>
@@ -2632,7 +4228,7 @@
     <dataField name="Count of TradeID" fld="0" subtotal="count" baseField="2" baseItem="1"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="1">
+    <format dxfId="9">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="0"/>
@@ -2640,6 +4236,68 @@
       </pivotArea>
     </format>
   </formats>
+  <chartFormats count="4">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="3">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="3" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="9" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="3">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="3" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="9" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="3">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="3" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="9" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="0" format="3" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="3">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="3" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="9" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -2728,7 +4386,7 @@
     <tableColumn id="8" xr3:uid="{011760A3-A9D1-4015-8D75-7EFE2A2FEB20}" name="Risk Status"/>
     <tableColumn id="9" xr3:uid="{8E6DF200-182D-483A-8ED0-12101EFECD0F}" name="Profit per R"/>
     <tableColumn id="10" xr3:uid="{BB6361CF-CAA7-4423-9C5D-82E0E0F6DBCD}" name="Result"/>
-    <tableColumn id="11" xr3:uid="{420DB1BF-4073-4932-87BC-11D2FECAB843}" name="TradeDate" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{420DB1BF-4073-4932-87BC-11D2FECAB843}" name="TradeDate" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2748,14 +4406,14 @@
     <tableColumn id="5" xr3:uid="{539426CC-F875-4D64-977A-05C6F1BCDBCD}" name="Direction"/>
     <tableColumn id="6" xr3:uid="{BFF7C4D2-29D9-4645-98DB-6FBF609AB80F}" name="Profit"/>
     <tableColumn id="7" xr3:uid="{CD8DBAA1-576E-4991-87E5-049F5C232A1F}" name="R"/>
-    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="24">
+    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="32">
       <calculatedColumnFormula>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="23">
+    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="31">
       <calculatedColumnFormula>IFERROR(Table1[[#This Row],[Profit]]/Table1[[#This Row],[R]],"0")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{CC96218F-2F0A-46BB-98E4-8AE8218DB3D7}" name="Result"/>
-    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="30"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2767,10 +4425,10 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{DAF88BD0-F115-4C64-AE11-7DD8AB7505A7}" name="Pair"/>
     <tableColumn id="2" xr3:uid="{89E35073-D474-496E-86E0-7646DF314B64}" name="Profit"/>
-    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="21">
+    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="29">
       <calculatedColumnFormula>TRIM(Table2[[#This Row],[Pair]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="20">
+    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="28">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Pair]]=Table2[[#This Row],[Clean Space]],"GOOD","NADFO")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2783,7 +4441,7 @@
   <autoFilter ref="K8:L12" xr:uid="{A99A2C5F-61E0-444B-907C-487860A13E40}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{0A321640-D79C-4135-83F6-E38913427047}" name="raw text"/>
-    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="19">
+    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="27">
       <calculatedColumnFormula>PROPER(Table4[[#This Row],[raw text]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2796,10 +4454,10 @@
   <autoFilter ref="K16:M19" xr:uid="{4576F3CB-3E9B-40EE-B5BA-0228DC3EBD7C}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{3D4EC290-099D-468C-B78D-8A8F427D8214}" name="text num"/>
-    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="18">
+    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="26">
       <calculatedColumnFormula>VALUE(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="17">
+    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="25">
       <calculatedColumnFormula>ISNUMBER(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2808,10 +4466,10 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}" name="Table5" displayName="Table5" ref="Q17:Q25" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}" name="Table5" displayName="Table5" ref="Q17:Q25" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
   <autoFilter ref="Q17:Q25" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{B868BDD4-CA52-440D-A1EA-1585934AF042}" name="TradeID" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{B868BDD4-CA52-440D-A1EA-1585934AF042}" name="TradeID" dataDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5156,10 +6814,10 @@
   <cols>
     <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.21875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -5339,6 +6997,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -9124,10 +10783,10 @@
     <mergeCell ref="N6:P6"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="13" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="12" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
hanaya khdit data man pivot w7atithom f data analysis table
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADD6BDFA-A858-4534-82D6-E5556A2C4FA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8152FD41-AF95-4D72-98B6-7D9170B84CA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="2" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="5" r:id="rId1"/>
     <sheet name="pivot table" sheetId="4" r:id="rId2"/>
-    <sheet name="trading_raw_data2" sheetId="1" r:id="rId3"/>
-    <sheet name="data analysis" sheetId="2" r:id="rId4"/>
+    <sheet name="data analysis" sheetId="2" r:id="rId3"/>
+    <sheet name="trading_raw_data2" sheetId="1" r:id="rId4"/>
     <sheet name="data cleaning " sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -80,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="797" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="804" uniqueCount="81">
   <si>
     <t>TradeID</t>
   </si>
@@ -317,6 +317,12 @@
   </si>
   <si>
     <t>New York Total</t>
+  </si>
+  <si>
+    <t>LONDON WIN RATE</t>
+  </si>
+  <si>
+    <t>NEW YORK WIN RATE</t>
   </si>
 </sst>
 </file>
@@ -865,10 +871,10 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -915,67 +921,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="33">
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="169" formatCode="0.0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="168" formatCode="0.000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="167" formatCode="0.0000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="166" formatCode="0.00000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.000000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
+  <dxfs count="15">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1029,6 +975,12 @@
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1040,1578 +992,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="106"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="6"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:pivotSource>
-    <c:name>[trading_raw_data-main.xlsx]pivot table!PivotTable1</c:name>
-    <c:fmtId val="0"/>
-  </c:pivotSource>
-  <c:chart>
-    <c:autoTitleDeleted val="0"/>
-    <c:pivotFmts>
-      <c:pivotFmt>
-        <c:idx val="0"/>
-        <c:spPr>
-          <a:solidFill>
-            <a:srgbClr val="FF0000"/>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="8"/>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent4">
-                <a:tint val="58000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:marker>
-        <c:dLbl>
-          <c:idx val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                  <a:solidFill>
-                    <a:srgbClr val="00B0F0"/>
-                  </a:solidFill>
-                  <a:effectLst>
-                    <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
-                      <a:srgbClr val="000000">
-                        <a:alpha val="43137"/>
-                      </a:srgbClr>
-                    </a:outerShdw>
-                  </a:effectLst>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-          <c:dLblPos val="outEnd"/>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
-          </c:extLst>
-        </c:dLbl>
-      </c:pivotFmt>
-      <c:pivotFmt>
-        <c:idx val="1"/>
-        <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent3">
-              <a:lumMod val="60000"/>
-              <a:lumOff val="40000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="8"/>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent4">
-                <a:tint val="86000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:marker>
-        <c:dLbl>
-          <c:idx val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                  <a:solidFill>
-                    <a:srgbClr val="00B0F0"/>
-                  </a:solidFill>
-                  <a:effectLst>
-                    <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
-                      <a:srgbClr val="000000">
-                        <a:alpha val="43137"/>
-                      </a:srgbClr>
-                    </a:outerShdw>
-                  </a:effectLst>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-          <c:dLblPos val="outEnd"/>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
-          </c:extLst>
-        </c:dLbl>
-      </c:pivotFmt>
-      <c:pivotFmt>
-        <c:idx val="2"/>
-        <c:spPr>
-          <a:solidFill>
-            <a:srgbClr val="FF0000"/>
-          </a:solidFill>
-          <a:ln>
-            <a:solidFill>
-              <a:srgbClr val="FF0000"/>
-            </a:solidFill>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="8"/>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent4">
-                <a:shade val="86000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:marker>
-        <c:dLbl>
-          <c:idx val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                  <a:solidFill>
-                    <a:srgbClr val="00B0F0"/>
-                  </a:solidFill>
-                  <a:effectLst>
-                    <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
-                      <a:srgbClr val="000000">
-                        <a:alpha val="43137"/>
-                      </a:srgbClr>
-                    </a:outerShdw>
-                  </a:effectLst>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
-          </c:extLst>
-        </c:dLbl>
-      </c:pivotFmt>
-      <c:pivotFmt>
-        <c:idx val="3"/>
-        <c:spPr>
-          <a:solidFill>
-            <a:schemeClr val="accent3">
-              <a:lumMod val="60000"/>
-              <a:lumOff val="40000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="8"/>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent4">
-                <a:shade val="58000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:marker>
-        <c:dLbl>
-          <c:idx val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                  <a:solidFill>
-                    <a:srgbClr val="00B0F0"/>
-                  </a:solidFill>
-                  <a:effectLst>
-                    <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
-                      <a:srgbClr val="000000">
-                        <a:alpha val="43137"/>
-                      </a:srgbClr>
-                    </a:outerShdw>
-                  </a:effectLst>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
-          </c:extLst>
-        </c:dLbl>
-      </c:pivotFmt>
-    </c:pivotFmts>
-    <c:plotArea>
-      <c:layout/>
-      <c:barChart>
-        <c:barDir val="col"/>
-        <c:grouping val="clustered"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'pivot table'!$B$3:$B$5</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>London - Loss</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="FF0000"/>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:ln>
-                      <a:noFill/>
-                    </a:ln>
-                    <a:solidFill>
-                      <a:srgbClr val="00B0F0"/>
-                    </a:solidFill>
-                    <a:effectLst>
-                      <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
-                        <a:srgbClr val="000000">
-                          <a:alpha val="43137"/>
-                        </a:srgbClr>
-                      </a:outerShdw>
-                    </a:effectLst>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
-              </c:ext>
-            </c:extLst>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>'pivot table'!$A$6:$A$10</c:f>
-              <c:strCache>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>EURUSD</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>GBPUSD</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>US30</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>XAUUSD</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'pivot table'!$B$6:$B$10</c:f>
-              <c:numCache>
-                <c:formatCode>0</c:formatCode>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>8</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-0375-4A3D-B9BB-59EE074CEEA9}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'pivot table'!$C$3:$C$5</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>London - Win</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent3">
-                <a:lumMod val="60000"/>
-                <a:lumOff val="40000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:spPr>
-              <a:noFill/>
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:txPr>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
-                <a:spAutoFit/>
-              </a:bodyPr>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:ln>
-                      <a:noFill/>
-                    </a:ln>
-                    <a:solidFill>
-                      <a:srgbClr val="00B0F0"/>
-                    </a:solidFill>
-                    <a:effectLst>
-                      <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
-                        <a:srgbClr val="000000">
-                          <a:alpha val="43137"/>
-                        </a:srgbClr>
-                      </a:outerShdw>
-                    </a:effectLst>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:endParaRPr lang="en-US"/>
-              </a:p>
-            </c:txPr>
-            <c:dLblPos val="outEnd"/>
-            <c:showLegendKey val="0"/>
-            <c:showVal val="1"/>
-            <c:showCatName val="0"/>
-            <c:showSerName val="0"/>
-            <c:showPercent val="0"/>
-            <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="0"/>
-            <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:showLeaderLines val="1"/>
-                <c15:leaderLines>
-                  <c:spPr>
-                    <a:ln w="9525">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="35000"/>
-                          <a:lumOff val="65000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                    </a:ln>
-                    <a:effectLst/>
-                  </c:spPr>
-                </c15:leaderLines>
-              </c:ext>
-            </c:extLst>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>'pivot table'!$A$6:$A$10</c:f>
-              <c:strCache>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>EURUSD</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>GBPUSD</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>US30</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>XAUUSD</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'pivot table'!$C$6:$C$10</c:f>
-              <c:numCache>
-                <c:formatCode>0</c:formatCode>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>5</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-0375-4A3D-B9BB-59EE074CEEA9}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'pivot table'!$E$3:$E$5</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>New York - Loss</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:srgbClr val="FF0000"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:delete val="1"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>'pivot table'!$A$6:$A$10</c:f>
-              <c:strCache>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>EURUSD</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>GBPUSD</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>US30</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>XAUUSD</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'pivot table'!$E$6:$E$10</c:f>
-              <c:numCache>
-                <c:formatCode>0</c:formatCode>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>6</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>2</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000007-0375-4A3D-B9BB-59EE074CEEA9}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="3"/>
-          <c:order val="3"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>'pivot table'!$F$3:$F$5</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>New York - Win</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent3">
-                <a:lumMod val="60000"/>
-                <a:lumOff val="40000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:invertIfNegative val="0"/>
-          <c:dLbls>
-            <c:delete val="1"/>
-          </c:dLbls>
-          <c:cat>
-            <c:strRef>
-              <c:f>'pivot table'!$A$6:$A$10</c:f>
-              <c:strCache>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>EURUSD</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>GBPUSD</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>US30</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>XAUUSD</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>'pivot table'!$F$6:$F$10</c:f>
-              <c:numCache>
-                <c:formatCode>0</c:formatCode>
-                <c:ptCount val="4"/>
-                <c:pt idx="0">
-                  <c:v>3</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>14</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>6</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000008-0375-4A3D-B9BB-59EE074CEEA9}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:dLblPos val="outEnd"/>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="1"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:gapWidth val="199"/>
-        <c:axId val="310799823"/>
-        <c:axId val="310801263"/>
-      </c:barChart>
-      <c:catAx>
-        <c:axId val="310799823"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="15000"/>
-                <a:lumOff val="85000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0">
-                <a:ln>
-                  <a:noFill/>
-                </a:ln>
-                <a:solidFill>
-                  <a:srgbClr val="00B0F0"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
-                    <a:srgbClr val="000000">
-                      <a:alpha val="43137"/>
-                    </a:srgbClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="310801263"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="310801263"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:numFmt formatCode="0" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:ln>
-                  <a:noFill/>
-                </a:ln>
-                <a:solidFill>
-                  <a:srgbClr val="00B0F0"/>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
-                    <a:srgbClr val="000000">
-                      <a:alpha val="43137"/>
-                    </a:srgbClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="310799823"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln w="25400">
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="r"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:ln>
-                <a:noFill/>
-              </a:ln>
-              <a:solidFill>
-                <a:srgbClr val="00B0F0"/>
-              </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
-                  <a:srgbClr val="000000">
-                    <a:alpha val="43137"/>
-                  </a:srgbClr>
-                </a:outerShdw>
-              </a:effectLst>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-    <c:showDLblsOverMax val="0"/>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst>
-      <a:glow rad="381000">
-        <a:schemeClr val="accent1">
-          <a:alpha val="16000"/>
-        </a:schemeClr>
-      </a:glow>
-      <a:outerShdw blurRad="546100" dir="21540000" algn="t" rotWithShape="0">
-        <a:schemeClr val="accent6">
-          <a:lumMod val="75000"/>
-          <a:alpha val="40000"/>
-        </a:schemeClr>
-      </a:outerShdw>
-      <a:softEdge rad="0"/>
-    </a:effectLst>
-    <a:scene3d>
-      <a:camera prst="orthographicFront"/>
-      <a:lightRig rig="threePt" dir="t">
-        <a:rot lat="0" lon="0" rev="12000000"/>
-      </a:lightRig>
-    </a:scene3d>
-    <a:sp3d prstMaterial="dkEdge">
-      <a:bevelT w="165100" prst="coolSlant"/>
-    </a:sp3d>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:solidFill>
-            <a:srgbClr val="00B0F0"/>
-          </a:solidFill>
-          <a:effectLst>
-            <a:outerShdw dist="50800" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="43137"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:defRPr>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-  <c:extLst>
-    <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{781A3756-C4B2-4CAC-9D66-4F8BD8637D16}">
-      <c14:pivotOptions>
-        <c14:dropZoneFilter val="1"/>
-        <c14:dropZoneCategories val="1"/>
-        <c14:dropZoneData val="1"/>
-        <c14:dropZoneSeries val="1"/>
-        <c14:dropZonesVisible val="1"/>
-      </c14:pivotOptions>
-    </c:ext>
-    <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{E28EC0CA-F0BB-4C9C-879D-F8772B89E7AC}">
-      <c16:pivotOptions16>
-        <c16:showExpandCollapseFieldButtons val="1"/>
-      </c16:pivotOptions16>
-    </c:ext>
-  </c:extLst>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinearReversed" id="24">
-  <a:schemeClr val="accent4"/>
-</cs:colorStyle>
-</file>
-
-<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="212">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200" cap="all"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" b="0" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="38100" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr"/>
-      </a:solidFill>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="8"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:prstDash val="dash"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:prstDash val="dash"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="major">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="2000" b="0" kern="1200" cap="none" spc="0" normalizeH="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>75508</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>41564</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>699654</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>55418</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{633DD137-88C9-F68F-6DBE-95146FAF6680}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4228,7 +2608,7 @@
     <dataField name="Count of TradeID" fld="0" subtotal="count" baseField="2" baseItem="1"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="9">
+    <format dxfId="13">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="0"/>
@@ -4386,7 +2766,7 @@
     <tableColumn id="8" xr3:uid="{011760A3-A9D1-4015-8D75-7EFE2A2FEB20}" name="Risk Status"/>
     <tableColumn id="9" xr3:uid="{8E6DF200-182D-483A-8ED0-12101EFECD0F}" name="Profit per R"/>
     <tableColumn id="10" xr3:uid="{BB6361CF-CAA7-4423-9C5D-82E0E0F6DBCD}" name="Result"/>
-    <tableColumn id="11" xr3:uid="{420DB1BF-4073-4932-87BC-11D2FECAB843}" name="TradeDate" dataDxfId="19"/>
+    <tableColumn id="11" xr3:uid="{420DB1BF-4073-4932-87BC-11D2FECAB843}" name="TradeDate" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4406,14 +2786,14 @@
     <tableColumn id="5" xr3:uid="{539426CC-F875-4D64-977A-05C6F1BCDBCD}" name="Direction"/>
     <tableColumn id="6" xr3:uid="{BFF7C4D2-29D9-4645-98DB-6FBF609AB80F}" name="Profit"/>
     <tableColumn id="7" xr3:uid="{CD8DBAA1-576E-4991-87E5-049F5C232A1F}" name="R"/>
-    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="32">
+    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="12">
       <calculatedColumnFormula>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="31">
+    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="11">
       <calculatedColumnFormula>IFERROR(Table1[[#This Row],[Profit]]/Table1[[#This Row],[R]],"0")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{CC96218F-2F0A-46BB-98E4-8AE8218DB3D7}" name="Result"/>
-    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="30"/>
+    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4425,10 +2805,10 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{DAF88BD0-F115-4C64-AE11-7DD8AB7505A7}" name="Pair"/>
     <tableColumn id="2" xr3:uid="{89E35073-D474-496E-86E0-7646DF314B64}" name="Profit"/>
-    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="29">
+    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="9">
       <calculatedColumnFormula>TRIM(Table2[[#This Row],[Pair]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="28">
+    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="8">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Pair]]=Table2[[#This Row],[Clean Space]],"GOOD","NADFO")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4441,7 +2821,7 @@
   <autoFilter ref="K8:L12" xr:uid="{A99A2C5F-61E0-444B-907C-487860A13E40}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{0A321640-D79C-4135-83F6-E38913427047}" name="raw text"/>
-    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="27">
+    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="7">
       <calculatedColumnFormula>PROPER(Table4[[#This Row],[raw text]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4454,10 +2834,10 @@
   <autoFilter ref="K16:M19" xr:uid="{4576F3CB-3E9B-40EE-B5BA-0228DC3EBD7C}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{3D4EC290-099D-468C-B78D-8A8F427D8214}" name="text num"/>
-    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="26">
+    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="6">
       <calculatedColumnFormula>VALUE(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="25">
+    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="5">
       <calculatedColumnFormula>ISNUMBER(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4466,10 +2846,10 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}" name="Table5" displayName="Table5" ref="Q17:Q25" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}" name="Table5" displayName="Table5" ref="Q17:Q25" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
   <autoFilter ref="Q17:Q25" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{B868BDD4-CA52-440D-A1EA-1585934AF042}" name="TradeID" dataDxfId="22"/>
+    <tableColumn id="1" xr3:uid="{B868BDD4-CA52-440D-A1EA-1585934AF042}" name="TradeID" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6868,25 +5248,25 @@
       <c r="A6" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="23">
+      <c r="B6" s="22">
         <v>5</v>
       </c>
-      <c r="C6" s="23">
+      <c r="C6" s="22">
         <v>9</v>
       </c>
-      <c r="D6" s="23">
+      <c r="D6" s="22">
         <v>14</v>
       </c>
-      <c r="E6" s="23">
+      <c r="E6" s="22">
         <v>5</v>
       </c>
-      <c r="F6" s="23">
+      <c r="F6" s="22">
         <v>3</v>
       </c>
-      <c r="G6" s="23">
+      <c r="G6" s="22">
         <v>8</v>
       </c>
-      <c r="H6" s="23">
+      <c r="H6" s="22">
         <v>22</v>
       </c>
     </row>
@@ -6894,25 +5274,25 @@
       <c r="A7" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="23">
+      <c r="B7" s="22">
         <v>5</v>
       </c>
-      <c r="C7" s="23">
+      <c r="C7" s="22">
         <v>9</v>
       </c>
-      <c r="D7" s="23">
+      <c r="D7" s="22">
         <v>14</v>
       </c>
-      <c r="E7" s="23">
+      <c r="E7" s="22">
         <v>5</v>
       </c>
-      <c r="F7" s="23">
+      <c r="F7" s="22">
         <v>14</v>
       </c>
-      <c r="G7" s="23">
+      <c r="G7" s="22">
         <v>19</v>
       </c>
-      <c r="H7" s="23">
+      <c r="H7" s="22">
         <v>33</v>
       </c>
     </row>
@@ -6920,25 +5300,25 @@
       <c r="A8" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="23">
+      <c r="B8" s="22">
         <v>5</v>
       </c>
-      <c r="C8" s="23">
-        <v>10</v>
-      </c>
-      <c r="D8" s="23">
+      <c r="C8" s="22">
+        <v>10</v>
+      </c>
+      <c r="D8" s="22">
         <v>15</v>
       </c>
-      <c r="E8" s="23">
+      <c r="E8" s="22">
         <v>6</v>
       </c>
-      <c r="F8" s="23">
+      <c r="F8" s="22">
         <v>6</v>
       </c>
-      <c r="G8" s="23">
+      <c r="G8" s="22">
         <v>12</v>
       </c>
-      <c r="H8" s="23">
+      <c r="H8" s="22">
         <v>27</v>
       </c>
     </row>
@@ -6946,25 +5326,25 @@
       <c r="A9" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="23">
+      <c r="B9" s="22">
         <v>8</v>
       </c>
-      <c r="C9" s="23">
+      <c r="C9" s="22">
         <v>5</v>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="22">
         <v>13</v>
       </c>
-      <c r="E9" s="23">
+      <c r="E9" s="22">
         <v>2</v>
       </c>
-      <c r="F9" s="23">
+      <c r="F9" s="22">
         <v>3</v>
       </c>
-      <c r="G9" s="23">
+      <c r="G9" s="22">
         <v>5</v>
       </c>
-      <c r="H9" s="23">
+      <c r="H9" s="22">
         <v>18</v>
       </c>
     </row>
@@ -6997,11 +5377,506 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
-  <drawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC7DF93-3E77-4DA9-9925-C234221B379B}">
+  <dimension ref="B5:N38"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="28.88671875" customWidth="1"/>
+    <col min="3" max="3" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5546875" customWidth="1"/>
+    <col min="8" max="8" width="11.77734375" customWidth="1"/>
+    <col min="9" max="9" width="12.6640625" customWidth="1"/>
+    <col min="10" max="10" width="19.6640625" customWidth="1"/>
+    <col min="11" max="11" width="19.44140625" customWidth="1"/>
+    <col min="12" max="12" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="2">
+        <f>COUNT(Table1[TradeID])</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="2">
+        <f>SUM(Table1[Profit])</f>
+        <v>12225</v>
+      </c>
+    </row>
+    <row r="7" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="2">
+        <f>AVERAGE(Table1[Profit])</f>
+        <v>122.25</v>
+      </c>
+    </row>
+    <row r="8" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="2">
+        <f>MAX(Table1[Profit])</f>
+        <v>750</v>
+      </c>
+    </row>
+    <row r="9" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="2">
+        <f>MIN(Table1[Profit])</f>
+        <v>-375</v>
+      </c>
+    </row>
+    <row r="10" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10" s="2">
+        <f>COUNTIF(Table1[Result],"Win")</f>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="11" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C11" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="2">
+        <f>COUNTIF(Table1[Result],"Loss")</f>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="2">
+        <f>D10/D5</f>
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="14" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C14" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="N14" s="9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C15" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" s="2">
+        <f>COUNTIF(Table1[Pair],C15)</f>
+        <v>33</v>
+      </c>
+      <c r="E15" s="4">
+        <f>SUMIF(Table1[Pair],C15,Table1[Profit])</f>
+        <v>6825</v>
+      </c>
+      <c r="F15" s="5">
+        <f>AVERAGEIF(Table1[Pair],C15,Table1[Profit])</f>
+        <v>206.81818181818181</v>
+      </c>
+      <c r="G15" s="2">
+        <f>COUNTIFS(Table1[Pair],C15,Table1[Result],"Win")</f>
+        <v>23</v>
+      </c>
+      <c r="H15" s="6">
+        <f>G15/D15</f>
+        <v>0.69696969696969702</v>
+      </c>
+      <c r="I15" s="2">
+        <f>COUNTIFS(Table1[Pair],C15,Table1[Result],"Loss")</f>
+        <v>10</v>
+      </c>
+      <c r="J15" s="8">
+        <f>E15/$D$6</f>
+        <v>0.55828220858895705</v>
+      </c>
+      <c r="K15" s="2">
+        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C15,Table1[Result],"Win")</f>
+        <v>346.73913043478262</v>
+      </c>
+      <c r="L15" s="2">
+        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C15,Table1[Result],"Loss")</f>
+        <v>-115</v>
+      </c>
+      <c r="M15" s="2">
+        <f>K15/ABS(L15)</f>
+        <v>3.0151228733459359</v>
+      </c>
+      <c r="N15">
+        <f>(H15*K15)+(100-H15*L15)</f>
+        <v>421.81818181818187</v>
+      </c>
+    </row>
+    <row r="16" spans="3:14" x14ac:dyDescent="0.3">
+      <c r="C16" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="2">
+        <f>COUNTIF(Table1[Pair],C16)</f>
+        <v>22</v>
+      </c>
+      <c r="E16" s="4">
+        <f>SUMIF(Table1[Pair],C16,Table1[Profit])</f>
+        <v>2900</v>
+      </c>
+      <c r="F16" s="5">
+        <f>AVERAGEIF(Table1[Pair],C16,Table1[Profit])</f>
+        <v>131.81818181818181</v>
+      </c>
+      <c r="G16" s="2">
+        <f>COUNTIFS(Table1[Pair],C16,Table1[Result],"Win")</f>
+        <v>12</v>
+      </c>
+      <c r="H16" s="6">
+        <f>G16/D16</f>
+        <v>0.54545454545454541</v>
+      </c>
+      <c r="I16" s="2">
+        <f>COUNTIFS(Table1[Pair],C16,Table1[Result],"Loss")</f>
+        <v>10</v>
+      </c>
+      <c r="J16" s="8">
+        <f>E16/$D$6</f>
+        <v>0.23721881390593047</v>
+      </c>
+      <c r="K16" s="2">
+        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C16,Table1[Result],"Win")</f>
+        <v>308.33333333333331</v>
+      </c>
+      <c r="L16" s="2">
+        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C16,Table1[Result],"Loss")</f>
+        <v>-80</v>
+      </c>
+      <c r="M16" s="2">
+        <f t="shared" ref="M16:M18" si="0">K16/ABS(L16)</f>
+        <v>3.8541666666666665</v>
+      </c>
+      <c r="N16">
+        <f t="shared" ref="N16:N18" si="1">(H16*K16)+(100-H16*L16)</f>
+        <v>311.81818181818176</v>
+      </c>
+    </row>
+    <row r="17" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="C17" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="2">
+        <f>COUNTIF(Table1[Pair],C17)</f>
+        <v>27</v>
+      </c>
+      <c r="E17" s="4">
+        <f>SUMIF(Table1[Pair],C17,Table1[Profit])</f>
+        <v>1925</v>
+      </c>
+      <c r="F17" s="5">
+        <f>AVERAGEIF(Table1[Pair],C17,Table1[Profit])</f>
+        <v>71.296296296296291</v>
+      </c>
+      <c r="G17" s="2">
+        <f>COUNTIFS(Table1[Pair],C17,Table1[Result],"Win")</f>
+        <v>16</v>
+      </c>
+      <c r="H17" s="6">
+        <f>G17/D17</f>
+        <v>0.59259259259259256</v>
+      </c>
+      <c r="I17" s="2">
+        <f>COUNTIFS(Table1[Pair],C17,Table1[Result],"Loss")</f>
+        <v>11</v>
+      </c>
+      <c r="J17" s="8">
+        <f>E17/$D$6</f>
+        <v>0.15746421267893659</v>
+      </c>
+      <c r="K17" s="2">
+        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C17,Table1[Result],"Win")</f>
+        <v>246.875</v>
+      </c>
+      <c r="L17" s="2">
+        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C17,Table1[Result],"Loss")</f>
+        <v>-184.09090909090909</v>
+      </c>
+      <c r="M17" s="2">
+        <f t="shared" si="0"/>
+        <v>1.3410493827160495</v>
+      </c>
+      <c r="N17">
+        <f t="shared" si="1"/>
+        <v>355.38720538720537</v>
+      </c>
+    </row>
+    <row r="18" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="C18" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" s="2">
+        <f>COUNTIF(Table1[Pair],C18)</f>
+        <v>18</v>
+      </c>
+      <c r="E18" s="4">
+        <f>SUMIF(Table1[Pair],C18,Table1[Profit])</f>
+        <v>575</v>
+      </c>
+      <c r="F18" s="5">
+        <f>AVERAGEIF(Table1[Pair],C18,Table1[Profit])</f>
+        <v>31.944444444444443</v>
+      </c>
+      <c r="G18" s="2">
+        <f>COUNTIFS(Table1[Pair],C18,Table1[Result],"Win")</f>
+        <v>8</v>
+      </c>
+      <c r="H18" s="6">
+        <f>G18/D18</f>
+        <v>0.44444444444444442</v>
+      </c>
+      <c r="I18" s="2">
+        <f>COUNTIFS(Table1[Pair],C18,Table1[Result],"Loss")</f>
+        <v>10</v>
+      </c>
+      <c r="J18" s="8">
+        <f>E18/$D$6</f>
+        <v>4.7034764826175871E-2</v>
+      </c>
+      <c r="K18" s="2">
+        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C18,Table1[Result],"Win")</f>
+        <v>250</v>
+      </c>
+      <c r="L18" s="2">
+        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C18,Table1[Result],"Loss")</f>
+        <v>-142.5</v>
+      </c>
+      <c r="M18" s="2">
+        <f t="shared" si="0"/>
+        <v>1.7543859649122806</v>
+      </c>
+      <c r="N18">
+        <f t="shared" si="1"/>
+        <v>274.4444444444444</v>
+      </c>
+    </row>
+    <row r="19" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="I19" s="7"/>
+    </row>
+    <row r="21" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D21" t="s">
+        <v>40</v>
+      </c>
+      <c r="E21">
+        <f>COUNT(Table1[R])</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B22" t="s">
+        <v>5</v>
+      </c>
+      <c r="C22">
+        <f>COUNTBLANK(Table1[Profit])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B23" t="s">
+        <v>0</v>
+      </c>
+      <c r="C23">
+        <f>COUNTBLANK(Table1[TradeID])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C24">
+        <f>COUNTBLANK(Table1[AccountID])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B25" t="s">
+        <v>2</v>
+      </c>
+      <c r="C25">
+        <f>COUNTBLANK(Table1[Pair])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B26" t="s">
+        <v>3</v>
+      </c>
+      <c r="C26">
+        <f>COUNTBLANK(Table1[Session])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B27" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27">
+        <f>COUNTBLANK(Table1[Direction])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B28" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28">
+        <f>COUNTBLANK(Table1[R])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B29" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29">
+        <f>COUNTBLANK(Table1[Result])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B30" t="s">
+        <v>8</v>
+      </c>
+      <c r="C30">
+        <f>COUNTBLANK(Table1[TradeDate])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B34" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="35" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B35" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" s="6">
+        <f>9/14</f>
+        <v>0.6428571428571429</v>
+      </c>
+      <c r="D35" s="6">
+        <f>3/8</f>
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="36" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B36" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C36" s="6">
+        <f>9/14</f>
+        <v>0.6428571428571429</v>
+      </c>
+      <c r="D36" s="6">
+        <f>14/19</f>
+        <v>0.73684210526315785</v>
+      </c>
+    </row>
+    <row r="37" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B37" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C37" s="6">
+        <f>10/15</f>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="D37" s="6">
+        <f>6/12</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="38" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B38" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C38" s="6">
+        <f>5/13</f>
+        <v>0.38461538461538464</v>
+      </c>
+      <c r="D38" s="6">
+        <f>3/5</f>
+        <v>0.6</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C15:J18">
+    <sortCondition descending="1" ref="E14:E18"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{906658B5-1F80-4C49-9035-7A91F11B2092}">
   <dimension ref="A1:P101"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -7237,11 +6112,11 @@
       <c r="K6" s="1">
         <v>46041</v>
       </c>
-      <c r="N6" s="22" t="s">
+      <c r="N6" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="O6" s="22"/>
-      <c r="P6" s="22"/>
+      <c r="O6" s="23"/>
+      <c r="P6" s="23"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7">
@@ -10783,449 +9658,16 @@
     <mergeCell ref="N6:P6"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="21" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="20" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
     <tablePart r:id="rId2"/>
   </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC7DF93-3E77-4DA9-9925-C234221B379B}">
-  <dimension ref="B5:N30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="28.88671875" customWidth="1"/>
-    <col min="3" max="3" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.109375" customWidth="1"/>
-    <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5546875" customWidth="1"/>
-    <col min="8" max="8" width="11.77734375" customWidth="1"/>
-    <col min="9" max="9" width="12.6640625" customWidth="1"/>
-    <col min="10" max="10" width="19.6640625" customWidth="1"/>
-    <col min="11" max="11" width="19.44140625" customWidth="1"/>
-    <col min="12" max="12" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.44140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="5" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" s="2">
-        <f>COUNT(Table1[TradeID])</f>
-        <v>100</v>
-      </c>
-    </row>
-    <row r="6" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C6" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="2">
-        <f>SUM(Table1[Profit])</f>
-        <v>12225</v>
-      </c>
-    </row>
-    <row r="7" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C7" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="2">
-        <f>AVERAGE(Table1[Profit])</f>
-        <v>122.25</v>
-      </c>
-    </row>
-    <row r="8" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C8" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="2">
-        <f>MAX(Table1[Profit])</f>
-        <v>750</v>
-      </c>
-    </row>
-    <row r="9" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C9" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" s="2">
-        <f>MIN(Table1[Profit])</f>
-        <v>-375</v>
-      </c>
-    </row>
-    <row r="10" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C10" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D10" s="2">
-        <f>COUNTIF(Table1[Result],"Win")</f>
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C11" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" s="2">
-        <f>COUNTIF(Table1[Result],"Loss")</f>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="12" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C12" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D12" s="2">
-        <f>D10/D5</f>
-        <v>0.59</v>
-      </c>
-    </row>
-    <row r="14" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C14" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="K14" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="L14" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="M14" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="N14" s="9" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="15" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C15" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D15" s="2">
-        <f>COUNTIF(Table1[Pair],C15)</f>
-        <v>33</v>
-      </c>
-      <c r="E15" s="4">
-        <f>SUMIF(Table1[Pair],C15,Table1[Profit])</f>
-        <v>6825</v>
-      </c>
-      <c r="F15" s="5">
-        <f>AVERAGEIF(Table1[Pair],C15,Table1[Profit])</f>
-        <v>206.81818181818181</v>
-      </c>
-      <c r="G15" s="2">
-        <f>COUNTIFS(Table1[Pair],C15,Table1[Result],"Win")</f>
-        <v>23</v>
-      </c>
-      <c r="H15" s="6">
-        <f>G15/D15</f>
-        <v>0.69696969696969702</v>
-      </c>
-      <c r="I15" s="2">
-        <f>COUNTIFS(Table1[Pair],C15,Table1[Result],"Loss")</f>
-        <v>10</v>
-      </c>
-      <c r="J15" s="8">
-        <f>E15/$D$6</f>
-        <v>0.55828220858895705</v>
-      </c>
-      <c r="K15" s="2">
-        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C15,Table1[Result],"Win")</f>
-        <v>346.73913043478262</v>
-      </c>
-      <c r="L15" s="2">
-        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C15,Table1[Result],"Loss")</f>
-        <v>-115</v>
-      </c>
-      <c r="M15" s="2">
-        <f>K15/ABS(L15)</f>
-        <v>3.0151228733459359</v>
-      </c>
-      <c r="N15">
-        <f>(H15*K15)+(100-H15*L15)</f>
-        <v>421.81818181818187</v>
-      </c>
-    </row>
-    <row r="16" spans="3:14" x14ac:dyDescent="0.3">
-      <c r="C16" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D16" s="2">
-        <f>COUNTIF(Table1[Pair],C16)</f>
-        <v>22</v>
-      </c>
-      <c r="E16" s="4">
-        <f>SUMIF(Table1[Pair],C16,Table1[Profit])</f>
-        <v>2900</v>
-      </c>
-      <c r="F16" s="5">
-        <f>AVERAGEIF(Table1[Pair],C16,Table1[Profit])</f>
-        <v>131.81818181818181</v>
-      </c>
-      <c r="G16" s="2">
-        <f>COUNTIFS(Table1[Pair],C16,Table1[Result],"Win")</f>
-        <v>12</v>
-      </c>
-      <c r="H16" s="6">
-        <f>G16/D16</f>
-        <v>0.54545454545454541</v>
-      </c>
-      <c r="I16" s="2">
-        <f>COUNTIFS(Table1[Pair],C16,Table1[Result],"Loss")</f>
-        <v>10</v>
-      </c>
-      <c r="J16" s="8">
-        <f>E16/$D$6</f>
-        <v>0.23721881390593047</v>
-      </c>
-      <c r="K16" s="2">
-        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C16,Table1[Result],"Win")</f>
-        <v>308.33333333333331</v>
-      </c>
-      <c r="L16" s="2">
-        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C16,Table1[Result],"Loss")</f>
-        <v>-80</v>
-      </c>
-      <c r="M16" s="2">
-        <f t="shared" ref="M16:M18" si="0">K16/ABS(L16)</f>
-        <v>3.8541666666666665</v>
-      </c>
-      <c r="N16">
-        <f t="shared" ref="N16:N18" si="1">(H16*K16)+(100-H16*L16)</f>
-        <v>311.81818181818176</v>
-      </c>
-    </row>
-    <row r="17" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C17" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D17" s="2">
-        <f>COUNTIF(Table1[Pair],C17)</f>
-        <v>27</v>
-      </c>
-      <c r="E17" s="4">
-        <f>SUMIF(Table1[Pair],C17,Table1[Profit])</f>
-        <v>1925</v>
-      </c>
-      <c r="F17" s="5">
-        <f>AVERAGEIF(Table1[Pair],C17,Table1[Profit])</f>
-        <v>71.296296296296291</v>
-      </c>
-      <c r="G17" s="2">
-        <f>COUNTIFS(Table1[Pair],C17,Table1[Result],"Win")</f>
-        <v>16</v>
-      </c>
-      <c r="H17" s="6">
-        <f>G17/D17</f>
-        <v>0.59259259259259256</v>
-      </c>
-      <c r="I17" s="2">
-        <f>COUNTIFS(Table1[Pair],C17,Table1[Result],"Loss")</f>
-        <v>11</v>
-      </c>
-      <c r="J17" s="8">
-        <f>E17/$D$6</f>
-        <v>0.15746421267893659</v>
-      </c>
-      <c r="K17" s="2">
-        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C17,Table1[Result],"Win")</f>
-        <v>246.875</v>
-      </c>
-      <c r="L17" s="2">
-        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C17,Table1[Result],"Loss")</f>
-        <v>-184.09090909090909</v>
-      </c>
-      <c r="M17" s="2">
-        <f t="shared" si="0"/>
-        <v>1.3410493827160495</v>
-      </c>
-      <c r="N17">
-        <f t="shared" si="1"/>
-        <v>355.38720538720537</v>
-      </c>
-    </row>
-    <row r="18" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="C18" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D18" s="2">
-        <f>COUNTIF(Table1[Pair],C18)</f>
-        <v>18</v>
-      </c>
-      <c r="E18" s="4">
-        <f>SUMIF(Table1[Pair],C18,Table1[Profit])</f>
-        <v>575</v>
-      </c>
-      <c r="F18" s="5">
-        <f>AVERAGEIF(Table1[Pair],C18,Table1[Profit])</f>
-        <v>31.944444444444443</v>
-      </c>
-      <c r="G18" s="2">
-        <f>COUNTIFS(Table1[Pair],C18,Table1[Result],"Win")</f>
-        <v>8</v>
-      </c>
-      <c r="H18" s="6">
-        <f>G18/D18</f>
-        <v>0.44444444444444442</v>
-      </c>
-      <c r="I18" s="2">
-        <f>COUNTIFS(Table1[Pair],C18,Table1[Result],"Loss")</f>
-        <v>10</v>
-      </c>
-      <c r="J18" s="8">
-        <f>E18/$D$6</f>
-        <v>4.7034764826175871E-2</v>
-      </c>
-      <c r="K18" s="2">
-        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C18,Table1[Result],"Win")</f>
-        <v>250</v>
-      </c>
-      <c r="L18" s="2">
-        <f>AVERAGEIFS(Table1[Profit],Table1[Pair],C18,Table1[Result],"Loss")</f>
-        <v>-142.5</v>
-      </c>
-      <c r="M18" s="2">
-        <f t="shared" si="0"/>
-        <v>1.7543859649122806</v>
-      </c>
-      <c r="N18">
-        <f t="shared" si="1"/>
-        <v>274.4444444444444</v>
-      </c>
-    </row>
-    <row r="19" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="I19" s="7"/>
-    </row>
-    <row r="21" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B21" t="s">
-        <v>39</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="D21" t="s">
-        <v>40</v>
-      </c>
-      <c r="E21">
-        <f>COUNT(Table1[R])</f>
-        <v>100</v>
-      </c>
-    </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B22" t="s">
-        <v>5</v>
-      </c>
-      <c r="C22">
-        <f>COUNTBLANK(Table1[Profit])</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B23" t="s">
-        <v>0</v>
-      </c>
-      <c r="C23">
-        <f>COUNTBLANK(Table1[TradeID])</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B24" t="s">
-        <v>1</v>
-      </c>
-      <c r="C24">
-        <f>COUNTBLANK(Table1[AccountID])</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B25" t="s">
-        <v>2</v>
-      </c>
-      <c r="C25">
-        <f>COUNTBLANK(Table1[Pair])</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B26" t="s">
-        <v>3</v>
-      </c>
-      <c r="C26">
-        <f>COUNTBLANK(Table1[Session])</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B27" t="s">
-        <v>4</v>
-      </c>
-      <c r="C27">
-        <f>COUNTBLANK(Table1[Direction])</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B28" t="s">
-        <v>6</v>
-      </c>
-      <c r="C28">
-        <f>COUNTBLANK(Table1[R])</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B29" t="s">
-        <v>7</v>
-      </c>
-      <c r="C29">
-        <f>COUNTBLANK(Table1[Result])</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="2:14" x14ac:dyDescent="0.3">
-      <c r="B30" t="s">
-        <v>8</v>
-      </c>
-      <c r="C30">
-        <f>COUNTBLANK(Table1[TradeDate])</f>
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C15:J18">
-    <sortCondition descending="1" ref="E14:E18"/>
-  </sortState>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
hnaya zadt f table data analysis avg profit dyal kol pairs
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8152FD41-AF95-4D72-98B6-7D9170B84CA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B8C3ACE-1D3A-4CD1-99CE-582AECAC6710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="2" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="5" r:id="rId1"/>
@@ -80,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="804" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="88">
   <si>
     <t>TradeID</t>
   </si>
@@ -313,16 +313,37 @@
     <t>REVIEW</t>
   </si>
   <si>
-    <t>London Total</t>
-  </si>
-  <si>
-    <t>New York Total</t>
-  </si>
-  <si>
     <t>LONDON WIN RATE</t>
   </si>
   <si>
     <t>NEW YORK WIN RATE</t>
+  </si>
+  <si>
+    <t>London Count of TradeID</t>
+  </si>
+  <si>
+    <t>New York Count of TradeID</t>
+  </si>
+  <si>
+    <t>Total Count of TradeID</t>
+  </si>
+  <si>
+    <t>London Average of Profit</t>
+  </si>
+  <si>
+    <t>New York Average of Profit</t>
+  </si>
+  <si>
+    <t>Total Average of Profit</t>
+  </si>
+  <si>
+    <t>Average of Profit</t>
+  </si>
+  <si>
+    <t>avg profit london</t>
+  </si>
+  <si>
+    <t>avg profit new york</t>
   </si>
 </sst>
 </file>
@@ -842,7 +863,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -875,6 +896,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -921,7 +944,55 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="23">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2439,7 +2510,7 @@
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2DA79A61-38FD-45EA-A18C-EAC9CD91845A}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7" rowHeaderCaption="session rows" colHeaderCaption="result column">
-  <location ref="A3:H10" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
+  <location ref="A3:O11" firstHeaderRow="1" firstDataRow="4" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
@@ -2460,7 +2531,7 @@
       </items>
     </pivotField>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -2575,43 +2646,130 @@
       <x/>
     </i>
   </rowItems>
-  <colFields count="2">
+  <colFields count="3">
     <field x="3"/>
     <field x="9"/>
+    <field x="-2"/>
   </colFields>
-  <colItems count="7">
+  <colItems count="14">
     <i>
       <x/>
       <x/>
+      <x/>
+    </i>
+    <i r="2" i="1">
+      <x v="1"/>
     </i>
     <i r="1">
+      <x v="1"/>
+      <x/>
+    </i>
+    <i r="2" i="1">
       <x v="1"/>
     </i>
     <i t="default">
       <x/>
     </i>
+    <i t="default" i="1">
+      <x/>
+    </i>
     <i>
       <x v="1"/>
       <x/>
+      <x/>
+    </i>
+    <i r="2" i="1">
+      <x v="1"/>
     </i>
     <i r="1">
+      <x v="1"/>
+      <x/>
+    </i>
+    <i r="2" i="1">
       <x v="1"/>
     </i>
     <i t="default">
       <x v="1"/>
     </i>
+    <i t="default" i="1">
+      <x v="1"/>
+    </i>
     <i t="grand">
       <x/>
     </i>
+    <i t="grand" i="1">
+      <x/>
+    </i>
   </colItems>
-  <dataFields count="1">
+  <dataFields count="2">
     <dataField name="Count of TradeID" fld="0" subtotal="count" baseField="2" baseItem="1"/>
+    <dataField name="Average of Profit" fld="5" subtotal="average" baseField="2" baseItem="0"/>
   </dataFields>
-  <formats count="1">
-    <format dxfId="13">
+  <formats count="6">
+    <format dxfId="21">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="0"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="5">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="3">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="2" count="0"/>
+          <reference field="3" count="1" selected="0" defaultSubtotal="1">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="4">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="3" count="1" defaultSubtotal="1">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="3">
+      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
+        <references count="3">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="2" count="0"/>
+          <reference field="3" count="1" selected="0" defaultSubtotal="1">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="2">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="3" count="0" defaultSubtotal="1"/>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="0">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="3" count="1" defaultSubtotal="1">
+            <x v="1"/>
+          </reference>
         </references>
       </pivotArea>
     </format>
@@ -2766,7 +2924,7 @@
     <tableColumn id="8" xr3:uid="{011760A3-A9D1-4015-8D75-7EFE2A2FEB20}" name="Risk Status"/>
     <tableColumn id="9" xr3:uid="{8E6DF200-182D-483A-8ED0-12101EFECD0F}" name="Profit per R"/>
     <tableColumn id="10" xr3:uid="{BB6361CF-CAA7-4423-9C5D-82E0E0F6DBCD}" name="Result"/>
-    <tableColumn id="11" xr3:uid="{420DB1BF-4073-4932-87BC-11D2FECAB843}" name="TradeDate" dataDxfId="14"/>
+    <tableColumn id="11" xr3:uid="{420DB1BF-4073-4932-87BC-11D2FECAB843}" name="TradeDate" dataDxfId="22"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2786,14 +2944,14 @@
     <tableColumn id="5" xr3:uid="{539426CC-F875-4D64-977A-05C6F1BCDBCD}" name="Direction"/>
     <tableColumn id="6" xr3:uid="{BFF7C4D2-29D9-4645-98DB-6FBF609AB80F}" name="Profit"/>
     <tableColumn id="7" xr3:uid="{CD8DBAA1-576E-4991-87E5-049F5C232A1F}" name="R"/>
-    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="12">
+    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="20">
       <calculatedColumnFormula>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="11">
+    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="19">
       <calculatedColumnFormula>IFERROR(Table1[[#This Row],[Profit]]/Table1[[#This Row],[R]],"0")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{CC96218F-2F0A-46BB-98E4-8AE8218DB3D7}" name="Result"/>
-    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2805,10 +2963,10 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{DAF88BD0-F115-4C64-AE11-7DD8AB7505A7}" name="Pair"/>
     <tableColumn id="2" xr3:uid="{89E35073-D474-496E-86E0-7646DF314B64}" name="Profit"/>
-    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="9">
+    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="17">
       <calculatedColumnFormula>TRIM(Table2[[#This Row],[Pair]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="8">
+    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="16">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Pair]]=Table2[[#This Row],[Clean Space]],"GOOD","NADFO")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2821,7 +2979,7 @@
   <autoFilter ref="K8:L12" xr:uid="{A99A2C5F-61E0-444B-907C-487860A13E40}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{0A321640-D79C-4135-83F6-E38913427047}" name="raw text"/>
-    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="7">
+    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="15">
       <calculatedColumnFormula>PROPER(Table4[[#This Row],[raw text]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2834,10 +2992,10 @@
   <autoFilter ref="K16:M19" xr:uid="{4576F3CB-3E9B-40EE-B5BA-0228DC3EBD7C}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{3D4EC290-099D-468C-B78D-8A8F427D8214}" name="text num"/>
-    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="6">
+    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="14">
       <calculatedColumnFormula>VALUE(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="5">
+    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="13">
       <calculatedColumnFormula>ISNUMBER(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2846,10 +3004,10 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}" name="Table5" displayName="Table5" ref="Q17:Q25" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}" name="Table5" displayName="Table5" ref="Q17:Q25" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
   <autoFilter ref="Q17:Q25" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{B868BDD4-CA52-440D-A1EA-1585934AF042}" name="TradeID" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{B868BDD4-CA52-440D-A1EA-1585934AF042}" name="TradeID" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5189,189 +5347,337 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A00360D7-0D73-4CE4-AFB9-0AF5F61FAEDB}">
-  <dimension ref="A3:H10"/>
+  <dimension ref="A3:O11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="23.21875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="19" t="s">
-        <v>72</v>
-      </c>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B3" s="19" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>10</v>
       </c>
-      <c r="D4" t="s">
-        <v>77</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="H4" t="s">
         <v>16</v>
       </c>
-      <c r="G4" t="s">
-        <v>78</v>
-      </c>
-      <c r="H4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="19" t="s">
-        <v>74</v>
-      </c>
+      <c r="L4" t="s">
+        <v>80</v>
+      </c>
+      <c r="M4" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="N4" t="s">
+        <v>81</v>
+      </c>
+      <c r="O4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>17</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>12</v>
       </c>
-      <c r="E5" t="s">
+      <c r="G5" s="10"/>
+      <c r="H5" t="s">
         <v>17</v>
       </c>
-      <c r="F5" t="s">
+      <c r="J5" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="20" t="s">
+      <c r="M5" s="10"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A6" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6" t="s">
+        <v>85</v>
+      </c>
+      <c r="D6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E6" t="s">
+        <v>85</v>
+      </c>
+      <c r="G6" s="10"/>
+      <c r="H6" t="s">
+        <v>72</v>
+      </c>
+      <c r="I6" t="s">
+        <v>85</v>
+      </c>
+      <c r="J6" t="s">
+        <v>72</v>
+      </c>
+      <c r="K6" t="s">
+        <v>85</v>
+      </c>
+      <c r="M6" s="10"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A7" s="20" t="s">
         <v>9</v>
-      </c>
-      <c r="B6" s="22">
-        <v>5</v>
-      </c>
-      <c r="C6" s="22">
-        <v>9</v>
-      </c>
-      <c r="D6" s="22">
-        <v>14</v>
-      </c>
-      <c r="E6" s="22">
-        <v>5</v>
-      </c>
-      <c r="F6" s="22">
-        <v>3</v>
-      </c>
-      <c r="G6" s="22">
-        <v>8</v>
-      </c>
-      <c r="H6" s="22">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="20" t="s">
-        <v>15</v>
       </c>
       <c r="B7" s="22">
         <v>5</v>
       </c>
       <c r="C7" s="22">
+        <v>-90</v>
+      </c>
+      <c r="D7" s="22">
         <v>9</v>
       </c>
-      <c r="D7" s="22">
-        <v>14</v>
-      </c>
       <c r="E7" s="22">
-        <v>5</v>
+        <v>269.44444444444446</v>
       </c>
       <c r="F7" s="22">
         <v>14</v>
       </c>
-      <c r="G7" s="22">
-        <v>19</v>
+      <c r="G7" s="24">
+        <v>141.07142857142858</v>
       </c>
       <c r="H7" s="22">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+      <c r="I7" s="22">
+        <v>-70</v>
+      </c>
+      <c r="J7" s="22">
+        <v>3</v>
+      </c>
+      <c r="K7" s="22">
+        <v>425</v>
+      </c>
+      <c r="L7" s="22">
+        <v>8</v>
+      </c>
+      <c r="M7" s="24">
+        <v>115.625</v>
+      </c>
+      <c r="N7" s="22">
+        <v>22</v>
+      </c>
+      <c r="O7" s="22">
+        <v>131.81818181818181</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="20" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B8" s="22">
         <v>5</v>
       </c>
       <c r="C8" s="22">
-        <v>10</v>
+        <v>-95</v>
       </c>
       <c r="D8" s="22">
+        <v>9</v>
+      </c>
+      <c r="E8" s="22">
+        <v>394.44444444444446</v>
+      </c>
+      <c r="F8" s="22">
+        <v>14</v>
+      </c>
+      <c r="G8" s="24">
+        <v>219.64285714285714</v>
+      </c>
+      <c r="H8" s="22">
+        <v>5</v>
+      </c>
+      <c r="I8" s="22">
+        <v>-135</v>
+      </c>
+      <c r="J8" s="22">
+        <v>14</v>
+      </c>
+      <c r="K8" s="22">
+        <v>316.07142857142856</v>
+      </c>
+      <c r="L8" s="22">
+        <v>19</v>
+      </c>
+      <c r="M8" s="24">
+        <v>197.36842105263159</v>
+      </c>
+      <c r="N8" s="22">
+        <v>33</v>
+      </c>
+      <c r="O8" s="22">
+        <v>206.81818181818181</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A9" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="22">
+        <v>5</v>
+      </c>
+      <c r="C9" s="22">
+        <v>-155</v>
+      </c>
+      <c r="D9" s="22">
+        <v>10</v>
+      </c>
+      <c r="E9" s="22">
+        <v>205</v>
+      </c>
+      <c r="F9" s="22">
         <v>15</v>
       </c>
-      <c r="E8" s="22">
+      <c r="G9" s="24">
+        <v>85</v>
+      </c>
+      <c r="H9" s="22">
         <v>6</v>
       </c>
-      <c r="F8" s="22">
+      <c r="I9" s="22">
+        <v>-208.33333333333334</v>
+      </c>
+      <c r="J9" s="22">
         <v>6</v>
       </c>
-      <c r="G8" s="22">
+      <c r="K9" s="22">
+        <v>316.66666666666669</v>
+      </c>
+      <c r="L9" s="22">
         <v>12</v>
       </c>
-      <c r="H8" s="22">
+      <c r="M9" s="24">
+        <v>54.166666666666664</v>
+      </c>
+      <c r="N9" s="22">
         <v>27</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="20" t="s">
+      <c r="O9" s="22">
+        <v>71.296296296296291</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A10" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="22">
+      <c r="B10" s="22">
         <v>8</v>
       </c>
-      <c r="C9" s="22">
+      <c r="C10" s="22">
+        <v>-146.875</v>
+      </c>
+      <c r="D10" s="22">
         <v>5</v>
       </c>
-      <c r="D9" s="22">
+      <c r="E10" s="22">
+        <v>260</v>
+      </c>
+      <c r="F10" s="22">
         <v>13</v>
       </c>
-      <c r="E9" s="22">
+      <c r="G10" s="24">
+        <v>9.615384615384615</v>
+      </c>
+      <c r="H10" s="22">
         <v>2</v>
       </c>
-      <c r="F9" s="22">
+      <c r="I10" s="22">
+        <v>-125</v>
+      </c>
+      <c r="J10" s="22">
         <v>3</v>
       </c>
-      <c r="G9" s="22">
+      <c r="K10" s="22">
+        <v>233.33333333333334</v>
+      </c>
+      <c r="L10" s="22">
         <v>5</v>
       </c>
-      <c r="H9" s="22">
+      <c r="M10" s="24">
+        <v>90</v>
+      </c>
+      <c r="N10" s="22">
         <v>18</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="20" t="s">
+      <c r="O10" s="22">
+        <v>31.944444444444443</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A11" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="B10" s="21">
+      <c r="B11" s="21">
         <v>23</v>
       </c>
-      <c r="C10" s="21">
+      <c r="C11" s="21">
+        <v>-125</v>
+      </c>
+      <c r="D11" s="21">
         <v>33</v>
       </c>
-      <c r="D10" s="21">
+      <c r="E11" s="21">
+        <v>282.57575757575756</v>
+      </c>
+      <c r="F11" s="21">
         <v>56</v>
       </c>
-      <c r="E10" s="21">
+      <c r="G11" s="21">
+        <v>115.17857142857143</v>
+      </c>
+      <c r="H11" s="21">
         <v>18</v>
       </c>
-      <c r="F10" s="21">
+      <c r="I11" s="21">
+        <v>-140.27777777777777</v>
+      </c>
+      <c r="J11" s="21">
         <v>26</v>
       </c>
-      <c r="G10" s="21">
+      <c r="K11" s="21">
+        <v>319.23076923076923</v>
+      </c>
+      <c r="L11" s="21">
         <v>44</v>
       </c>
-      <c r="H10" s="21">
+      <c r="M11" s="21">
+        <v>131.25</v>
+      </c>
+      <c r="N11" s="21">
         <v>100</v>
+      </c>
+      <c r="O11" s="21">
+        <v>122.25</v>
       </c>
     </row>
   </sheetData>
@@ -5388,8 +5694,8 @@
     <col min="2" max="2" width="28.88671875" customWidth="1"/>
     <col min="3" max="3" width="16.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.5546875" customWidth="1"/>
     <col min="8" max="8" width="11.77734375" customWidth="1"/>
     <col min="9" max="9" width="12.6640625" customWidth="1"/>
@@ -5804,18 +6110,24 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B34" s="3" t="s">
         <v>27</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B35" s="2" t="s">
         <v>9</v>
       </c>
@@ -5827,8 +6139,14 @@
         <f>3/8</f>
         <v>0.375</v>
       </c>
-    </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E35" s="25">
+        <v>141.07142857142858</v>
+      </c>
+      <c r="F35" s="25">
+        <v>115.625</v>
+      </c>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B36" s="2" t="s">
         <v>15</v>
       </c>
@@ -5840,8 +6158,14 @@
         <f>14/19</f>
         <v>0.73684210526315785</v>
       </c>
-    </row>
-    <row r="37" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E36" s="25">
+        <v>219.64285714285714</v>
+      </c>
+      <c r="F36" s="25">
+        <v>197.36842105263159</v>
+      </c>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B37" s="2" t="s">
         <v>13</v>
       </c>
@@ -5853,8 +6177,14 @@
         <f>6/12</f>
         <v>0.5</v>
       </c>
-    </row>
-    <row r="38" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="E37" s="25">
+        <v>85</v>
+      </c>
+      <c r="F37" s="25">
+        <v>54.166666666666664</v>
+      </c>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B38" s="2" t="s">
         <v>18</v>
       </c>
@@ -5865,6 +6195,12 @@
       <c r="D38" s="6">
         <f>3/5</f>
         <v>0.6</v>
+      </c>
+      <c r="E38" s="25">
+        <v>9.615384615384615</v>
+      </c>
+      <c r="F38" s="25">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -9658,10 +9994,10 @@
     <mergeCell ref="N6:P6"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
hnaya zadt evg win evg loss
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B8C3ACE-1D3A-4CD1-99CE-582AECAC6710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B84C63A-B678-4A02-9C74-7A7780E76810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -80,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="802" uniqueCount="83">
   <si>
     <t>TradeID</t>
   </si>
@@ -319,31 +319,16 @@
     <t>NEW YORK WIN RATE</t>
   </si>
   <si>
-    <t>London Count of TradeID</t>
-  </si>
-  <si>
-    <t>New York Count of TradeID</t>
-  </si>
-  <si>
-    <t>Total Count of TradeID</t>
-  </si>
-  <si>
-    <t>London Average of Profit</t>
-  </si>
-  <si>
-    <t>New York Average of Profit</t>
-  </si>
-  <si>
-    <t>Total Average of Profit</t>
-  </si>
-  <si>
-    <t>Average of Profit</t>
-  </si>
-  <si>
     <t>avg profit london</t>
   </si>
   <si>
     <t>avg profit new york</t>
+  </si>
+  <si>
+    <t>avg  loss</t>
+  </si>
+  <si>
+    <t>avg win</t>
   </si>
 </sst>
 </file>
@@ -863,7 +848,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -893,11 +878,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="1" fontId="0" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -946,11 +930,17 @@
   </cellStyles>
   <dxfs count="23">
     <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <fill>
@@ -986,12 +976,6 @@
           <bgColor rgb="FFFFFF00"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2510,7 +2494,7 @@
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2DA79A61-38FD-45EA-A18C-EAC9CD91845A}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7" rowHeaderCaption="session rows" colHeaderCaption="result column">
-  <location ref="A3:O11" firstHeaderRow="1" firstDataRow="4" firstDataCol="1"/>
+  <location ref="A3:D9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
@@ -2523,7 +2507,7 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField axis="axisCol" showAll="0">
+    <pivotField showAll="0">
       <items count="3">
         <item x="1"/>
         <item x="0"/>
@@ -2531,7 +2515,7 @@
       </items>
     </pivotField>
     <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -2646,66 +2630,24 @@
       <x/>
     </i>
   </rowItems>
-  <colFields count="3">
-    <field x="3"/>
+  <colFields count="1">
     <field x="9"/>
-    <field x="-2"/>
   </colFields>
-  <colItems count="14">
+  <colItems count="3">
     <i>
-      <x/>
-      <x/>
-      <x/>
-    </i>
-    <i r="2" i="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-      <x/>
-    </i>
-    <i r="2" i="1">
-      <x v="1"/>
-    </i>
-    <i t="default">
-      <x/>
-    </i>
-    <i t="default" i="1">
       <x/>
     </i>
     <i>
-      <x v="1"/>
-      <x/>
-      <x/>
-    </i>
-    <i r="2" i="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-      <x/>
-    </i>
-    <i r="2" i="1">
-      <x v="1"/>
-    </i>
-    <i t="default">
-      <x v="1"/>
-    </i>
-    <i t="default" i="1">
       <x v="1"/>
     </i>
     <i t="grand">
       <x/>
     </i>
-    <i t="grand" i="1">
-      <x/>
-    </i>
   </colItems>
-  <dataFields count="2">
+  <dataFields count="1">
     <dataField name="Count of TradeID" fld="0" subtotal="count" baseField="2" baseItem="1"/>
-    <dataField name="Average of Profit" fld="5" subtotal="average" baseField="2" baseItem="0"/>
   </dataFields>
-  <formats count="6">
+  <formats count="1">
     <format dxfId="21">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
@@ -2713,129 +2655,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="5">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="2" count="0"/>
-          <reference field="3" count="1" selected="0" defaultSubtotal="1">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="4">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="3" count="1" defaultSubtotal="1">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="3">
-      <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="2" count="0"/>
-          <reference field="3" count="1" selected="0" defaultSubtotal="1">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="2">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="3" count="0" defaultSubtotal="1"/>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="0">
-      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="3" count="1" defaultSubtotal="1">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
   </formats>
-  <chartFormats count="4">
-    <chartFormat chart="0" format="0" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="3" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="9" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="3" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="9" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="2" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="3" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="9" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="0" format="3" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="3" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="9" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
@@ -5347,17 +5167,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A00360D7-0D73-4CE4-AFB9-0AF5F61FAEDB}">
-  <dimension ref="A3:O11"/>
+  <dimension ref="A3:D9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14.6640625" bestFit="1" customWidth="1"/>
@@ -5367,317 +5186,96 @@
     <col min="15" max="15" width="19.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="19" t="s">
+        <v>72</v>
+      </c>
       <c r="B3" s="19" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="19" t="s">
+        <v>74</v>
+      </c>
       <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" t="s">
-        <v>79</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="H4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="22">
+        <v>10</v>
+      </c>
+      <c r="C5" s="22">
+        <v>12</v>
+      </c>
+      <c r="D5" s="22">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" s="22">
+        <v>10</v>
+      </c>
+      <c r="C6" s="22">
+        <v>23</v>
+      </c>
+      <c r="D6" s="22">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="22">
+        <v>11</v>
+      </c>
+      <c r="C7" s="22">
         <v>16</v>
       </c>
-      <c r="L4" t="s">
-        <v>80</v>
-      </c>
-      <c r="M4" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="N4" t="s">
-        <v>81</v>
-      </c>
-      <c r="O4" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="B5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="10"/>
-      <c r="H5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J5" t="s">
-        <v>12</v>
-      </c>
-      <c r="M5" s="10"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A6" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="B6" t="s">
-        <v>72</v>
-      </c>
-      <c r="C6" t="s">
-        <v>85</v>
-      </c>
-      <c r="D6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E6" t="s">
-        <v>85</v>
-      </c>
-      <c r="G6" s="10"/>
-      <c r="H6" t="s">
-        <v>72</v>
-      </c>
-      <c r="I6" t="s">
-        <v>85</v>
-      </c>
-      <c r="J6" t="s">
-        <v>72</v>
-      </c>
-      <c r="K6" t="s">
-        <v>85</v>
-      </c>
-      <c r="M6" s="10"/>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A7" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="22">
-        <v>5</v>
-      </c>
-      <c r="C7" s="22">
-        <v>-90</v>
-      </c>
       <c r="D7" s="22">
-        <v>9</v>
-      </c>
-      <c r="E7" s="22">
-        <v>269.44444444444446</v>
-      </c>
-      <c r="F7" s="22">
-        <v>14</v>
-      </c>
-      <c r="G7" s="24">
-        <v>141.07142857142858</v>
-      </c>
-      <c r="H7" s="22">
-        <v>5</v>
-      </c>
-      <c r="I7" s="22">
-        <v>-70</v>
-      </c>
-      <c r="J7" s="22">
-        <v>3</v>
-      </c>
-      <c r="K7" s="22">
-        <v>425</v>
-      </c>
-      <c r="L7" s="22">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="22">
+        <v>10</v>
+      </c>
+      <c r="C8" s="22">
         <v>8</v>
       </c>
-      <c r="M7" s="24">
-        <v>115.625</v>
-      </c>
-      <c r="N7" s="22">
-        <v>22</v>
-      </c>
-      <c r="O7" s="22">
-        <v>131.81818181818181</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A8" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="22">
-        <v>5</v>
-      </c>
-      <c r="C8" s="22">
-        <v>-95</v>
-      </c>
       <c r="D8" s="22">
-        <v>9</v>
-      </c>
-      <c r="E8" s="22">
-        <v>394.44444444444446</v>
-      </c>
-      <c r="F8" s="22">
-        <v>14</v>
-      </c>
-      <c r="G8" s="24">
-        <v>219.64285714285714</v>
-      </c>
-      <c r="H8" s="22">
-        <v>5</v>
-      </c>
-      <c r="I8" s="22">
-        <v>-135</v>
-      </c>
-      <c r="J8" s="22">
-        <v>14</v>
-      </c>
-      <c r="K8" s="22">
-        <v>316.07142857142856</v>
-      </c>
-      <c r="L8" s="22">
-        <v>19</v>
-      </c>
-      <c r="M8" s="24">
-        <v>197.36842105263159</v>
-      </c>
-      <c r="N8" s="22">
-        <v>33</v>
-      </c>
-      <c r="O8" s="22">
-        <v>206.81818181818181</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="20" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="22">
-        <v>5</v>
-      </c>
-      <c r="C9" s="22">
-        <v>-155</v>
-      </c>
-      <c r="D9" s="22">
-        <v>10</v>
-      </c>
-      <c r="E9" s="22">
-        <v>205</v>
-      </c>
-      <c r="F9" s="22">
-        <v>15</v>
-      </c>
-      <c r="G9" s="24">
-        <v>85</v>
-      </c>
-      <c r="H9" s="22">
-        <v>6</v>
-      </c>
-      <c r="I9" s="22">
-        <v>-208.33333333333334</v>
-      </c>
-      <c r="J9" s="22">
-        <v>6</v>
-      </c>
-      <c r="K9" s="22">
-        <v>316.66666666666669</v>
-      </c>
-      <c r="L9" s="22">
-        <v>12</v>
-      </c>
-      <c r="M9" s="24">
-        <v>54.166666666666664</v>
-      </c>
-      <c r="N9" s="22">
-        <v>27</v>
-      </c>
-      <c r="O9" s="22">
-        <v>71.296296296296291</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A10" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="22">
-        <v>8</v>
-      </c>
-      <c r="C10" s="22">
-        <v>-146.875</v>
-      </c>
-      <c r="D10" s="22">
-        <v>5</v>
-      </c>
-      <c r="E10" s="22">
-        <v>260</v>
-      </c>
-      <c r="F10" s="22">
-        <v>13</v>
-      </c>
-      <c r="G10" s="24">
-        <v>9.615384615384615</v>
-      </c>
-      <c r="H10" s="22">
-        <v>2</v>
-      </c>
-      <c r="I10" s="22">
-        <v>-125</v>
-      </c>
-      <c r="J10" s="22">
-        <v>3</v>
-      </c>
-      <c r="K10" s="22">
-        <v>233.33333333333334</v>
-      </c>
-      <c r="L10" s="22">
-        <v>5</v>
-      </c>
-      <c r="M10" s="24">
-        <v>90</v>
-      </c>
-      <c r="N10" s="22">
-        <v>18</v>
-      </c>
-      <c r="O10" s="22">
-        <v>31.944444444444443</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A11" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="B11" s="21">
-        <v>23</v>
-      </c>
-      <c r="C11" s="21">
-        <v>-125</v>
-      </c>
-      <c r="D11" s="21">
-        <v>33</v>
-      </c>
-      <c r="E11" s="21">
-        <v>282.57575757575756</v>
-      </c>
-      <c r="F11" s="21">
-        <v>56</v>
-      </c>
-      <c r="G11" s="21">
-        <v>115.17857142857143</v>
-      </c>
-      <c r="H11" s="21">
-        <v>18</v>
-      </c>
-      <c r="I11" s="21">
-        <v>-140.27777777777777</v>
-      </c>
-      <c r="J11" s="21">
-        <v>26</v>
-      </c>
-      <c r="K11" s="21">
-        <v>319.23076923076923</v>
-      </c>
-      <c r="L11" s="21">
-        <v>44</v>
-      </c>
-      <c r="M11" s="21">
-        <v>131.25</v>
-      </c>
-      <c r="N11" s="21">
+      <c r="B9" s="21">
+        <v>41</v>
+      </c>
+      <c r="C9" s="21">
+        <v>59</v>
+      </c>
+      <c r="D9" s="21">
         <v>100</v>
-      </c>
-      <c r="O11" s="21">
-        <v>122.25</v>
       </c>
     </row>
   </sheetData>
@@ -6110,7 +5708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B34" s="3" t="s">
         <v>27</v>
       </c>
@@ -6121,13 +5719,19 @@
         <v>78</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
+        <v>80</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="35" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B35" s="2" t="s">
         <v>9</v>
       </c>
@@ -6139,14 +5743,21 @@
         <f>3/8</f>
         <v>0.375</v>
       </c>
-      <c r="E35" s="25">
+      <c r="E35" s="23">
         <v>141.07142857142858</v>
       </c>
-      <c r="F35" s="25">
+      <c r="F35" s="23">
         <v>115.625</v>
       </c>
-    </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="G35" s="6">
+        <f>10/22</f>
+        <v>0.45454545454545453</v>
+      </c>
+      <c r="H35" s="6">
+        <v>0.54545454545454541</v>
+      </c>
+    </row>
+    <row r="36" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B36" s="2" t="s">
         <v>15</v>
       </c>
@@ -6158,14 +5769,16 @@
         <f>14/19</f>
         <v>0.73684210526315785</v>
       </c>
-      <c r="E36" s="25">
+      <c r="E36" s="23">
         <v>219.64285714285714</v>
       </c>
-      <c r="F36" s="25">
+      <c r="F36" s="23">
         <v>197.36842105263159</v>
       </c>
-    </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="G36" s="6"/>
+      <c r="H36" s="6"/>
+    </row>
+    <row r="37" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B37" s="2" t="s">
         <v>13</v>
       </c>
@@ -6177,14 +5790,16 @@
         <f>6/12</f>
         <v>0.5</v>
       </c>
-      <c r="E37" s="25">
+      <c r="E37" s="23">
         <v>85</v>
       </c>
-      <c r="F37" s="25">
+      <c r="F37" s="23">
         <v>54.166666666666664</v>
       </c>
-    </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="G37" s="6"/>
+      <c r="H37" s="6"/>
+    </row>
+    <row r="38" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B38" s="2" t="s">
         <v>18</v>
       </c>
@@ -6196,12 +5811,14 @@
         <f>3/5</f>
         <v>0.6</v>
       </c>
-      <c r="E38" s="25">
+      <c r="E38" s="23">
         <v>9.615384615384615</v>
       </c>
-      <c r="F38" s="25">
+      <c r="F38" s="23">
         <v>90</v>
       </c>
+      <c r="G38" s="6"/>
+      <c r="H38" s="6"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C15:J18">
@@ -6448,11 +6065,11 @@
       <c r="K6" s="1">
         <v>46041</v>
       </c>
-      <c r="N6" s="23" t="s">
+      <c r="N6" s="24" t="s">
         <v>63</v>
       </c>
-      <c r="O6" s="23"/>
-      <c r="P6" s="23"/>
+      <c r="O6" s="24"/>
+      <c r="P6" s="24"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7">

</xml_diff>

<commit_message>
hnaya zadt columns joj dyal avg win w loss
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B84C63A-B678-4A02-9C74-7A7780E76810}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A1D7129-08E6-4594-8FCB-D431C8F52157}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
+    <workbookView xWindow="10356" yWindow="0" windowWidth="12780" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="5" r:id="rId1"/>
@@ -298,9 +298,6 @@
     <t>Grand Total</t>
   </si>
   <si>
-    <t>Count of TradeID</t>
-  </si>
-  <si>
     <t>result column</t>
   </si>
   <si>
@@ -329,6 +326,9 @@
   </si>
   <si>
     <t>avg win</t>
+  </si>
+  <si>
+    <t>Average of Profit</t>
   </si>
 </sst>
 </file>
@@ -928,54 +928,15 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="18">
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <font>
@@ -2496,7 +2457,7 @@
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2DA79A61-38FD-45EA-A18C-EAC9CD91845A}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7" rowHeaderCaption="session rows" colHeaderCaption="result column">
   <location ref="A3:D9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="11">
-    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
       <items count="5">
@@ -2515,7 +2476,7 @@
       </items>
     </pivotField>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -2645,10 +2606,10 @@
     </i>
   </colItems>
   <dataFields count="1">
-    <dataField name="Count of TradeID" fld="0" subtotal="count" baseField="2" baseItem="1"/>
+    <dataField name="Average of Profit" fld="5" subtotal="average" baseField="2" baseItem="2"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="21">
+    <format dxfId="16">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="0"/>
@@ -2744,7 +2705,7 @@
     <tableColumn id="8" xr3:uid="{011760A3-A9D1-4015-8D75-7EFE2A2FEB20}" name="Risk Status"/>
     <tableColumn id="9" xr3:uid="{8E6DF200-182D-483A-8ED0-12101EFECD0F}" name="Profit per R"/>
     <tableColumn id="10" xr3:uid="{BB6361CF-CAA7-4423-9C5D-82E0E0F6DBCD}" name="Result"/>
-    <tableColumn id="11" xr3:uid="{420DB1BF-4073-4932-87BC-11D2FECAB843}" name="TradeDate" dataDxfId="22"/>
+    <tableColumn id="11" xr3:uid="{420DB1BF-4073-4932-87BC-11D2FECAB843}" name="TradeDate" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2764,14 +2725,14 @@
     <tableColumn id="5" xr3:uid="{539426CC-F875-4D64-977A-05C6F1BCDBCD}" name="Direction"/>
     <tableColumn id="6" xr3:uid="{BFF7C4D2-29D9-4645-98DB-6FBF609AB80F}" name="Profit"/>
     <tableColumn id="7" xr3:uid="{CD8DBAA1-576E-4991-87E5-049F5C232A1F}" name="R"/>
-    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="20">
+    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="15">
       <calculatedColumnFormula>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="19">
+    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="14">
       <calculatedColumnFormula>IFERROR(Table1[[#This Row],[Profit]]/Table1[[#This Row],[R]],"0")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{CC96218F-2F0A-46BB-98E4-8AE8218DB3D7}" name="Result"/>
-    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="18"/>
+    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2783,10 +2744,10 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{DAF88BD0-F115-4C64-AE11-7DD8AB7505A7}" name="Pair"/>
     <tableColumn id="2" xr3:uid="{89E35073-D474-496E-86E0-7646DF314B64}" name="Profit"/>
-    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="17">
+    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="12">
       <calculatedColumnFormula>TRIM(Table2[[#This Row],[Pair]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="16">
+    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="11">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Pair]]=Table2[[#This Row],[Clean Space]],"GOOD","NADFO")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2799,7 +2760,7 @@
   <autoFilter ref="K8:L12" xr:uid="{A99A2C5F-61E0-444B-907C-487860A13E40}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{0A321640-D79C-4135-83F6-E38913427047}" name="raw text"/>
-    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="15">
+    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="10">
       <calculatedColumnFormula>PROPER(Table4[[#This Row],[raw text]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2812,10 +2773,10 @@
   <autoFilter ref="K16:M19" xr:uid="{4576F3CB-3E9B-40EE-B5BA-0228DC3EBD7C}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{3D4EC290-099D-468C-B78D-8A8F427D8214}" name="text num"/>
-    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="14">
+    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="9">
       <calculatedColumnFormula>VALUE(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="13">
+    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="8">
       <calculatedColumnFormula>ISNUMBER(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2824,10 +2785,10 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}" name="Table5" displayName="Table5" ref="Q17:Q25" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}" name="Table5" displayName="Table5" ref="Q17:Q25" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
   <autoFilter ref="Q17:Q25" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{B868BDD4-CA52-440D-A1EA-1585934AF042}" name="TradeID" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{B868BDD4-CA52-440D-A1EA-1585934AF042}" name="TradeID" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3220,7 +3181,7 @@
         <v>2</v>
       </c>
       <c r="H2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I2">
         <v>250</v>
@@ -3255,7 +3216,7 @@
         <v>2</v>
       </c>
       <c r="H3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I3">
         <v>250</v>
@@ -3290,7 +3251,7 @@
         <v>1.5</v>
       </c>
       <c r="H4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I4">
         <v>250</v>
@@ -3325,7 +3286,7 @@
         <v>1.5</v>
       </c>
       <c r="H5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I5">
         <v>250</v>
@@ -3360,7 +3321,7 @@
         <v>2</v>
       </c>
       <c r="H6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I6">
         <v>100</v>
@@ -3395,7 +3356,7 @@
         <v>2</v>
       </c>
       <c r="H7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I7">
         <v>100</v>
@@ -3430,7 +3391,7 @@
         <v>2.5</v>
       </c>
       <c r="H8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I8">
         <v>50</v>
@@ -3465,7 +3426,7 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I9">
         <v>100</v>
@@ -3500,7 +3461,7 @@
         <v>1</v>
       </c>
       <c r="H10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I10">
         <v>50</v>
@@ -3535,7 +3496,7 @@
         <v>-0.5</v>
       </c>
       <c r="H11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I11">
         <v>50</v>
@@ -3570,7 +3531,7 @@
         <v>-0.5</v>
       </c>
       <c r="H12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I12">
         <v>100</v>
@@ -3605,7 +3566,7 @@
         <v>-1</v>
       </c>
       <c r="H13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I13">
         <v>100</v>
@@ -3640,7 +3601,7 @@
         <v>-0.5</v>
       </c>
       <c r="H14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I14">
         <v>250</v>
@@ -3675,7 +3636,7 @@
         <v>-1.5</v>
       </c>
       <c r="H15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I15">
         <v>100</v>
@@ -3710,7 +3671,7 @@
         <v>3</v>
       </c>
       <c r="H16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I16">
         <v>250</v>
@@ -3745,7 +3706,7 @@
         <v>3</v>
       </c>
       <c r="H17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I17">
         <v>250</v>
@@ -3780,7 +3741,7 @@
         <v>2.5</v>
       </c>
       <c r="H18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I18">
         <v>250</v>
@@ -3815,7 +3776,7 @@
         <v>1.5</v>
       </c>
       <c r="H19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I19">
         <v>250</v>
@@ -3850,7 +3811,7 @@
         <v>3</v>
       </c>
       <c r="H20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I20">
         <v>100</v>
@@ -3885,7 +3846,7 @@
         <v>3</v>
       </c>
       <c r="H21" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I21">
         <v>100</v>
@@ -3920,7 +3881,7 @@
         <v>1</v>
       </c>
       <c r="H22" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I22">
         <v>250</v>
@@ -3955,7 +3916,7 @@
         <v>2</v>
       </c>
       <c r="H23" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I23">
         <v>50</v>
@@ -3990,7 +3951,7 @@
         <v>1</v>
       </c>
       <c r="H24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I24">
         <v>100</v>
@@ -4025,7 +3986,7 @@
         <v>-0.5</v>
       </c>
       <c r="H25" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I25">
         <v>50</v>
@@ -4060,7 +4021,7 @@
         <v>-0.5</v>
       </c>
       <c r="H26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I26">
         <v>100</v>
@@ -4095,7 +4056,7 @@
         <v>-0.5</v>
       </c>
       <c r="H27" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I27">
         <v>100</v>
@@ -4130,7 +4091,7 @@
         <v>-1</v>
       </c>
       <c r="H28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I28">
         <v>50</v>
@@ -4165,7 +4126,7 @@
         <v>-1.5</v>
       </c>
       <c r="H29" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I29">
         <v>200</v>
@@ -4200,7 +4161,7 @@
         <v>-1.5</v>
       </c>
       <c r="H30" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I30">
         <v>250</v>
@@ -4235,7 +4196,7 @@
         <v>-0.5</v>
       </c>
       <c r="H31" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I31">
         <v>250</v>
@@ -4270,7 +4231,7 @@
         <v>-1</v>
       </c>
       <c r="H32" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I32">
         <v>100</v>
@@ -4305,7 +4266,7 @@
         <v>-1</v>
       </c>
       <c r="H33" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I33">
         <v>100</v>
@@ -4340,7 +4301,7 @@
         <v>-1.5</v>
       </c>
       <c r="H34" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I34">
         <v>50</v>
@@ -4375,7 +4336,7 @@
         <v>1</v>
       </c>
       <c r="H35" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I35">
         <v>50</v>
@@ -4410,7 +4371,7 @@
         <v>1</v>
       </c>
       <c r="H36" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I36">
         <v>50</v>
@@ -4445,7 +4406,7 @@
         <v>3</v>
       </c>
       <c r="H37" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I37">
         <v>50</v>
@@ -4480,7 +4441,7 @@
         <v>3</v>
       </c>
       <c r="H38" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I38">
         <v>50</v>
@@ -4515,7 +4476,7 @@
         <v>2</v>
       </c>
       <c r="H39" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I39">
         <v>100</v>
@@ -4550,7 +4511,7 @@
         <v>1</v>
       </c>
       <c r="H40" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I40">
         <v>200</v>
@@ -4585,7 +4546,7 @@
         <v>1</v>
       </c>
       <c r="H41" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I41">
         <v>200</v>
@@ -4620,7 +4581,7 @@
         <v>1</v>
       </c>
       <c r="H42" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I42">
         <v>250</v>
@@ -4655,7 +4616,7 @@
         <v>1.5</v>
       </c>
       <c r="H43" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I43">
         <v>200</v>
@@ -4690,7 +4651,7 @@
         <v>2.5</v>
       </c>
       <c r="H44" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I44">
         <v>200</v>
@@ -4725,7 +4686,7 @@
         <v>-1</v>
       </c>
       <c r="H45" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I45">
         <v>250</v>
@@ -4760,7 +4721,7 @@
         <v>-1</v>
       </c>
       <c r="H46" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I46">
         <v>250</v>
@@ -4795,7 +4756,7 @@
         <v>-1</v>
       </c>
       <c r="H47" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I47">
         <v>200</v>
@@ -4830,7 +4791,7 @@
         <v>-1</v>
       </c>
       <c r="H48" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I48">
         <v>200</v>
@@ -4865,7 +4826,7 @@
         <v>-1.5</v>
       </c>
       <c r="H49" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I49">
         <v>50</v>
@@ -4900,7 +4861,7 @@
         <v>-1.5</v>
       </c>
       <c r="H50" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I50">
         <v>50</v>
@@ -4935,7 +4896,7 @@
         <v>-1.5</v>
       </c>
       <c r="H51" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I51">
         <v>50</v>
@@ -4970,7 +4931,7 @@
         <v>-0.5</v>
       </c>
       <c r="H52" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I52">
         <v>100</v>
@@ -5005,7 +4966,7 @@
         <v>1</v>
       </c>
       <c r="H53" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I53">
         <v>100</v>
@@ -5040,7 +5001,7 @@
         <v>1.5</v>
       </c>
       <c r="H54" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I54">
         <v>100</v>
@@ -5075,7 +5036,7 @@
         <v>2.5</v>
       </c>
       <c r="H55" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I55">
         <v>100</v>
@@ -5110,7 +5071,7 @@
         <v>1.5</v>
       </c>
       <c r="H56" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I56">
         <v>200</v>
@@ -5145,7 +5106,7 @@
         <v>2.5</v>
       </c>
       <c r="H57" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I57">
         <v>200</v>
@@ -5170,9 +5131,9 @@
   <dimension ref="A3:D9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="4.21875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
@@ -5188,15 +5149,15 @@
   <sheetData>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="B3" s="19" t="s">
         <v>72</v>
-      </c>
-      <c r="B3" s="19" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B4" t="s">
         <v>17</v>
@@ -5213,13 +5174,13 @@
         <v>9</v>
       </c>
       <c r="B5" s="22">
-        <v>10</v>
+        <v>-80</v>
       </c>
       <c r="C5" s="22">
-        <v>12</v>
+        <v>308.33333333333331</v>
       </c>
       <c r="D5" s="22">
-        <v>22</v>
+        <v>131.81818181818181</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -5227,13 +5188,13 @@
         <v>15</v>
       </c>
       <c r="B6" s="22">
-        <v>10</v>
+        <v>-115</v>
       </c>
       <c r="C6" s="22">
-        <v>23</v>
+        <v>346.73913043478262</v>
       </c>
       <c r="D6" s="22">
-        <v>33</v>
+        <v>206.81818181818181</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -5241,13 +5202,13 @@
         <v>13</v>
       </c>
       <c r="B7" s="22">
-        <v>11</v>
+        <v>-184.09090909090909</v>
       </c>
       <c r="C7" s="22">
-        <v>16</v>
+        <v>246.875</v>
       </c>
       <c r="D7" s="22">
-        <v>27</v>
+        <v>71.296296296296291</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -5255,13 +5216,13 @@
         <v>18</v>
       </c>
       <c r="B8" s="22">
-        <v>10</v>
+        <v>-142.5</v>
       </c>
       <c r="C8" s="22">
-        <v>8</v>
+        <v>250</v>
       </c>
       <c r="D8" s="22">
-        <v>18</v>
+        <v>31.944444444444443</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -5269,13 +5230,13 @@
         <v>71</v>
       </c>
       <c r="B9" s="21">
-        <v>41</v>
+        <v>-131.70731707317074</v>
       </c>
       <c r="C9" s="21">
-        <v>59</v>
+        <v>298.72881355932202</v>
       </c>
       <c r="D9" s="21">
-        <v>100</v>
+        <v>122.25</v>
       </c>
     </row>
   </sheetData>
@@ -5713,22 +5674,22 @@
         <v>27</v>
       </c>
       <c r="C34" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D34" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="E34" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="F34" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="F34" s="3" t="s">
+      <c r="G34" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="G34" s="3" t="s">
+      <c r="H34" s="3" t="s">
         <v>81</v>
-      </c>
-      <c r="H34" s="3" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.3">
@@ -5749,13 +5710,8 @@
       <c r="F35" s="23">
         <v>115.625</v>
       </c>
-      <c r="G35" s="6">
-        <f>10/22</f>
-        <v>0.45454545454545453</v>
-      </c>
-      <c r="H35" s="6">
-        <v>0.54545454545454541</v>
-      </c>
+      <c r="G35" s="6"/>
+      <c r="H35" s="6"/>
     </row>
     <row r="36" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B36" s="2" t="s">
@@ -9611,10 +9567,10 @@
     <mergeCell ref="N6:P6"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="9" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="8" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
hnaya zadt sheet jdida ela function nab9a ntaba9 fihom
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A1D7129-08E6-4594-8FCB-D431C8F52157}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6864E0AD-C136-42B3-BBBE-D08DFE830DC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10356" yWindow="0" windowWidth="12780" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="5" r:id="rId1"/>
     <sheet name="pivot table" sheetId="4" r:id="rId2"/>
     <sheet name="data analysis" sheetId="2" r:id="rId3"/>
     <sheet name="trading_raw_data2" sheetId="1" r:id="rId4"/>
-    <sheet name="data cleaning " sheetId="3" r:id="rId5"/>
+    <sheet name="functions" sheetId="6" r:id="rId5"/>
+    <sheet name="data cleaning " sheetId="3" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId6"/>
+    <pivotCache cacheId="0" r:id="rId7"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -80,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="802" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="832" uniqueCount="103">
   <si>
     <t>TradeID</t>
   </si>
@@ -328,7 +329,67 @@
     <t>avg win</t>
   </si>
   <si>
-    <t>Average of Profit</t>
+    <t>Sum of Profit</t>
+  </si>
+  <si>
+    <t>London Total</t>
+  </si>
+  <si>
+    <t>New York Total</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id </t>
+  </si>
+  <si>
+    <t>aba</t>
+  </si>
+  <si>
+    <t>sisa</t>
+  </si>
+  <si>
+    <t>kola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jihan </t>
+  </si>
+  <si>
+    <t>hana</t>
+  </si>
+  <si>
+    <t>bila</t>
+  </si>
+  <si>
+    <t>oha</t>
+  </si>
+  <si>
+    <t>fifa</t>
+  </si>
+  <si>
+    <t>fofo</t>
+  </si>
+  <si>
+    <t>ma</t>
+  </si>
+  <si>
+    <t>usa</t>
+  </si>
+  <si>
+    <t>ge</t>
+  </si>
+  <si>
+    <t>fr</t>
+  </si>
+  <si>
+    <t>match function</t>
   </si>
 </sst>
 </file>
@@ -848,7 +909,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -879,6 +940,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -928,16 +990,7 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="18">
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
+  <dxfs count="15">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2455,7 +2508,7 @@
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2DA79A61-38FD-45EA-A18C-EAC9CD91845A}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7" rowHeaderCaption="session rows" colHeaderCaption="result column">
-  <location ref="A3:D9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <location ref="A3:H10" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -2468,7 +2521,7 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField showAll="0">
+    <pivotField axis="axisCol" showAll="0">
       <items count="3">
         <item x="1"/>
         <item x="0"/>
@@ -2591,14 +2644,29 @@
       <x/>
     </i>
   </rowItems>
-  <colFields count="1">
+  <colFields count="2">
+    <field x="3"/>
     <field x="9"/>
   </colFields>
-  <colItems count="3">
+  <colItems count="7">
     <i>
+      <x/>
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i t="default">
       <x/>
     </i>
     <i>
+      <x v="1"/>
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i t="default">
       <x v="1"/>
     </i>
     <i t="grand">
@@ -2606,10 +2674,10 @@
     </i>
   </colItems>
   <dataFields count="1">
-    <dataField name="Average of Profit" fld="5" subtotal="average" baseField="2" baseItem="2"/>
+    <dataField name="Sum of Profit" fld="5" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="1">
-    <format dxfId="16">
+    <format dxfId="13">
       <pivotArea collapsedLevelsAreSubtotals="1" fieldPosition="0">
         <references count="1">
           <reference field="2" count="0"/>
@@ -2705,7 +2773,7 @@
     <tableColumn id="8" xr3:uid="{011760A3-A9D1-4015-8D75-7EFE2A2FEB20}" name="Risk Status"/>
     <tableColumn id="9" xr3:uid="{8E6DF200-182D-483A-8ED0-12101EFECD0F}" name="Profit per R"/>
     <tableColumn id="10" xr3:uid="{BB6361CF-CAA7-4423-9C5D-82E0E0F6DBCD}" name="Result"/>
-    <tableColumn id="11" xr3:uid="{420DB1BF-4073-4932-87BC-11D2FECAB843}" name="TradeDate" dataDxfId="17"/>
+    <tableColumn id="11" xr3:uid="{420DB1BF-4073-4932-87BC-11D2FECAB843}" name="TradeDate" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2725,14 +2793,14 @@
     <tableColumn id="5" xr3:uid="{539426CC-F875-4D64-977A-05C6F1BCDBCD}" name="Direction"/>
     <tableColumn id="6" xr3:uid="{BFF7C4D2-29D9-4645-98DB-6FBF609AB80F}" name="Profit"/>
     <tableColumn id="7" xr3:uid="{CD8DBAA1-576E-4991-87E5-049F5C232A1F}" name="R"/>
-    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="15">
+    <tableColumn id="13" xr3:uid="{5604F9D2-2C8F-4B63-9FB0-08636A1FD8D3}" name="Risk Status" dataDxfId="12">
       <calculatedColumnFormula>IF(OR(Table1[[#This Row],[R]]&gt;=2,Table1[[#This Row],[Profit]]&gt;500),"GOOD","REVIEW")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="14">
+    <tableColumn id="14" xr3:uid="{4778648E-2E5E-4C3F-BBFA-07AD84B520D7}" name="Profit per R" dataDxfId="11">
       <calculatedColumnFormula>IFERROR(Table1[[#This Row],[Profit]]/Table1[[#This Row],[R]],"0")</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{CC96218F-2F0A-46BB-98E4-8AE8218DB3D7}" name="Result"/>
-    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="13"/>
+    <tableColumn id="9" xr3:uid="{33DFF7EB-37F8-4413-89B2-47AF0ABF1AB0}" name="TradeDate" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2744,10 +2812,10 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{DAF88BD0-F115-4C64-AE11-7DD8AB7505A7}" name="Pair"/>
     <tableColumn id="2" xr3:uid="{89E35073-D474-496E-86E0-7646DF314B64}" name="Profit"/>
-    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="12">
+    <tableColumn id="3" xr3:uid="{D53F66F4-7509-4885-B440-8C48CF492C8C}" name="Clean Space" dataDxfId="9">
       <calculatedColumnFormula>TRIM(Table2[[#This Row],[Pair]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="11">
+    <tableColumn id="4" xr3:uid="{8C11A028-E104-4984-B143-1E828A3E1EC5}" name="check trim" dataDxfId="8">
       <calculatedColumnFormula>IF(Table2[[#This Row],[Pair]]=Table2[[#This Row],[Clean Space]],"GOOD","NADFO")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2760,7 +2828,7 @@
   <autoFilter ref="K8:L12" xr:uid="{A99A2C5F-61E0-444B-907C-487860A13E40}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{0A321640-D79C-4135-83F6-E38913427047}" name="raw text"/>
-    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="10">
+    <tableColumn id="2" xr3:uid="{AFAFC69E-5221-4C5C-BCDC-FA9796537B90}" name="text" dataDxfId="7">
       <calculatedColumnFormula>PROPER(Table4[[#This Row],[raw text]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2773,10 +2841,10 @@
   <autoFilter ref="K16:M19" xr:uid="{4576F3CB-3E9B-40EE-B5BA-0228DC3EBD7C}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{3D4EC290-099D-468C-B78D-8A8F427D8214}" name="text num"/>
-    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="9">
+    <tableColumn id="2" xr3:uid="{8229FBAA-503A-4FA9-B868-506EDAF0BEB3}" name="convert" dataDxfId="6">
       <calculatedColumnFormula>VALUE(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="8">
+    <tableColumn id="3" xr3:uid="{A32329F0-3CAE-4B77-9C4A-66E55F5E38EA}" name="check" dataDxfId="5">
       <calculatedColumnFormula>ISNUMBER(Table3[[#This Row],[text num]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2785,10 +2853,10 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}" name="Table5" displayName="Table5" ref="Q17:Q25" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}" name="Table5" displayName="Table5" ref="Q17:Q25" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
   <autoFilter ref="Q17:Q25" xr:uid="{9284F1F2-066B-4F54-888C-872719B32047}"/>
   <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{B868BDD4-CA52-440D-A1EA-1585934AF042}" name="TradeID" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{B868BDD4-CA52-440D-A1EA-1585934AF042}" name="TradeID" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5128,14 +5196,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A00360D7-0D73-4CE4-AFB9-0AF5F61FAEDB}">
-  <dimension ref="A3:D9"/>
+  <dimension ref="A3:H10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
@@ -5147,7 +5216,7 @@
     <col min="15" max="15" width="19.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
         <v>82</v>
       </c>
@@ -5155,88 +5224,168 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="19" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>17</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C5" t="s">
         <v>12</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="22">
+        <v>-450</v>
+      </c>
+      <c r="C6" s="22">
+        <v>2425</v>
+      </c>
+      <c r="D6" s="22">
+        <v>1975</v>
+      </c>
+      <c r="E6" s="22">
+        <v>-350</v>
+      </c>
+      <c r="F6" s="22">
+        <v>1275</v>
+      </c>
+      <c r="G6" s="22">
+        <v>925</v>
+      </c>
+      <c r="H6" s="22">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="22">
+        <v>-475</v>
+      </c>
+      <c r="C7" s="22">
+        <v>3550</v>
+      </c>
+      <c r="D7" s="22">
+        <v>3075</v>
+      </c>
+      <c r="E7" s="22">
+        <v>-675</v>
+      </c>
+      <c r="F7" s="22">
+        <v>4425</v>
+      </c>
+      <c r="G7" s="22">
+        <v>3750</v>
+      </c>
+      <c r="H7" s="22">
+        <v>6825</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="22">
+        <v>-775</v>
+      </c>
+      <c r="C8" s="22">
+        <v>2050</v>
+      </c>
+      <c r="D8" s="22">
+        <v>1275</v>
+      </c>
+      <c r="E8" s="22">
+        <v>-1250</v>
+      </c>
+      <c r="F8" s="22">
+        <v>1900</v>
+      </c>
+      <c r="G8" s="22">
+        <v>650</v>
+      </c>
+      <c r="H8" s="22">
+        <v>1925</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="22">
+        <v>-1175</v>
+      </c>
+      <c r="C9" s="22">
+        <v>1300</v>
+      </c>
+      <c r="D9" s="22">
+        <v>125</v>
+      </c>
+      <c r="E9" s="22">
+        <v>-250</v>
+      </c>
+      <c r="F9" s="22">
+        <v>700</v>
+      </c>
+      <c r="G9" s="22">
+        <v>450</v>
+      </c>
+      <c r="H9" s="22">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="20" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="22">
-        <v>-80</v>
-      </c>
-      <c r="C5" s="22">
-        <v>308.33333333333331</v>
-      </c>
-      <c r="D5" s="22">
-        <v>131.81818181818181</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="22">
-        <v>-115</v>
-      </c>
-      <c r="C6" s="22">
-        <v>346.73913043478262</v>
-      </c>
-      <c r="D6" s="22">
-        <v>206.81818181818181</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="20" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="22">
-        <v>-184.09090909090909</v>
-      </c>
-      <c r="C7" s="22">
-        <v>246.875</v>
-      </c>
-      <c r="D7" s="22">
-        <v>71.296296296296291</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="20" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="22">
-        <v>-142.5</v>
-      </c>
-      <c r="C8" s="22">
-        <v>250</v>
-      </c>
-      <c r="D8" s="22">
-        <v>31.944444444444443</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="B9" s="21">
-        <v>-131.70731707317074</v>
-      </c>
-      <c r="C9" s="21">
-        <v>298.72881355932202</v>
-      </c>
-      <c r="D9" s="21">
-        <v>122.25</v>
+      <c r="B10" s="21">
+        <v>-2875</v>
+      </c>
+      <c r="C10" s="21">
+        <v>9325</v>
+      </c>
+      <c r="D10" s="21">
+        <v>6450</v>
+      </c>
+      <c r="E10" s="21">
+        <v>-2525</v>
+      </c>
+      <c r="F10" s="21">
+        <v>8300</v>
+      </c>
+      <c r="G10" s="21">
+        <v>5775</v>
+      </c>
+      <c r="H10" s="21">
+        <v>12225</v>
       </c>
     </row>
   </sheetData>
@@ -6021,11 +6170,11 @@
       <c r="K6" s="1">
         <v>46041</v>
       </c>
-      <c r="N6" s="24" t="s">
+      <c r="N6" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="O6" s="24"/>
-      <c r="P6" s="24"/>
+      <c r="O6" s="25"/>
+      <c r="P6" s="25"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7">
@@ -9567,10 +9716,10 @@
     <mergeCell ref="N6:P6"/>
   </mergeCells>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="4" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -9581,6 +9730,183 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD321151-4306-4E94-877E-3E0A5CCF7860}">
+  <dimension ref="A3:J13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="9" max="9" width="15.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I3" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="J3" s="25"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4" s="24" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="D4" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="J4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
+        <v>1000</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C5" s="2">
+        <v>12</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="I5">
+        <f>MATCH(J5,A5:A13,0)</f>
+        <v>6</v>
+      </c>
+      <c r="J5">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6" s="2">
+        <v>2000</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C6" s="2">
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7" s="2">
+        <v>3000</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C7" s="2">
+        <v>27</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8" s="2">
+        <v>4000</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C8" s="2">
+        <v>38</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9" s="2">
+        <v>5000</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C9" s="2">
+        <v>39</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10" s="2">
+        <v>6000</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C10" s="2">
+        <v>26</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11" s="2">
+        <v>7000</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C11" s="2">
+        <v>44</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="2">
+        <v>8000</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C12" s="2">
+        <v>87</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="2">
+        <v>9000</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C13" s="2">
+        <v>56</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="I3:J3"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5" xr:uid="{95AF04DE-4D2C-4A78-97A7-E1ED043615F0}">
+      <formula1>$A$5:$A$13</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDB00B21-86E3-4E60-9B16-646B4376A26A}">
   <dimension ref="F7:X25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
hnaya zadt function dyal index
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6864E0AD-C136-42B3-BBBE-D08DFE830DC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE20BE3D-180F-48A8-9407-6EF85668B348}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="832" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="833" uniqueCount="104">
   <si>
     <t>TradeID</t>
   </si>
@@ -390,6 +390,9 @@
   </si>
   <si>
     <t>match function</t>
+  </si>
+  <si>
+    <t>index  function</t>
   </si>
 </sst>
 </file>
@@ -9735,6 +9738,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="9" max="9" width="15.88671875" customWidth="1"/>
+    <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -9836,6 +9840,10 @@
       <c r="D9" s="2" t="s">
         <v>98</v>
       </c>
+      <c r="I9" s="25" t="s">
+        <v>103</v>
+      </c>
+      <c r="J9" s="25"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
@@ -9850,6 +9858,13 @@
       <c r="D10" s="2" t="s">
         <v>100</v>
       </c>
+      <c r="I10" cm="1">
+        <f t="array" ref="I10">INDEX(A5:A13,J10)</f>
+        <v>4000</v>
+      </c>
+      <c r="J10">
+        <v>4</v>
+      </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
@@ -9894,8 +9909,9 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="I3:J3"/>
+    <mergeCell ref="I9:J9"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5" xr:uid="{95AF04DE-4D2C-4A78-97A7-E1ED043615F0}">

</xml_diff>

<commit_message>
hnaya kantrini ela if function
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08F4842A-71EF-4337-B7D0-19A2C25460F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC1336B1-7DF9-4873-94F1-4E2918A7A853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="837" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="829" uniqueCount="103">
   <si>
     <t>TradeID</t>
   </si>
@@ -377,18 +377,6 @@
     <t>fofo</t>
   </si>
   <si>
-    <t>ma</t>
-  </si>
-  <si>
-    <t>usa</t>
-  </si>
-  <si>
-    <t>ge</t>
-  </si>
-  <si>
-    <t>fr</t>
-  </si>
-  <si>
     <t>match function</t>
   </si>
   <si>
@@ -399,6 +387,9 @@
   </si>
   <si>
     <t>h look up</t>
+  </si>
+  <si>
+    <t>if</t>
   </si>
 </sst>
 </file>
@@ -933,7 +924,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -978,6 +969,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -9774,7 +9766,7 @@
   <sheetData>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="I3" s="27" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="J3" s="27"/>
     </row>
@@ -9791,6 +9783,9 @@
       <c r="D4" s="24" t="s">
         <v>87</v>
       </c>
+      <c r="E4" s="30" t="s">
+        <v>102</v>
+      </c>
       <c r="J4" t="s">
         <v>60</v>
       </c>
@@ -9805,8 +9800,13 @@
       <c r="C5" s="2">
         <v>12</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>98</v>
+      <c r="D5" s="2" t="str">
+        <f>IF(C5&gt;20,"kbir","sghir")</f>
+        <v>sghir</v>
+      </c>
+      <c r="E5" t="str">
+        <f>IF(D5&gt;20,"")</f>
+        <v/>
       </c>
       <c r="I5">
         <f>MATCH(J5,A5:A13,0)</f>
@@ -9826,8 +9826,9 @@
       <c r="C6" s="2">
         <v>13</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>98</v>
+      <c r="D6" s="2" t="str">
+        <f t="shared" ref="D6:D13" si="0">IF(C6&gt;20,"kbir","sghir")</f>
+        <v>sghir</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
@@ -9840,8 +9841,9 @@
       <c r="C7" s="2">
         <v>27</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>99</v>
+      <c r="D7" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>kbir</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
@@ -9854,8 +9856,9 @@
       <c r="C8" s="2">
         <v>38</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>98</v>
+      <c r="D8" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>kbir</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
@@ -9868,11 +9871,12 @@
       <c r="C9" s="2">
         <v>39</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>98</v>
+      <c r="D9" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>kbir</v>
       </c>
       <c r="I9" s="27" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="J9" s="27"/>
     </row>
@@ -9886,8 +9890,9 @@
       <c r="C10" s="2">
         <v>26</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>100</v>
+      <c r="D10" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>kbir</v>
       </c>
       <c r="I10" cm="1">
         <f t="array" ref="I10">INDEX(A5:A13,J10)</f>
@@ -9907,8 +9912,9 @@
       <c r="C11" s="2">
         <v>44</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>101</v>
+      <c r="D11" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>kbir</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
@@ -9921,8 +9927,9 @@
       <c r="C12" s="2">
         <v>87</v>
       </c>
-      <c r="D12" s="2" t="s">
-        <v>100</v>
+      <c r="D12" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>kbir</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
@@ -9935,13 +9942,14 @@
       <c r="C13" s="2">
         <v>56</v>
       </c>
-      <c r="D13" s="2" t="s">
-        <v>101</v>
+      <c r="D13" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>kbir</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="K16" s="27" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="L16" s="27"/>
       <c r="M16" s="27"/>
@@ -9951,7 +9959,7 @@
         <v>90</v>
       </c>
       <c r="J17" s="26" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="K17" s="29"/>
       <c r="L17" s="27"/>

</xml_diff>

<commit_message>
hnaya hnaya nja7t bach nkhadam h look up
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B513528-647F-4B86-940A-DE7E8F8B468B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07CF8B97-FC81-4A2C-A708-66DAC71E011C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="822" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="827" uniqueCount="102">
   <si>
     <t>TradeID</t>
   </si>
@@ -379,6 +379,15 @@
   <si>
     <t>if</t>
   </si>
+  <si>
+    <t>colum</t>
+  </si>
+  <si>
+    <t>row</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h look up </t>
+  </si>
 </sst>
 </file>
 
@@ -523,7 +532,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -706,6 +715,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -897,7 +912,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -936,6 +951,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -9723,10 +9741,13 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD321151-4306-4E94-877E-3E0A5CCF7860}">
-  <dimension ref="A4:I16"/>
+  <dimension ref="A4:J16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="10" max="10" width="14.44140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
         <v>88</v>
       </c>
@@ -9743,7 +9764,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>1000</v>
       </c>
@@ -9762,7 +9783,7 @@
         <v>kbir</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>2000</v>
       </c>
@@ -9781,7 +9802,7 @@
         <v>kbir</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>3000</v>
       </c>
@@ -9799,8 +9820,12 @@
         <f t="shared" si="0"/>
         <v>kbir</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I7" s="26" t="s">
+        <v>101</v>
+      </c>
+      <c r="J7" s="26"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>4000</v>
       </c>
@@ -9819,7 +9844,7 @@
         <v>kbir</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>5000</v>
       </c>
@@ -9837,8 +9862,14 @@
         <f t="shared" si="0"/>
         <v>kbir</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I9" s="24" t="s">
+        <v>99</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>6000</v>
       </c>
@@ -9856,8 +9887,14 @@
         <f t="shared" si="0"/>
         <v>kbir</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I10" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>7000</v>
       </c>
@@ -9876,7 +9913,7 @@
         <v>kbir</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>8000</v>
       </c>
@@ -9894,8 +9931,13 @@
         <f t="shared" si="0"/>
         <v>kbir</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="I12" s="28" t="str">
+        <f>HLOOKUP(J9,B4:D13,MATCH(J10,B4:B13,0))</f>
+        <v>sghir</v>
+      </c>
+      <c r="J12" s="28"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>9000</v>
       </c>
@@ -9914,10 +9956,14 @@
         <v>kbir</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="I16" s="25"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="I12:J12"/>
+    <mergeCell ref="I7:J7"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
hna fchalt f vlookup
</commit_message>
<xml_diff>
--- a/trading_raw_data-main.xlsx
+++ b/trading_raw_data-main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\THINKPAD\Desktop\excel projrct\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07CF8B97-FC81-4A2C-A708-66DAC71E011C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E568EB1E-3C7C-4DA6-877D-9A3928011E73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{29389193-7256-4448-99EA-708D1049F25F}"/>
   </bookViews>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="827" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="101">
   <si>
     <t>TradeID</t>
   </si>
@@ -347,9 +347,6 @@
     <t>country</t>
   </si>
   <si>
-    <t xml:space="preserve">id </t>
-  </si>
-  <si>
     <t>aba</t>
   </si>
   <si>
@@ -377,9 +374,6 @@
     <t>fofo</t>
   </si>
   <si>
-    <t>if</t>
-  </si>
-  <si>
     <t>colum</t>
   </si>
   <si>
@@ -387,6 +381,9 @@
   </si>
   <si>
     <t xml:space="preserve">h look up </t>
+  </si>
+  <si>
+    <t>v look up</t>
   </si>
 </sst>
 </file>
@@ -950,10 +947,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -9741,228 +9738,240 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD321151-4306-4E94-877E-3E0A5CCF7860}">
-  <dimension ref="A4:J16"/>
+  <dimension ref="A4:K24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="10" max="10" width="14.44140625" customWidth="1"/>
+    <col min="8" max="8" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B4" s="24" t="s">
-        <v>85</v>
-      </c>
-      <c r="C4" s="24" t="s">
-        <v>86</v>
-      </c>
-      <c r="D4" s="24" t="s">
-        <v>87</v>
-      </c>
-      <c r="E4" s="27" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="2">
-        <v>1000</v>
-      </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="2">
+        <v>12</v>
+      </c>
+      <c r="C5" s="2" t="str">
+        <f>IF(B5&gt;20,"kbir","sghir")</f>
+        <v>sghir</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C5" s="2">
-        <v>12</v>
-      </c>
-      <c r="D5" s="2" t="str">
-        <f>IF(C5&gt;20,"kbir","sghir")</f>
+      <c r="B6" s="2">
+        <v>13</v>
+      </c>
+      <c r="C6" s="2" t="str">
+        <f t="shared" ref="C6:C13" si="0">IF(B6&gt;20,"kbir","sghir")</f>
         <v>sghir</v>
       </c>
-      <c r="E5" t="str">
-        <f>IF(D5&gt;20,"kbir","sghir")</f>
-        <v>kbir</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="2">
-        <v>2000</v>
-      </c>
-      <c r="B6" s="2" t="s">
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C6" s="2">
-        <v>13</v>
-      </c>
-      <c r="D6" s="2" t="str">
-        <f t="shared" ref="D6:E13" si="0">IF(C6&gt;20,"kbir","sghir")</f>
-        <v>sghir</v>
-      </c>
-      <c r="E6" t="str">
+      <c r="B7" s="2">
+        <v>27</v>
+      </c>
+      <c r="C7" s="2" t="str">
         <f t="shared" si="0"/>
         <v>kbir</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="2">
-        <v>3000</v>
-      </c>
-      <c r="B7" s="2" t="s">
+      <c r="G7" s="26" t="s">
+        <v>99</v>
+      </c>
+      <c r="H7" s="26"/>
+      <c r="I7" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="J7" s="26"/>
+      <c r="K7" s="26"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C7" s="2">
-        <v>27</v>
-      </c>
-      <c r="D7" s="2" t="str">
+      <c r="B8" s="2">
+        <v>38</v>
+      </c>
+      <c r="C8" s="2" t="str">
         <f t="shared" si="0"/>
         <v>kbir</v>
       </c>
-      <c r="E7" t="str">
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B9" s="2">
+        <v>39</v>
+      </c>
+      <c r="C9" s="2" t="str">
         <f t="shared" si="0"/>
         <v>kbir</v>
       </c>
-      <c r="I7" s="26" t="s">
-        <v>101</v>
-      </c>
-      <c r="J7" s="26"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="2">
-        <v>4000</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="C8" s="2">
-        <v>38</v>
-      </c>
-      <c r="D8" s="2" t="str">
+      <c r="G9" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="J9" s="28" t="s">
+        <v>98</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="2">
+        <v>26</v>
+      </c>
+      <c r="C10" s="2" t="str">
         <f t="shared" si="0"/>
         <v>kbir</v>
       </c>
-      <c r="E8" t="str">
+      <c r="G10" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="K10" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="2">
+        <v>44</v>
+      </c>
+      <c r="C11" s="2" t="str">
         <f t="shared" si="0"/>
         <v>kbir</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="2">
-        <v>5000</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C9" s="2">
-        <v>39</v>
-      </c>
-      <c r="D9" s="2" t="str">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B12" s="2">
+        <v>87</v>
+      </c>
+      <c r="C12" s="2" t="str">
         <f t="shared" si="0"/>
         <v>kbir</v>
       </c>
-      <c r="E9" t="str">
+      <c r="G12" s="27" t="str">
+        <f>HLOOKUP(H9,A4:C13,MATCH(H10,A4:A13,0))</f>
+        <v>sghir</v>
+      </c>
+      <c r="H12" s="27"/>
+      <c r="J12" s="27"/>
+      <c r="K12" s="27"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B13" s="2">
+        <v>56</v>
+      </c>
+      <c r="C13" s="2" t="str">
         <f t="shared" si="0"/>
         <v>kbir</v>
       </c>
-      <c r="I9" s="24" t="s">
-        <v>99</v>
-      </c>
-      <c r="J9" s="2" t="s">
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J15" s="28" t="s">
+        <v>85</v>
+      </c>
+      <c r="K15" s="28" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="2">
-        <v>6000</v>
-      </c>
-      <c r="B10" s="2" t="s">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G16" s="25"/>
+      <c r="J16" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="K16" s="2" t="e">
+        <f>VLOOKUP(J16,A5:A13,3,FALSE)</f>
+        <v>#REF!</v>
+      </c>
+    </row>
+    <row r="17" spans="10:11" x14ac:dyDescent="0.3">
+      <c r="J17" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="K17" s="2"/>
+    </row>
+    <row r="18" spans="10:11" x14ac:dyDescent="0.3">
+      <c r="J18" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="K18" s="2"/>
+    </row>
+    <row r="19" spans="10:11" x14ac:dyDescent="0.3">
+      <c r="J19" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="K19" s="2"/>
+    </row>
+    <row r="20" spans="10:11" x14ac:dyDescent="0.3">
+      <c r="J20" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="K20" s="2"/>
+    </row>
+    <row r="21" spans="10:11" x14ac:dyDescent="0.3">
+      <c r="J21" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="K21" s="2"/>
+    </row>
+    <row r="22" spans="10:11" x14ac:dyDescent="0.3">
+      <c r="J22" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="C10" s="2">
-        <v>26</v>
-      </c>
-      <c r="D10" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>kbir</v>
-      </c>
-      <c r="E10" t="str">
-        <f t="shared" si="0"/>
-        <v>kbir</v>
-      </c>
-      <c r="I10" s="24" t="s">
-        <v>100</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="2">
-        <v>7000</v>
-      </c>
-      <c r="B11" s="2" t="s">
+      <c r="K22" s="2"/>
+    </row>
+    <row r="23" spans="10:11" x14ac:dyDescent="0.3">
+      <c r="J23" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C11" s="2">
-        <v>44</v>
-      </c>
-      <c r="D11" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>kbir</v>
-      </c>
-      <c r="E11" t="str">
-        <f t="shared" si="0"/>
-        <v>kbir</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A12" s="2">
-        <v>8000</v>
-      </c>
-      <c r="B12" s="2" t="s">
+      <c r="K23" s="2"/>
+    </row>
+    <row r="24" spans="10:11" x14ac:dyDescent="0.3">
+      <c r="J24" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C12" s="2">
-        <v>87</v>
-      </c>
-      <c r="D12" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>kbir</v>
-      </c>
-      <c r="E12" t="str">
-        <f t="shared" si="0"/>
-        <v>kbir</v>
-      </c>
-      <c r="I12" s="28" t="str">
-        <f>HLOOKUP(J9,B4:D13,MATCH(J10,B4:B13,0))</f>
-        <v>sghir</v>
-      </c>
-      <c r="J12" s="28"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="2">
-        <v>9000</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="C13" s="2">
-        <v>56</v>
-      </c>
-      <c r="D13" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>kbir</v>
-      </c>
-      <c r="E13" t="str">
-        <f t="shared" si="0"/>
-        <v>kbir</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="I16" s="25"/>
+      <c r="K24" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="I12:J12"/>
-    <mergeCell ref="I7:J7"/>
+  <mergeCells count="4">
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="J12:K12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>